<commit_message>
Update WAR data - 2026-03-02
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12456,7 +12456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI48"/>
+  <dimension ref="A1:CI50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -12777,12 +12777,12 @@
       </c>
       <c r="BA1" s="109" t="inlineStr">
         <is>
-          <t>Colonna53</t>
+          <t>WAR-24 (1)</t>
         </is>
       </c>
       <c r="BB1" s="109" t="inlineStr">
         <is>
-          <t>Colonna54</t>
+          <t>WAR-24 (2)</t>
         </is>
       </c>
       <c r="BC1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>3</v>
       </c>
       <c r="E2" s="111">
-        <f>SUM(G2:AZ2)</f>
+        <f>SUM(G2:BB2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:AZ2),1)</f>
+        <f>ROUND(AVERAGE(G2:BB2),1)</f>
         <v/>
       </c>
       <c r="G2" s="110" t="n"/>
@@ -13086,11 +13086,11 @@
         <v>0</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:AZ3)</f>
+        <f>SUM(G3:BB3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:AZ3),1)</f>
+        <f>ROUND(AVERAGE(G3:BB3),1)</f>
         <v/>
       </c>
     </row>
@@ -13110,11 +13110,11 @@
         <v>4</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:AZ4)</f>
+        <f>SUM(G4:BB4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:AZ4),1)</f>
+        <f>ROUND(AVERAGE(G4:BB4),1)</f>
         <v/>
       </c>
       <c r="I4" s="79" t="n">
@@ -13162,11 +13162,11 @@
         <v>1</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:AZ5)</f>
+        <f>SUM(G5:BB5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:AZ5),1)</f>
+        <f>ROUND(AVERAGE(G5:BB5),1)</f>
         <v/>
       </c>
       <c r="AO5" t="n">
@@ -13185,20 +13185,20 @@
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="68" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:AZ6)</f>
+        <f>SUM(G6:BB6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:AZ6),1)</f>
+        <f>ROUND(AVERAGE(G6:BB6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13319,6 +13319,14 @@
         <v>2</v>
       </c>
       <c r="AZ6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BA6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13340,11 +13348,11 @@
         <v>6</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:AZ7)</f>
+        <f>SUM(G7:BB7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:AZ7),1)</f>
+        <f>ROUND(AVERAGE(G7:BB7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13391,21 +13399,29 @@
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:AZ8)</f>
+        <f>SUM(G8:BB8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:AZ8),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G8:BB8),1)</f>
+        <v/>
+      </c>
+      <c r="BA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -13415,20 +13431,20 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:AZ9)</f>
+        <f>SUM(G9:BB9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:AZ9),1)</f>
+        <f>ROUND(AVERAGE(G9:BB9),1)</f>
         <v/>
       </c>
       <c r="G9" s="79" t="n">
@@ -13508,6 +13524,16 @@
       </c>
       <c r="AV9" t="n">
         <v>3</v>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -13526,11 +13552,11 @@
         <v>0</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:AZ10)</f>
+        <f>SUM(G10:BB10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:AZ10),1)</f>
+        <f>ROUND(AVERAGE(G10:BB10),1)</f>
         <v/>
       </c>
     </row>
@@ -13550,11 +13576,11 @@
         <v>6</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:AZ11)</f>
+        <f>SUM(G11:BB11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:AZ11),1)</f>
+        <f>ROUND(AVERAGE(G11:BB11),1)</f>
         <v/>
       </c>
       <c r="I11" s="79" t="n">
@@ -13624,11 +13650,11 @@
         <v>7</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:AZ12)</f>
+        <f>SUM(G12:BB12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:AZ12),1)</f>
+        <f>ROUND(AVERAGE(G12:BB12),1)</f>
         <v/>
       </c>
       <c r="Q12" s="79" t="n">
@@ -13696,11 +13722,11 @@
         <v>12</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:AZ13)</f>
+        <f>SUM(G13:BB13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:AZ13),1)</f>
+        <f>ROUND(AVERAGE(G13:BB13),1)</f>
         <v/>
       </c>
       <c r="G13" s="79" t="n">
@@ -13792,11 +13818,11 @@
         <v>0</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:AZ14)</f>
+        <f>SUM(G14:BB14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:AZ14),1)</f>
+        <f>ROUND(AVERAGE(G14:BB14),1)</f>
         <v/>
       </c>
     </row>
@@ -13807,20 +13833,20 @@
         </is>
       </c>
       <c r="B15" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:AZ15)</f>
+        <f>SUM(G15:BB15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:AZ15),1)</f>
+        <f>ROUND(AVERAGE(G15:BB15),1)</f>
         <v/>
       </c>
       <c r="I15" s="79" t="n">
@@ -13918,6 +13944,14 @@
       </c>
       <c r="AZ15" t="n">
         <v>3</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -13936,11 +13970,11 @@
         <v>1</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:AZ16)</f>
+        <f>SUM(G16:BB16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:AZ16),1)</f>
+        <f>ROUND(AVERAGE(G16:BB16),1)</f>
         <v/>
       </c>
       <c r="AE16" s="79" t="n">
@@ -13963,14 +13997,14 @@
         <v>1</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:AZ17)</f>
+        <f>SUM(G17:BB17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:AZ17),1)</f>
+        <f>ROUND(AVERAGE(G17:BB17),1)</f>
         <v/>
       </c>
       <c r="S17" s="79" t="n">
@@ -14030,6 +14064,12 @@
       </c>
       <c r="AV17" t="n">
         <v>3</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -14045,14 +14085,14 @@
         <v>0</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:AZ18)</f>
+        <f>SUM(G18:BB18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:AZ18),1)</f>
+        <f>ROUND(AVERAGE(G18:BB18),1)</f>
         <v/>
       </c>
       <c r="G18" s="79" t="n">
@@ -14077,6 +14117,12 @@
         <v>3</v>
       </c>
       <c r="AZ18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14093,14 +14139,14 @@
         <v>0</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:AZ19)</f>
+        <f>SUM(G19:BB19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:AZ19),1)</f>
+        <f>ROUND(AVERAGE(G19:BB19),1)</f>
         <v/>
       </c>
       <c r="AE19" s="79" t="n">
@@ -14108,6 +14154,12 @@
       </c>
       <c r="AF19" s="80" t="n">
         <v>1</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -14123,14 +14175,14 @@
         <v>0</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:AZ20)</f>
+        <f>SUM(G20:BB20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:AZ20),1)</f>
+        <f>ROUND(AVERAGE(G20:BB20),1)</f>
         <v/>
       </c>
       <c r="I20" s="79" t="n">
@@ -14196,6 +14248,12 @@
       </c>
       <c r="AZ20" t="n">
         <v>3</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -14214,11 +14272,11 @@
         <v>10</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:AZ21)</f>
+        <f>SUM(G21:BB21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:AZ21),1)</f>
+        <f>ROUND(AVERAGE(G21:BB21),1)</f>
         <v/>
       </c>
       <c r="G21" s="79" t="inlineStr">
@@ -14295,20 +14353,20 @@
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:AZ22)</f>
+        <f>SUM(G22:BB22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:AZ22),1)</f>
+        <f>ROUND(AVERAGE(G22:BB22),1)</f>
         <v/>
       </c>
       <c r="G22" s="79" t="n">
@@ -14390,6 +14448,14 @@
       </c>
       <c r="AT22" t="n">
         <v>2</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -14405,14 +14471,14 @@
         <v>1</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:AZ23)</f>
+        <f>SUM(G23:BB23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:AZ23),1)</f>
+        <f>ROUND(AVERAGE(G23:BB23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
@@ -14483,6 +14549,12 @@
         <v>3</v>
       </c>
       <c r="AL23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB23" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14499,14 +14571,14 @@
         <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:AZ24)</f>
+        <f>SUM(G24:BB24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:AZ24),1)</f>
+        <f>ROUND(AVERAGE(G24:BB24),1)</f>
         <v/>
       </c>
       <c r="I24" s="79" t="n">
@@ -14565,6 +14637,12 @@
         <v>3</v>
       </c>
       <c r="AL24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14584,11 +14662,11 @@
         <v>3</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:AZ25)</f>
+        <f>SUM(G25:BB25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:AZ25),1)</f>
+        <f>ROUND(AVERAGE(G25:BB25),1)</f>
         <v/>
       </c>
       <c r="Y25" s="79" t="n">
@@ -14628,11 +14706,11 @@
         <v>8</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:AZ26)</f>
+        <f>SUM(G26:BB26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:AZ26),1)</f>
+        <f>ROUND(AVERAGE(G26:BB26),1)</f>
         <v/>
       </c>
       <c r="S26" s="79" t="n">
@@ -14710,11 +14788,11 @@
         <v>10</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:AZ27)</f>
+        <f>SUM(G27:BB27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:AZ27),1)</f>
+        <f>ROUND(AVERAGE(G27:BB27),1)</f>
         <v/>
       </c>
       <c r="I27" s="79" t="inlineStr">
@@ -14795,7 +14873,7 @@
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>Roberta</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
@@ -14805,235 +14883,315 @@
         <v>0</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:AZ28)</f>
+        <f>SUM(G28:BB28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:AZ28),1)</f>
-        <v/>
-      </c>
-      <c r="AO28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP28" t="n">
-        <v>1</v>
+        <f>ROUND(AVERAGE(G28:BB28),1)</f>
+        <v/>
+      </c>
+      <c r="G28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C29" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:AZ29)</f>
+        <f>SUM(G29:BB29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:AZ29),1)</f>
+        <f>ROUND(AVERAGE(G29:BB29),1)</f>
         <v/>
       </c>
       <c r="G29" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H29" s="80" t="n">
         <v>3</v>
       </c>
       <c r="I29" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J29" s="80" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="K29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="O29" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P29" s="80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q29" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R29" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="AU29" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV29" t="n">
+      <c r="U29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y29" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB29" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT29" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:AZ30)</f>
+        <f>SUM(G30:BB30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:AZ30),1)</f>
-        <v/>
-      </c>
-      <c r="G30" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I30" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L30" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="M30" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P30" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="R30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V30" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y30" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z30" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK30" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL30" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM30" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN30" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G30:BB30),1)</f>
+        <v/>
       </c>
       <c r="AS30" t="n">
         <v>3</v>
       </c>
       <c r="AT30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>th4nos</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C31" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:AZ31)</f>
+        <f>SUM(G31:BB31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:AZ31),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G31:BB31),1)</f>
+        <v/>
+      </c>
+      <c r="O31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W31" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X31" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF31" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>1</v>
       </c>
       <c r="AS31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:AZ32)</f>
+        <f>SUM(G32:BB32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:AZ32),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G32:BB32),1)</f>
+        <v/>
+      </c>
+      <c r="G32" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L32" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="O32" s="79" t="n">
         <v>3</v>
@@ -15045,24 +15203,36 @@
         <v>3</v>
       </c>
       <c r="R32" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S32" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T32" s="80" t="n">
         <v>2</v>
       </c>
       <c r="W32" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X32" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="Y32" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z32" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA32" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB32" s="80" t="n">
+        <v>2</v>
+      </c>
       <c r="AC32" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD32" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF32" s="80" t="n">
         <v>3</v>
       </c>
       <c r="AI32" t="inlineStr">
@@ -15081,247 +15251,193 @@
       <c r="AL32" t="n">
         <v>3</v>
       </c>
-      <c r="AO32" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP32" t="n">
-        <v>1</v>
+      <c r="AM32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>3</v>
       </c>
       <c r="AS32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB32" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
         <v>4</v>
       </c>
       <c r="C33" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:AZ33)</f>
+        <f>SUM(G33:BB33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:AZ33),1)</f>
-        <v/>
-      </c>
-      <c r="G33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G33:BB33),1)</f>
+        <v/>
+      </c>
+      <c r="U33" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W33" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X33" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="L33" s="80" t="inlineStr">
+      <c r="Y33" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA33" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB33" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC33" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE33" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="O33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI33" t="inlineStr">
+      <c r="AJ33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ33" t="inlineStr">
+      <c r="AK33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL33" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AK33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL33" t="n">
-        <v>3</v>
-      </c>
       <c r="AM33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN33" t="n">
         <v>3</v>
       </c>
-      <c r="AS33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV33" t="n">
+      <c r="AO33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB33" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="79" t="n">
         <v>4</v>
       </c>
-      <c r="C34" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="79" t="n">
-        <v>11</v>
-      </c>
       <c r="E34" s="68">
-        <f>SUM(G34:AZ34)</f>
+        <f>SUM(G34:BB34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:AZ34),1)</f>
-        <v/>
-      </c>
-      <c r="U34" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V34" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W34" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X34" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G34:BB34),1)</f>
+        <v/>
+      </c>
+      <c r="AM34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP34" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="Y34" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z34" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA34" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB34" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC34" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD34" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE34" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF34" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AM34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ34" t="n">
-        <v>2</v>
+      <c r="AS34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="68" t="n">
         <v>0</v>
@@ -15330,44 +15446,42 @@
         <v>4</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:AZ35)</f>
+        <f>SUM(G35:BB35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:AZ35),1)</f>
+        <f>ROUND(AVERAGE(G35:BB35),1)</f>
         <v/>
       </c>
       <c r="AM35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>3</v>
       </c>
       <c r="AS35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV35" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="AY35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ35" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
@@ -15377,45 +15491,57 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:AZ36)</f>
+        <f>SUM(G36:BB36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:AZ36),1)</f>
+        <f>ROUND(AVERAGE(G36:BB36),1)</f>
         <v/>
       </c>
       <c r="AM36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO36" t="n">
         <v>3</v>
       </c>
       <c r="AP36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT36" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV36" t="n">
+        <v>3</v>
       </c>
       <c r="AY36" t="n">
         <v>3</v>
       </c>
       <c r="AZ36" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BA36" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB36" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
@@ -15425,75 +15551,73 @@
         <v>0</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:AZ37)</f>
+        <f>SUM(G37:BB37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:AZ37),1)</f>
-        <v/>
-      </c>
-      <c r="AM37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP37" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY37" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ37" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G37:BB37),1)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:AZ38)</f>
+        <f>SUM(G38:BB38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:AZ38),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G38:BB38),1)</f>
+        <v/>
+      </c>
+      <c r="AM38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP38" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BB38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
@@ -15503,18 +15627,18 @@
         <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:AZ39)</f>
+        <f>SUM(G39:BB39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:AZ39),1)</f>
+        <f>ROUND(AVERAGE(G39:BB39),1)</f>
         <v/>
       </c>
       <c r="AM39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN39" t="n">
         <v>3</v>
@@ -15523,19 +15647,37 @@
         <v>3</v>
       </c>
       <c r="AP39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT39" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY39" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ39" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB39" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>fede61mito</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
@@ -15545,51 +15687,21 @@
         <v>0</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:AZ40)</f>
+        <f>SUM(G40:BB40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:AZ40),1)</f>
-        <v/>
-      </c>
-      <c r="AM40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS40" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT40" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU40" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY40" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ40" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G40:BB40),1)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
@@ -15602,42 +15714,52 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:AZ41)</f>
+        <f>SUM(G41:BB41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:AZ41),1)</f>
+        <f>ROUND(AVERAGE(G41:BB41),1)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>Xx_Herman_xX</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:AZ42)</f>
+        <f>SUM(G42:BB42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:AZ42),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G42:BB42),1)</f>
+        <v/>
+      </c>
+      <c r="BA42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>Xx_Herman_xX</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -15650,18 +15772,18 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:AZ43)</f>
+        <f>SUM(G43:BB43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:AZ43),1)</f>
+        <f>ROUND(AVERAGE(G43:BB43),1)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>dibba10</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -15671,21 +15793,27 @@
         <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:AZ44)</f>
+        <f>SUM(G44:BB44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:AZ44),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G44:BB44),1)</f>
+        <v/>
+      </c>
+      <c r="BA44" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB44" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -15695,21 +15823,27 @@
         <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:AZ45)</f>
+        <f>SUM(G45:BB45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:AZ45),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G45:BB45),1)</f>
+        <v/>
+      </c>
+      <c r="BA45" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB45" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>thommyspine</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -15722,18 +15856,18 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:AZ46)</f>
+        <f>SUM(G46:BB46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:AZ46),1)</f>
+        <f>ROUND(AVERAGE(G46:BB46),1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -15746,18 +15880,18 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:AZ47)</f>
+        <f>SUM(G47:BB47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:AZ47),1)</f>
+        <f>ROUND(AVERAGE(G47:BB47),1)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>eltishqipe</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -15770,11 +15904,59 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:AZ48)</f>
+        <f>SUM(G48:BB48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:AZ48),1)</f>
+        <f>ROUND(AVERAGE(G48:BB48),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="79" t="inlineStr">
+        <is>
+          <t>StepanYT Ita Uk</t>
+        </is>
+      </c>
+      <c r="B49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="68">
+        <f>SUM(G49:BB49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="68">
+        <f>ROUND(AVERAGE(G49:BB49),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>I puma</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:BB50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:BB50),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-12
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12456,7 +12456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI50"/>
+  <dimension ref="A1:CI49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -12787,12 +12787,12 @@
       </c>
       <c r="BC1" s="109" t="inlineStr">
         <is>
-          <t>Colonna55</t>
+          <t>WAR-25 (1)</t>
         </is>
       </c>
       <c r="BD1" s="109" t="inlineStr">
         <is>
-          <t>Colonna56</t>
+          <t>WAR-25 (2)</t>
         </is>
       </c>
       <c r="BE1" s="109" t="inlineStr">
@@ -12958,20 +12958,20 @@
         </is>
       </c>
       <c r="B2" s="110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" s="111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="110" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="111">
-        <f>SUM(G2:BB2)</f>
+        <f>SUM(G2:BD2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BB2),1)</f>
+        <f>ROUND(AVERAGE(G2:BD2),1)</f>
         <v/>
       </c>
       <c r="G2" s="110" t="n"/>
@@ -13036,8 +13036,16 @@
       <c r="AZ2" s="111" t="n"/>
       <c r="BA2" s="111" t="n"/>
       <c r="BB2" s="111" t="n"/>
-      <c r="BC2" s="111" t="n"/>
-      <c r="BD2" s="111" t="n"/>
+      <c r="BC2" s="111" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD2" s="111" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="BE2" s="111" t="n"/>
       <c r="BF2" s="111" t="n"/>
       <c r="BG2" s="111" t="n"/>
@@ -13086,93 +13094,195 @@
         <v>0</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BB3)</f>
+        <f>SUM(G3:BD3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BB3),1)</f>
+        <f>ROUND(AVERAGE(G3:BD3),1)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="79" t="inlineStr">
         <is>
-          <t>ajejebrazorf</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BB4)</f>
+        <f>SUM(G4:BD4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BB4),1)</f>
-        <v/>
-      </c>
-      <c r="I4" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J4" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="W4" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="X4" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI4" t="inlineStr">
+        <f>ROUND(AVERAGE(G4:BD4),1)</f>
+        <v/>
+      </c>
+      <c r="AO4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP4" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="79" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C5" s="68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BB5)</f>
+        <f>SUM(G5:BD5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BB5),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G5:BD5),1)</f>
+        <v/>
+      </c>
+      <c r="G5" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="R5" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W5" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="X5" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Y5" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z5" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA5" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB5" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC5" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AD5" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>1</v>
       </c>
       <c r="AO5" t="n">
         <v>2</v>
       </c>
       <c r="AP5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AY5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BA5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB5" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13181,454 +13291,384 @@
     <row r="6">
       <c r="A6" s="79" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C6" s="68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BB6)</f>
+        <f>SUM(G6:BD6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BB6),1)</f>
-        <v/>
-      </c>
-      <c r="G6" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="80" t="n">
-        <v>0</v>
+        <f>ROUND(AVERAGE(G6:BD6),1)</f>
+        <v/>
       </c>
       <c r="K6" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M6" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N6" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P6" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="R6" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W6" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="X6" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y6" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z6" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA6" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB6" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC6" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AD6" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="Q6" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R6" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC6" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD6" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="AM6" t="n">
         <v>3</v>
       </c>
       <c r="AN6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AU6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AV6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AY6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BA6" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB6" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="79" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B7" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BB7)</f>
+        <f>SUM(G7:BD7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BB7),1)</f>
-        <v/>
-      </c>
-      <c r="K7" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M7" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q7" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R7" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC7" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD7" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G7:BD7),1)</f>
+        <v/>
+      </c>
+      <c r="BA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BB8)</f>
+        <f>SUM(G8:BD8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BB8),1)</f>
-        <v/>
-      </c>
-      <c r="BA8" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G8:BD8),1)</f>
+        <v/>
+      </c>
+      <c r="G8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T8" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V8" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X8" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y8" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB8" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC8" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD8" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BB8" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BC8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="79" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BB9)</f>
+        <f>SUM(G9:BD9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BB9),1)</f>
-        <v/>
-      </c>
-      <c r="G9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P9" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R9" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="S9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="U9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V9" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X9" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y9" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z9" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB9" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD9" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV9" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G9:BD9),1)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="79" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BB10)</f>
+        <f>SUM(G10:BD10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BB10),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G10:BD10),1)</f>
+        <v/>
+      </c>
+      <c r="I10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="O10" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="P10" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S10" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="79" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="68" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="79" t="n">
-        <v>6</v>
-      </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BB11)</f>
+        <f>SUM(G11:BD11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BB11),1)</f>
-        <v/>
-      </c>
-      <c r="I11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G11:BD11),1)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="U11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V11" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z11" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB11" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="O11" s="79" t="inlineStr">
+      <c r="AE11" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF11" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="P11" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="S11" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="T11" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK11" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AN11" t="inlineStr">
+      <c r="AZ11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13637,57 +13677,85 @@
     <row r="12">
       <c r="A12" s="79" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BB12)</f>
+        <f>SUM(G12:BD12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BB12),1)</f>
-        <v/>
-      </c>
-      <c r="Q12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R12" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G12:BD12),1)</f>
+        <v/>
+      </c>
+      <c r="G12" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="U12" s="79" t="n">
         <v>3</v>
       </c>
       <c r="V12" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W12" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="X12" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="Y12" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z12" s="80" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB12" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE12" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF12" s="80" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AB12" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>2</v>
       </c>
       <c r="AS12" t="n">
         <v>1</v>
@@ -13695,21 +13763,17 @@
       <c r="AT12" t="n">
         <v>2</v>
       </c>
-      <c r="AY12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AZ12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="AU12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="79" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>Giorgio</t>
         </is>
       </c>
       <c r="B13" s="79" t="n">
@@ -13719,165 +13783,191 @@
         <v>0</v>
       </c>
       <c r="D13" s="79" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BB13)</f>
+        <f>SUM(G13:BD13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BB13),1)</f>
-        <v/>
-      </c>
-      <c r="G13" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M13" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W13" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="X13" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z13" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB13" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>1</v>
+        <f>ROUND(AVERAGE(G13:BD13),1)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="79" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BB14)</f>
+        <f>SUM(G14:BD14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BB14),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G14:BD14),1)</f>
+        <v/>
+      </c>
+      <c r="I14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P14" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V14" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC14" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD14" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF14" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B15" s="79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C15" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BB15)</f>
+        <f>SUM(G15:BD15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BB15),1)</f>
-        <v/>
-      </c>
-      <c r="I15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P15" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V15" s="80" t="n">
-        <v>1</v>
+        <f>ROUND(AVERAGE(G15:BD15),1)</f>
+        <v/>
+      </c>
+      <c r="S15" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T15" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W15" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X15" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z15" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="AA15" s="79" t="n">
         <v>3</v>
@@ -13886,52 +13976,32 @@
         <v>3</v>
       </c>
       <c r="AC15" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD15" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF15" s="80" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AI15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AI15" t="inlineStr">
+      <c r="AJ15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="AK15" t="n">
         <v>3</v>
       </c>
       <c r="AL15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AU15" t="n">
         <v>3</v>
@@ -13939,25 +14009,17 @@
       <c r="AV15" t="n">
         <v>3</v>
       </c>
-      <c r="AY15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ15" t="n">
-        <v>3</v>
-      </c>
       <c r="BA15" t="n">
         <v>1</v>
       </c>
-      <c r="BB15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="BB15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="79" t="inlineStr">
         <is>
-          <t>GioStyle</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B16" s="79" t="n">
@@ -13967,151 +14029,169 @@
         <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BB16)</f>
+        <f>SUM(G16:BD16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BB16),1)</f>
-        <v/>
-      </c>
-      <c r="AE16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF16" s="80" t="n">
+        <f>ROUND(AVERAGE(G16:BD16),1)</f>
+        <v/>
+      </c>
+      <c r="G16" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD16" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BB17)</f>
+        <f>SUM(G17:BD17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BB17),1)</f>
-        <v/>
-      </c>
-      <c r="S17" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T17" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W17" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X17" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z17" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB17" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD17" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV17" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G17:BD17),1)</f>
+        <v/>
+      </c>
+      <c r="AE17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF17" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="BA17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="79" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C18" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BB18)</f>
+        <f>SUM(G18:BD18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BB18),1)</f>
-        <v/>
-      </c>
-      <c r="G18" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G18:BD18),1)</f>
+        <v/>
       </c>
       <c r="I18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z18" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="J18" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="M18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R18" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W18" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X18" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB18" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC18" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>1</v>
       </c>
       <c r="AY18" t="n">
         <v>3</v>
@@ -14120,402 +14200,378 @@
         <v>3</v>
       </c>
       <c r="BA18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BB18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C19" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BB19)</f>
+        <f>SUM(G19:BD19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BB19),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G19:BD19),1)</f>
+        <v/>
+      </c>
+      <c r="G19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S19" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X19" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AE19" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="AF19" s="80" t="n">
-        <v>1</v>
+      <c r="AF19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AS19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>2</v>
       </c>
       <c r="BA19" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB19" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B20" s="79" t="n">
         <v>2</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BB20)</f>
+        <f>SUM(G20:BD20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BB20),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G20:BD20),1)</f>
+        <v/>
+      </c>
+      <c r="G20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I20" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="J20" s="80" t="inlineStr">
+      <c r="J20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="T20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V20" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF20" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="M20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N20" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="80" t="inlineStr">
+      <c r="AJ20" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="W20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X20" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB20" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ20" t="n">
+      <c r="AK20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL20" t="n">
         <v>3</v>
       </c>
       <c r="BA20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>Luxor</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BB21)</f>
+        <f>SUM(G21:BD21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BB21),1)</f>
-        <v/>
-      </c>
-      <c r="G21" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G21:BD21),1)</f>
+        <v/>
+      </c>
+      <c r="I21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI21" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="H21" s="80" t="inlineStr">
+      <c r="AJ21" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="I21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W21" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X21" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV21" t="n">
-        <v>2</v>
+      <c r="AK21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="79" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C22" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BB22)</f>
+        <f>SUM(G22:BD22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BB22),1)</f>
-        <v/>
-      </c>
-      <c r="G22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J22" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P22" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G22:BD22),1)</f>
+        <v/>
+      </c>
+      <c r="Y22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z22" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="S22" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T22" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X22" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB22" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="AC22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD22" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="AE22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF22" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AS22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AF22" s="80" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BB23)</f>
+        <f>SUM(G23:BD23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BB23),1)</f>
-        <v/>
-      </c>
-      <c r="G23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="N23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R23" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G23:BD23),1)</f>
+        <v/>
       </c>
       <c r="S23" s="79" t="n">
         <v>3</v>
@@ -14523,17 +14579,39 @@
       <c r="T23" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="U23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V23" s="80" t="n">
+      <c r="U23" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="V23" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD23" s="80" t="n">
         <v>3</v>
       </c>
       <c r="AE23" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF23" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AI23" t="inlineStr">
         <is>
@@ -14546,22 +14624,24 @@
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL23" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA23" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB23" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
@@ -14571,39 +14651,53 @@
         <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BB24)</f>
+        <f>SUM(G24:BD24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BB24),1)</f>
-        <v/>
-      </c>
-      <c r="I24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J24" s="80" t="n">
+        <f>ROUND(AVERAGE(G24:BD24),1)</f>
+        <v/>
+      </c>
+      <c r="I24" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J24" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="K24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" s="80" t="n">
         <v>3</v>
       </c>
       <c r="M24" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N24" s="80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P24" s="80" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="P24" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="Q24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R24" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="R24" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="W24" s="79" t="n">
         <v>3</v>
@@ -14615,286 +14709,254 @@
         <v>3</v>
       </c>
       <c r="Z24" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="AA24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB24" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC24" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD24" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="AE24" s="79" t="n">
         <v>3</v>
       </c>
       <c r="AF24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK24" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB24" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BB25)</f>
+        <f>SUM(G25:BD25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BB25),1)</f>
-        <v/>
-      </c>
-      <c r="Y25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z25" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AC25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD25" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE25" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF25" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G25:BD25),1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B26" s="79" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C26" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BB26)</f>
+        <f>SUM(G26:BD26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BB26),1)</f>
-        <v/>
-      </c>
-      <c r="S26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T26" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U26" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G26:BD26),1)</f>
+        <v/>
+      </c>
+      <c r="G26" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y26" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI26" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="V26" s="80" t="inlineStr">
+      <c r="AJ26" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="W26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X26" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z26" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD26" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE26" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF26" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="AK26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BB27)</f>
+        <f>SUM(G27:BD27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BB27),1)</f>
-        <v/>
-      </c>
-      <c r="I27" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J27" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="K27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M27" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O27" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Q27" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R27" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z27" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB27" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC27" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD27" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF27" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN27" t="n">
+        <f>ROUND(AVERAGE(G27:BD27),1)</f>
+        <v/>
+      </c>
+      <c r="AS27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT27" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BB28)</f>
+        <f>SUM(G28:BD28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BB28),1)</f>
+        <f>ROUND(AVERAGE(G28:BD28),1)</f>
         <v/>
       </c>
       <c r="G28" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" s="80" t="n">
         <v>3</v>
@@ -14905,11 +14967,21 @@
       <c r="J28" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="K28" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L28" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="O28" s="79" t="n">
         <v>3</v>
       </c>
       <c r="P28" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q28" s="79" t="n">
         <v>3</v>
@@ -14917,6 +14989,64 @@
       <c r="R28" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="S28" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T28" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y28" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB28" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC28" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>3</v>
+      </c>
       <c r="AU28" t="n">
         <v>3</v>
       </c>
@@ -14924,70 +15054,40 @@
         <v>3</v>
       </c>
       <c r="BA28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BB28" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD28" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C29" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BB29)</f>
+        <f>SUM(G29:BD29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BB29),1)</f>
-        <v/>
-      </c>
-      <c r="G29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I29" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="M29" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O29" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P29" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q29" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="R29" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G29:BD29),1)</f>
+        <v/>
       </c>
       <c r="U29" s="79" t="n">
         <v>3</v>
@@ -14995,6 +15095,14 @@
       <c r="V29" s="80" t="n">
         <v>2</v>
       </c>
+      <c r="W29" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X29" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="Y29" s="79" t="n">
         <v>2</v>
       </c>
@@ -15007,6 +15115,18 @@
       <c r="AB29" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="AC29" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF29" s="80" t="n">
+        <v>2</v>
+      </c>
       <c r="AI29" t="inlineStr">
         <is>
           <t>SKIP</t>
@@ -15020,243 +15140,181 @@
       <c r="AK29" t="n">
         <v>2</v>
       </c>
-      <c r="AL29" t="n">
-        <v>3</v>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AM29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN29" t="n">
         <v>3</v>
       </c>
-      <c r="AS29" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT29" t="n">
+      <c r="AO29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD29" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BB30)</f>
+        <f>SUM(G30:BD30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BB30),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G30:BD30),1)</f>
+        <v/>
+      </c>
+      <c r="AM30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP30" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AS30" t="n">
         <v>3</v>
       </c>
       <c r="AT30" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>th4nos</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C31" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BB31)</f>
+        <f>SUM(G31:BD31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BB31),1)</f>
-        <v/>
-      </c>
-      <c r="O31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P31" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R31" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W31" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X31" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD31" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF31" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK31" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL31" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G31:BD31),1)</f>
+        <v/>
+      </c>
+      <c r="AM31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>2</v>
       </c>
       <c r="AO31" t="n">
         <v>3</v>
       </c>
       <c r="AP31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS31" t="n">
         <v>2</v>
       </c>
       <c r="AT31" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BB32)</f>
+        <f>SUM(G32:BD32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BB32),1)</f>
-        <v/>
-      </c>
-      <c r="G32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L32" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P32" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T32" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB32" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK32" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL32" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G32:BD32),1)</f>
+        <v/>
       </c>
       <c r="AM32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN32" t="n">
         <v>3</v>
       </c>
+      <c r="AO32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>2</v>
+      </c>
       <c r="AS32" t="n">
         <v>3</v>
       </c>
@@ -15269,138 +15327,70 @@
       <c r="AV32" t="n">
         <v>3</v>
       </c>
+      <c r="AY32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>3</v>
+      </c>
       <c r="BA32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB32" t="n">
         <v>3</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD32" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>terracrom</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C33" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BB33)</f>
+        <f>SUM(G33:BD33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BB33),1)</f>
-        <v/>
-      </c>
-      <c r="U33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X33" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC33" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AM33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP33" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY33" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ33" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA33" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB33" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G33:BD33),1)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="79" t="n">
         <v>4</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BB34)</f>
+        <f>SUM(G34:BD34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BB34),1)</f>
+        <f>ROUND(AVERAGE(G34:BD34),1)</f>
         <v/>
       </c>
       <c r="AM34" t="n">
@@ -15410,30 +15400,32 @@
         <v>3</v>
       </c>
       <c r="AO34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP34" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA34" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AS34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV34" t="n">
-        <v>0</v>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
@@ -15443,21 +15435,21 @@
         <v>0</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BB35)</f>
+        <f>SUM(G35:BD35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BB35),1)</f>
+        <f>ROUND(AVERAGE(G35:BD35),1)</f>
         <v/>
       </c>
       <c r="AM35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO35" t="n">
         <v>3</v>
@@ -15466,22 +15458,40 @@
         <v>3</v>
       </c>
       <c r="AS35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT35" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>3</v>
       </c>
       <c r="AY35" t="n">
         <v>3</v>
       </c>
       <c r="AZ35" t="n">
         <v>2</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB35" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD35" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>fede61mito</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
@@ -15491,57 +15501,21 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BB36)</f>
+        <f>SUM(G36:BD36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BB36),1)</f>
-        <v/>
-      </c>
-      <c r="AM36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP36" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY36" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ36" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA36" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB36" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G36:BD36),1)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
@@ -15554,70 +15528,42 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BB37)</f>
+        <f>SUM(G37:BD37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BB37),1)</f>
+        <f>ROUND(AVERAGE(G37:BD37),1)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BB38)</f>
+        <f>SUM(G38:BD38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BB38),1)</f>
-        <v/>
-      </c>
-      <c r="AM38" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN38" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO38" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP38" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS38" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT38" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G38:BD38),1)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
@@ -15627,57 +15573,27 @@
         <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BB39)</f>
+        <f>SUM(G39:BD39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BB39),1)</f>
-        <v/>
-      </c>
-      <c r="AM39" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU39" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY39" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ39" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G39:BD39),1)</f>
+        <v/>
       </c>
       <c r="BA39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
@@ -15687,79 +15603,85 @@
         <v>0</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BB40)</f>
+        <f>SUM(G40:BD40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BB40),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G40:BD40),1)</f>
+        <v/>
+      </c>
+      <c r="BA40" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB40" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>thommyspine</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BB41)</f>
+        <f>SUM(G41:BD41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BB41),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G41:BD41),1)</f>
+        <v/>
+      </c>
+      <c r="BC41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>Xx_Herman_xX</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BB42)</f>
+        <f>SUM(G42:BD42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BB42),1)</f>
-        <v/>
-      </c>
-      <c r="BA42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G42:BD42),1)</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -15769,51 +15691,61 @@
         <v>0</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BB43)</f>
+        <f>SUM(G43:BD43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BB43),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G43:BD43),1)</f>
+        <v/>
+      </c>
+      <c r="BC43" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD43" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="79" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BB44)</f>
+        <f>SUM(G44:BD44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BB44),1)</f>
-        <v/>
-      </c>
-      <c r="BA44" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB44" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G44:BD44),1)</f>
+        <v/>
+      </c>
+      <c r="BC44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -15823,27 +15755,21 @@
         <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BB45)</f>
+        <f>SUM(G45:BD45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BB45),1)</f>
-        <v/>
-      </c>
-      <c r="BA45" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB45" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G45:BD45),1)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>thommyspine</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -15856,42 +15782,52 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BB46)</f>
+        <f>SUM(G46:BD46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BB46),1)</f>
+        <f>ROUND(AVERAGE(G46:BD46),1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BB47)</f>
+        <f>SUM(G47:BD47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BB47),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G47:BD47),1)</f>
+        <v/>
+      </c>
+      <c r="BC47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -15904,18 +15840,18 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BB48)</f>
+        <f>SUM(G48:BD48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BB48),1)</f>
+        <f>ROUND(AVERAGE(G48:BD48),1)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Samu-Nighix</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -15928,35 +15864,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BB49)</f>
+        <f>SUM(G49:BD49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BB49),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>I puma</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:BB50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BB50),1)</f>
+        <f>ROUND(AVERAGE(G49:BD49),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-15
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12456,7 +12456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI49"/>
+  <dimension ref="A1:CI50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -12797,12 +12797,12 @@
       </c>
       <c r="BE1" s="109" t="inlineStr">
         <is>
-          <t>Colonna57</t>
+          <t>WAR-26 (1)</t>
         </is>
       </c>
       <c r="BF1" s="109" t="inlineStr">
         <is>
-          <t>Colonna58</t>
+          <t>WAR-26 (2)</t>
         </is>
       </c>
       <c r="BG1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>4</v>
       </c>
       <c r="E2" s="111">
-        <f>SUM(G2:BD2)</f>
+        <f>SUM(G2:BF2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BD2),1)</f>
+        <f>ROUND(AVERAGE(G2:BF2),1)</f>
         <v/>
       </c>
       <c r="G2" s="110" t="n"/>
@@ -13094,11 +13094,11 @@
         <v>0</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BD3)</f>
+        <f>SUM(G3:BF3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BD3),1)</f>
+        <f>ROUND(AVERAGE(G3:BF3),1)</f>
         <v/>
       </c>
     </row>
@@ -13115,14 +13115,14 @@
         <v>0</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BD4)</f>
+        <f>SUM(G4:BF4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BD4),1)</f>
+        <f>ROUND(AVERAGE(G4:BF4),1)</f>
         <v/>
       </c>
       <c r="AO4" t="n">
@@ -13132,6 +13132,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BE4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -13147,14 +13153,14 @@
         <v>5</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BD5)</f>
+        <f>SUM(G5:BF5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BD5),1)</f>
+        <f>ROUND(AVERAGE(G5:BF5),1)</f>
         <v/>
       </c>
       <c r="G5" s="79" t="n">
@@ -13286,6 +13292,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BE5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -13301,14 +13313,14 @@
         <v>0</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BD6)</f>
+        <f>SUM(G6:BF6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BD6),1)</f>
+        <f>ROUND(AVERAGE(G6:BF6),1)</f>
         <v/>
       </c>
       <c r="K6" s="79" t="n">
@@ -13351,6 +13363,12 @@
         <v>3</v>
       </c>
       <c r="BD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13370,11 +13388,11 @@
         <v>1</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BD7)</f>
+        <f>SUM(G7:BF7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BD7),1)</f>
+        <f>ROUND(AVERAGE(G7:BF7),1)</f>
         <v/>
       </c>
       <c r="BA7" t="n">
@@ -13402,11 +13420,11 @@
         <v>15</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BD8)</f>
+        <f>SUM(G8:BF8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BD8),1)</f>
+        <f>ROUND(AVERAGE(G8:BF8),1)</f>
         <v/>
       </c>
       <c r="G8" s="79" t="n">
@@ -13520,11 +13538,11 @@
         <v>0</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BD9)</f>
+        <f>SUM(G9:BF9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BD9),1)</f>
+        <f>ROUND(AVERAGE(G9:BF9),1)</f>
         <v/>
       </c>
     </row>
@@ -13544,11 +13562,11 @@
         <v>6</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BD10)</f>
+        <f>SUM(G10:BF10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BD10),1)</f>
+        <f>ROUND(AVERAGE(G10:BF10),1)</f>
         <v/>
       </c>
       <c r="I10" s="79" t="n">
@@ -13618,11 +13636,11 @@
         <v>7</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BD11)</f>
+        <f>SUM(G11:BF11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BD11),1)</f>
+        <f>ROUND(AVERAGE(G11:BF11),1)</f>
         <v/>
       </c>
       <c r="Q11" s="79" t="n">
@@ -13690,11 +13708,11 @@
         <v>12</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BD12)</f>
+        <f>SUM(G12:BF12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BD12),1)</f>
+        <f>ROUND(AVERAGE(G12:BF12),1)</f>
         <v/>
       </c>
       <c r="G12" s="79" t="n">
@@ -13786,11 +13804,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BD13)</f>
+        <f>SUM(G13:BF13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BD13),1)</f>
+        <f>ROUND(AVERAGE(G13:BF13),1)</f>
         <v/>
       </c>
     </row>
@@ -13810,11 +13828,11 @@
         <v>17</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BD14)</f>
+        <f>SUM(G14:BF14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BD14),1)</f>
+        <f>ROUND(AVERAGE(G14:BF14),1)</f>
         <v/>
       </c>
       <c r="I14" s="79" t="n">
@@ -13944,11 +13962,11 @@
         <v>10</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BD15)</f>
+        <f>SUM(G15:BF15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BD15),1)</f>
+        <f>ROUND(AVERAGE(G15:BF15),1)</f>
         <v/>
       </c>
       <c r="S15" s="79" t="n">
@@ -14029,14 +14047,14 @@
         <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BD16)</f>
+        <f>SUM(G16:BF16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BD16),1)</f>
+        <f>ROUND(AVERAGE(G16:BF16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14073,6 +14091,12 @@
         <v>3</v>
       </c>
       <c r="BD16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF16" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14092,11 +14116,11 @@
         <v>2</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BD17)</f>
+        <f>SUM(G17:BF17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BD17),1)</f>
+        <f>ROUND(AVERAGE(G17:BF17),1)</f>
         <v/>
       </c>
       <c r="AE17" s="79" t="n">
@@ -14128,11 +14152,11 @@
         <v>11</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BD18)</f>
+        <f>SUM(G18:BF18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BD18),1)</f>
+        <f>ROUND(AVERAGE(G18:BF18),1)</f>
         <v/>
       </c>
       <c r="I18" s="79" t="n">
@@ -14213,20 +14237,20 @@
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C19" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BD19)</f>
+        <f>SUM(G19:BF19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BD19),1)</f>
+        <f>ROUND(AVERAGE(G19:BF19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14313,6 +14337,14 @@
         <v>3</v>
       </c>
       <c r="BB19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BE19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -14334,11 +14366,11 @@
         <v>12</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BD20)</f>
+        <f>SUM(G20:BF20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BD20),1)</f>
+        <f>ROUND(AVERAGE(G20:BF20),1)</f>
         <v/>
       </c>
       <c r="G20" s="79" t="n">
@@ -14434,11 +14466,11 @@
         <v>9</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BD21)</f>
+        <f>SUM(G21:BF21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BD21),1)</f>
+        <f>ROUND(AVERAGE(G21:BF21),1)</f>
         <v/>
       </c>
       <c r="I21" s="79" t="n">
@@ -14522,11 +14554,11 @@
         <v>3</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BD22)</f>
+        <f>SUM(G22:BF22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BD22),1)</f>
+        <f>ROUND(AVERAGE(G22:BF22),1)</f>
         <v/>
       </c>
       <c r="Y22" s="79" t="n">
@@ -14566,11 +14598,11 @@
         <v>9</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BD23)</f>
+        <f>SUM(G23:BF23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BD23),1)</f>
+        <f>ROUND(AVERAGE(G23:BF23),1)</f>
         <v/>
       </c>
       <c r="S23" s="79" t="n">
@@ -14654,11 +14686,11 @@
         <v>10</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BD24)</f>
+        <f>SUM(G24:BF24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BD24),1)</f>
+        <f>ROUND(AVERAGE(G24:BF24),1)</f>
         <v/>
       </c>
       <c r="I24" s="79" t="inlineStr">
@@ -14749,14 +14781,14 @@
         <v>0</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BD25)</f>
+        <f>SUM(G25:BF25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BD25),1)</f>
+        <f>ROUND(AVERAGE(G25:BF25),1)</f>
         <v/>
       </c>
       <c r="G25" s="79" t="n">
@@ -14793,6 +14825,12 @@
         <v>3</v>
       </c>
       <c r="BB25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14812,11 +14850,11 @@
         <v>12</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BD26)</f>
+        <f>SUM(G26:BF26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BD26),1)</f>
+        <f>ROUND(AVERAGE(G26:BF26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -14918,11 +14956,11 @@
         <v>1</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BD27)</f>
+        <f>SUM(G27:BF27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BD27),1)</f>
+        <f>ROUND(AVERAGE(G27:BF27),1)</f>
         <v/>
       </c>
       <c r="AS27" t="n">
@@ -14945,14 +14983,14 @@
         <v>2</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BD28)</f>
+        <f>SUM(G28:BF28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BD28),1)</f>
+        <f>ROUND(AVERAGE(G28:BF28),1)</f>
         <v/>
       </c>
       <c r="G28" s="79" t="n">
@@ -15063,6 +15101,12 @@
         <v>3</v>
       </c>
       <c r="BD28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF28" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15073,20 +15117,20 @@
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BD29)</f>
+        <f>SUM(G29:BF29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BD29),1)</f>
+        <f>ROUND(AVERAGE(G29:BF29),1)</f>
         <v/>
       </c>
       <c r="U29" s="79" t="n">
@@ -15174,6 +15218,14 @@
       </c>
       <c r="BD29" t="n">
         <v>3</v>
+      </c>
+      <c r="BE29" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -15192,11 +15244,11 @@
         <v>5</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BD30)</f>
+        <f>SUM(G30:BF30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BD30),1)</f>
+        <f>ROUND(AVERAGE(G30:BF30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15239,20 +15291,20 @@
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BD31)</f>
+        <f>SUM(G31:BF31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BD31),1)</f>
+        <f>ROUND(AVERAGE(G31:BF31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
@@ -15278,6 +15330,14 @@
       </c>
       <c r="AZ31" t="n">
         <v>2</v>
+      </c>
+      <c r="BE31" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -15293,14 +15353,14 @@
         <v>0</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BD32)</f>
+        <f>SUM(G32:BF32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BD32),1)</f>
+        <f>ROUND(AVERAGE(G32:BF32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
@@ -15344,6 +15404,12 @@
       </c>
       <c r="BD32" t="n">
         <v>2</v>
+      </c>
+      <c r="BE32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -15362,11 +15428,11 @@
         <v>0</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BD33)</f>
+        <f>SUM(G33:BF33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BD33),1)</f>
+        <f>ROUND(AVERAGE(G33:BF33),1)</f>
         <v/>
       </c>
     </row>
@@ -15386,11 +15452,11 @@
         <v>4</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BD34)</f>
+        <f>SUM(G34:BF34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BD34),1)</f>
+        <f>ROUND(AVERAGE(G34:BF34),1)</f>
         <v/>
       </c>
       <c r="AM34" t="n">
@@ -15438,11 +15504,11 @@
         <v>7</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BD35)</f>
+        <f>SUM(G35:BF35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BD35),1)</f>
+        <f>ROUND(AVERAGE(G35:BF35),1)</f>
         <v/>
       </c>
       <c r="AM35" t="n">
@@ -15491,7 +15557,7 @@
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>fede61mito</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
@@ -15501,21 +15567,27 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BD36)</f>
+        <f>SUM(G36:BF36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BD36),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G36:BF36),1)</f>
+        <v/>
+      </c>
+      <c r="BE36" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF36" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
@@ -15528,18 +15600,18 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BD37)</f>
+        <f>SUM(G37:BF37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BD37),1)</f>
+        <f>ROUND(AVERAGE(G37:BF37),1)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
@@ -15549,21 +15621,27 @@
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BD38)</f>
+        <f>SUM(G38:BF38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BD38),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G38:BF38),1)</f>
+        <v/>
+      </c>
+      <c r="BA38" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB38" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
@@ -15573,31 +15651,37 @@
         <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BD39)</f>
+        <f>SUM(G39:BF39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BD39),1)</f>
+        <f>ROUND(AVERAGE(G39:BF39),1)</f>
         <v/>
       </c>
       <c r="BA39" t="n">
         <v>2</v>
       </c>
       <c r="BB39" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="BE39" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF39" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" s="68" t="n">
         <v>0</v>
@@ -15606,49 +15690,55 @@
         <v>1</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BD40)</f>
+        <f>SUM(G40:BF40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BD40),1)</f>
-        <v/>
-      </c>
-      <c r="BA40" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB40" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G40:BF40),1)</f>
+        <v/>
+      </c>
+      <c r="BE40" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>thommyspine</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BD41)</f>
+        <f>SUM(G41:BF41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BD41),1)</f>
-        <v/>
-      </c>
-      <c r="BC41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BD41" t="inlineStr">
+        <f>ROUND(AVERAGE(G41:BF41),1)</f>
+        <v/>
+      </c>
+      <c r="BC41" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD41" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF41" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15657,31 +15747,41 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BD42)</f>
+        <f>SUM(G42:BF42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BD42),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G42:BF42),1)</f>
+        <v/>
+      </c>
+      <c r="BC42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -15694,82 +15794,82 @@
         <v>1</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BD43)</f>
+        <f>SUM(G43:BF43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BD43),1)</f>
-        <v/>
-      </c>
-      <c r="BC43" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD43" t="n">
+        <f>ROUND(AVERAGE(G43:BF43),1)</f>
+        <v/>
+      </c>
+      <c r="BE43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF43" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BD44)</f>
+        <f>SUM(G44:BF44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BD44),1)</f>
-        <v/>
-      </c>
-      <c r="BC44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BD44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G44:BF44),1)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BD45)</f>
+        <f>SUM(G45:BF45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BD45),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G45:BF45),1)</f>
+        <v/>
+      </c>
+      <c r="BC45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -15782,52 +15882,42 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BD46)</f>
+        <f>SUM(G46:BF46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BD46),1)</f>
+        <f>ROUND(AVERAGE(G46:BF46),1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>Samu-Nighix</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BD47)</f>
+        <f>SUM(G47:BF47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BD47),1)</f>
-        <v/>
-      </c>
-      <c r="BC47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BD47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G47:BF47),1)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -15840,18 +15930,18 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BD48)</f>
+        <f>SUM(G48:BF48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BD48),1)</f>
+        <f>ROUND(AVERAGE(G48:BF48),1)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Samu-Nighix</t>
+          <t>Marchi™</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -15864,11 +15954,35 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BD49)</f>
+        <f>SUM(G49:BF49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BD49),1)</f>
+        <f>ROUND(AVERAGE(G49:BF49),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>Ernis</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:BF50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:BF50),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-18
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12456,7 +12456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI50"/>
+  <dimension ref="A1:CI49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -12807,12 +12807,12 @@
       </c>
       <c r="BG1" s="109" t="inlineStr">
         <is>
-          <t>Colonna59</t>
+          <t>WAR-27 (1)</t>
         </is>
       </c>
       <c r="BH1" s="109" t="inlineStr">
         <is>
-          <t>Colonna60</t>
+          <t>WAR-27 (2)</t>
         </is>
       </c>
       <c r="BI1" s="109" t="inlineStr">
@@ -12952,178 +12952,195 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="110" t="inlineStr">
-        <is>
-          <t>¥CATA¥</t>
-        </is>
-      </c>
-      <c r="B2" s="110" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" s="111" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="110" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="111">
-        <f>SUM(G2:BF2)</f>
+      <c r="A2" s="79" t="inlineStr">
+        <is>
+          <t>655321</t>
+        </is>
+      </c>
+      <c r="B2" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="68">
+        <f>SUM(G2:BH2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BF2),1)</f>
-        <v/>
-      </c>
-      <c r="G2" s="110" t="n"/>
-      <c r="H2" s="113" t="n"/>
-      <c r="I2" s="110" t="n"/>
-      <c r="J2" s="113" t="n"/>
-      <c r="K2" s="110" t="n"/>
-      <c r="L2" s="113" t="n"/>
-      <c r="M2" s="110" t="n"/>
-      <c r="N2" s="113" t="n"/>
-      <c r="O2" s="110" t="n"/>
-      <c r="P2" s="113" t="n"/>
-      <c r="Q2" s="110" t="n"/>
-      <c r="R2" s="113" t="n"/>
-      <c r="S2" s="110" t="n">
-        <v>2</v>
-      </c>
-      <c r="T2" s="113" t="n">
-        <v>3</v>
-      </c>
-      <c r="U2" s="110" t="n">
-        <v>2</v>
-      </c>
-      <c r="V2" s="113" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W2" s="110" t="n"/>
-      <c r="X2" s="113" t="n"/>
-      <c r="Y2" s="110" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z2" s="113" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="110" t="n"/>
-      <c r="AB2" s="113" t="n"/>
-      <c r="AC2" s="110" t="n"/>
-      <c r="AD2" s="113" t="n"/>
-      <c r="AE2" s="110" t="n"/>
-      <c r="AF2" s="113" t="n"/>
-      <c r="AG2" s="110" t="n"/>
-      <c r="AH2" s="113" t="n"/>
-      <c r="AI2" s="110" t="n"/>
-      <c r="AJ2" s="113" t="n"/>
-      <c r="AK2" s="110" t="n"/>
-      <c r="AL2" s="113" t="n"/>
-      <c r="AM2" s="110" t="n"/>
-      <c r="AN2" s="113" t="n"/>
-      <c r="AO2" s="110" t="n"/>
-      <c r="AP2" s="113" t="n"/>
-      <c r="AQ2" s="110" t="n"/>
-      <c r="AR2" s="113" t="n"/>
-      <c r="AS2" s="110" t="n"/>
-      <c r="AT2" s="113" t="n"/>
-      <c r="AU2" s="110" t="n"/>
-      <c r="AV2" s="113" t="n"/>
-      <c r="AW2" s="110" t="n"/>
-      <c r="AX2" s="113" t="n"/>
-      <c r="AY2" s="111" t="n"/>
-      <c r="AZ2" s="111" t="n"/>
-      <c r="BA2" s="111" t="n"/>
-      <c r="BB2" s="111" t="n"/>
-      <c r="BC2" s="111" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BD2" s="111" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BE2" s="111" t="n"/>
-      <c r="BF2" s="111" t="n"/>
-      <c r="BG2" s="111" t="n"/>
-      <c r="BH2" s="111" t="n"/>
-      <c r="BI2" s="111" t="n"/>
-      <c r="BJ2" s="111" t="n"/>
-      <c r="BK2" s="111" t="n"/>
-      <c r="BL2" s="111" t="n"/>
-      <c r="BM2" s="111" t="n"/>
-      <c r="BN2" s="111" t="n"/>
-      <c r="BO2" s="111" t="n"/>
-      <c r="BP2" s="111" t="n"/>
-      <c r="BQ2" s="111" t="n"/>
-      <c r="BR2" s="111" t="n"/>
-      <c r="BS2" s="111" t="n"/>
-      <c r="BT2" s="111" t="n"/>
-      <c r="BU2" s="111" t="n"/>
-      <c r="BV2" s="111" t="n"/>
-      <c r="BW2" s="111" t="n"/>
-      <c r="BX2" s="111" t="n"/>
-      <c r="BY2" s="111" t="n"/>
-      <c r="BZ2" s="111" t="n"/>
-      <c r="CA2" s="111" t="n"/>
-      <c r="CB2" s="111" t="n"/>
-      <c r="CC2" s="111" t="n"/>
-      <c r="CD2" s="111" t="n"/>
-      <c r="CE2" s="111" t="n"/>
-      <c r="CF2" s="111" t="n"/>
-      <c r="CG2" s="111" t="n"/>
-      <c r="CH2" s="111" t="n"/>
-      <c r="CI2" s="111" t="n"/>
+        <f>ROUND(AVERAGE(G2:BH2),1)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="79" t="inlineStr">
         <is>
-          <t>655321</t>
+          <t>alhfmfh</t>
         </is>
       </c>
       <c r="B3" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C3" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BF3)</f>
+        <f>SUM(G3:BH3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BF3),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G3:BH3),1)</f>
+        <v/>
+      </c>
+      <c r="AO3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BE3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="79" t="inlineStr">
         <is>
-          <t>alhfmfh</t>
+          <t>BigMc23</t>
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BF4)</f>
+        <f>SUM(G4:BH4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BF4),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G4:BH4),1)</f>
+        <v/>
+      </c>
+      <c r="G4" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="R4" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W4" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="X4" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Y4" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z4" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA4" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB4" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC4" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AD4" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>1</v>
       </c>
       <c r="AO4" t="n">
         <v>2</v>
@@ -13133,272 +13150,272 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AY4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BA4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="BE4" t="n">
         <v>2</v>
       </c>
       <c r="BF4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="79" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C5" s="68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BF5)</f>
+        <f>SUM(G5:BH5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BF5),1)</f>
-        <v/>
-      </c>
-      <c r="G5" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="80" t="n">
-        <v>0</v>
+        <f>ROUND(AVERAGE(G5:BH5),1)</f>
+        <v/>
       </c>
       <c r="K5" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L5" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M5" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="R5" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W5" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="X5" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y5" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z5" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA5" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB5" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC5" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AD5" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="Q5" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R5" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC5" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD5" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="AM5" t="n">
         <v>3</v>
       </c>
       <c r="AN5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AY5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BA5" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>3</v>
       </c>
       <c r="BE5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF5" t="n">
         <v>3</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="79" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BF6)</f>
+        <f>SUM(G6:BH6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BF6),1)</f>
-        <v/>
-      </c>
-      <c r="K6" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L6" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC6" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD6" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV6" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G6:BH6),1)</f>
+        <v/>
+      </c>
+      <c r="BA6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="79" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>dado</t>
         </is>
       </c>
       <c r="B7" s="79" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BF7)</f>
+        <f>SUM(G7:BH7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BF7),1)</f>
-        <v/>
-      </c>
-      <c r="BA7" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G7:BH7),1)</f>
+        <v/>
+      </c>
+      <c r="G7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V7" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W7" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X7" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y7" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA7" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB7" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC7" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD7" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BB7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13407,214 +13424,168 @@
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C8" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BF8)</f>
+        <f>SUM(G8:BH8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BF8),1)</f>
-        <v/>
-      </c>
-      <c r="G8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="S8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="U8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y8" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G8:BH8),1)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="79" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>ER DANDI 1927</t>
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BF9)</f>
+        <f>SUM(G9:BH9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BF9),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G9:BH9),1)</f>
+        <v/>
+      </c>
+      <c r="I9" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="O9" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="P9" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S9" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="79" t="inlineStr">
         <is>
-          <t>ER DANDI 1927</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="79" t="n">
         <v>7</v>
       </c>
-      <c r="C10" s="68" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="79" t="n">
-        <v>6</v>
-      </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BF10)</f>
+        <f>SUM(G10:BH10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BF10),1)</f>
-        <v/>
-      </c>
-      <c r="I10" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G10:BH10),1)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="U10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z10" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="O10" s="79" t="inlineStr">
+      <c r="AE10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="P10" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="S10" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK10" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
+      <c r="AZ10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13623,57 +13594,85 @@
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>gionny</t>
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C11" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BF11)</f>
+        <f>SUM(G11:BH11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BF11),1)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R11" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G11:BH11),1)</f>
+        <v/>
+      </c>
+      <c r="G11" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="U11" s="79" t="n">
         <v>3</v>
       </c>
       <c r="V11" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="W11" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="Y11" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z11" s="80" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB11" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF11" s="80" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AB11" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>2</v>
       </c>
       <c r="AS11" t="n">
         <v>1</v>
@@ -13681,399 +13680,431 @@
       <c r="AT11" t="n">
         <v>2</v>
       </c>
-      <c r="AY11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AZ11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="AU11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="79" t="inlineStr">
         <is>
-          <t>gionny</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BF12)</f>
+        <f>SUM(G12:BH12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BF12),1)</f>
-        <v/>
-      </c>
-      <c r="G12" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G12:BH12),1)</f>
+        <v/>
       </c>
       <c r="I12" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M12" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="80" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="79" t="n">
         <v>3</v>
       </c>
       <c r="P12" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R12" s="80" t="n">
         <v>3</v>
       </c>
       <c r="U12" s="79" t="n">
         <v>3</v>
       </c>
       <c r="V12" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W12" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="X12" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z12" s="80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB12" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC12" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD12" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF12" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL12" t="n">
         <v>2</v>
       </c>
       <c r="AM12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AO12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AP12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU12" t="n">
         <v>3</v>
       </c>
       <c r="AV12" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="79" t="inlineStr">
         <is>
-          <t>Giorgio</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B13" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C13" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="79" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BF13)</f>
+        <f>SUM(G13:BH13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BF13),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G13:BH13),1)</f>
+        <v/>
+      </c>
+      <c r="S13" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T13" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W13" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X13" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z13" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB13" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD13" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="79" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>HikariNoRob</t>
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C14" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BF14)</f>
+        <f>SUM(G14:BH14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BF14),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G14:BH14),1)</f>
+        <v/>
+      </c>
+      <c r="G14" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="I14" s="79" t="n">
         <v>3</v>
       </c>
       <c r="J14" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P14" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R14" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V14" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB14" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC14" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD14" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF14" s="80" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="Y14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB14" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD14" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B15" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C15" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BF15)</f>
+        <f>SUM(G15:BH15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BF15),1)</f>
-        <v/>
-      </c>
-      <c r="S15" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W15" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X15" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD15" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G15:BH15),1)</f>
+        <v/>
+      </c>
+      <c r="AE15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF15" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="BA15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="79" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B16" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C16" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BF16)</f>
+        <f>SUM(G16:BH16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BF16),1)</f>
-        <v/>
-      </c>
-      <c r="G16" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G16:BH16),1)</f>
+        <v/>
       </c>
       <c r="I16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J16" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z16" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="J16" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="M16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R16" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W16" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X16" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB16" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC16" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>1</v>
       </c>
       <c r="AY16" t="n">
         <v>3</v>
@@ -14082,182 +14113,266 @@
         <v>3</v>
       </c>
       <c r="BA16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BB16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH16" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BF17)</f>
+        <f>SUM(G17:BH17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BF17),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G17:BH17),1)</f>
+        <v/>
+      </c>
+      <c r="G17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S17" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X17" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AE17" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="AF17" s="80" t="n">
-        <v>1</v>
+      <c r="AF17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AS17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>2</v>
       </c>
       <c r="BA17" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB17" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BE17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BG17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="79" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B18" s="79" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BF18)</f>
+        <f>SUM(G18:BH18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BF18),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G18:BH18),1)</f>
+        <v/>
+      </c>
+      <c r="G18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I18" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="J18" s="80" t="inlineStr">
+      <c r="J18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M18" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="T18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V18" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE18" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF18" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="M18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q18" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R18" s="80" t="inlineStr">
+      <c r="AJ18" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="W18" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X18" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB18" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC18" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY18" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ18" t="n">
+      <c r="AK18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL18" t="n">
         <v>3</v>
       </c>
       <c r="BA18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B19" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="79" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="79" t="n">
-        <v>13</v>
-      </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BF19)</f>
+        <f>SUM(G19:BH19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BF19),1)</f>
-        <v/>
-      </c>
-      <c r="G19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H19" s="80" t="n">
-        <v>1</v>
+        <f>ROUND(AVERAGE(G19:BH19),1)</f>
+        <v/>
       </c>
       <c r="I19" s="79" t="n">
         <v>3</v>
@@ -14265,237 +14380,147 @@
       <c r="J19" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="M19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="80" t="n">
+        <v>3</v>
+      </c>
       <c r="O19" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="P19" s="80" t="inlineStr">
+      <c r="P19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="S19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T19" s="80" t="inlineStr">
+      <c r="AJ19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="W19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB19" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF19" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="AK19" t="n">
         <v>3</v>
       </c>
       <c r="AL19" t="n">
         <v>3</v>
       </c>
-      <c r="AO19" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AS19" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>2</v>
-      </c>
       <c r="BA19" t="n">
         <v>3</v>
       </c>
-      <c r="BB19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BE19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="BB19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BF20)</f>
+        <f>SUM(G20:BH20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BF20),1)</f>
-        <v/>
-      </c>
-      <c r="G20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V20" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G20:BH20),1)</f>
+        <v/>
+      </c>
+      <c r="Y20" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z20" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AC20" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD20" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="AE20" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF20" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB20" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C21" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="79" t="n">
         <v>9</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BF21)</f>
+        <f>SUM(G21:BH21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BF21),1)</f>
-        <v/>
-      </c>
-      <c r="I21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R21" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G21:BH21),1)</f>
+        <v/>
+      </c>
+      <c r="S21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="T21" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U21" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="V21" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="W21" s="79" t="n">
         <v>3</v>
@@ -14509,8 +14534,14 @@
       <c r="Z21" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="AC21" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD21" s="80" t="n">
+        <v>3</v>
+      </c>
       <c r="AE21" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF21" s="80" t="n">
         <v>3</v>
@@ -14526,154 +14557,198 @@
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA21" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB21" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD21" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="79" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BF22)</f>
+        <f>SUM(G22:BH22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BF22),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G22:BH22),1)</f>
+        <v/>
+      </c>
+      <c r="I22" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J22" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="K22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Q22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R22" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X22" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="Y22" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z22" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="Z22" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB22" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="AC22" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD22" s="80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE22" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF22" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BF23)</f>
+        <f>SUM(G23:BH23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BF23),1)</f>
-        <v/>
-      </c>
-      <c r="S23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U23" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G23:BH23),1)</f>
+        <v/>
+      </c>
+      <c r="G23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="V23" s="80" t="inlineStr">
+      <c r="BH23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="W23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI23" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ23" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL23" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC23" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD23" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
@@ -14683,95 +14758,103 @@
         <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BF24)</f>
+        <f>SUM(G24:BH24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BF24),1)</f>
-        <v/>
-      </c>
-      <c r="I24" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G24:BH24),1)</f>
+        <v/>
+      </c>
+      <c r="G24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="R24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="J24" s="80" t="inlineStr">
+      <c r="AJ24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="K24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M24" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Q24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z24" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB24" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC24" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD24" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF24" s="80" t="n">
-        <v>2</v>
+      <c r="AK24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>3</v>
       </c>
       <c r="AM24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN24" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B25" s="79" t="n">
@@ -14781,80 +14864,44 @@
         <v>0</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BF25)</f>
+        <f>SUM(G25:BH25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BF25),1)</f>
-        <v/>
-      </c>
-      <c r="G25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU25" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF25" t="n">
+        <f>ROUND(AVERAGE(G25:BH25),1)</f>
+        <v/>
+      </c>
+      <c r="AS25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT25" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B26" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C26" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BF26)</f>
+        <f>SUM(G26:BH26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BF26),1)</f>
+        <f>ROUND(AVERAGE(G26:BH26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -14864,51 +14911,61 @@
         <v>3</v>
       </c>
       <c r="I26" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J26" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L26" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="M26" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N26" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K26" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L26" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="O26" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P26" s="80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q26" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R26" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="U26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V26" s="80" t="n">
-        <v>2</v>
+      <c r="S26" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X26" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="Y26" s="79" t="n">
         <v>2</v>
       </c>
       <c r="Z26" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA26" s="79" t="n">
         <v>3</v>
       </c>
       <c r="AB26" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC26" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD26" s="80" t="n">
         <v>3</v>
       </c>
       <c r="AI26" t="inlineStr">
@@ -14937,148 +14994,194 @@
         <v>3</v>
       </c>
       <c r="AT26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BF27)</f>
+        <f>SUM(G27:BH27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BF27),1)</f>
-        <v/>
-      </c>
-      <c r="AS27" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT27" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G27:BH27),1)</f>
+        <v/>
+      </c>
+      <c r="U27" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V27" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X27" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Y27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z27" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA27" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB27" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD27" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE27" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF27" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AM27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>LucFir3</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BF28)</f>
+        <f>SUM(G28:BH28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BF28),1)</f>
-        <v/>
-      </c>
-      <c r="G28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G28:BH28),1)</f>
+        <v/>
+      </c>
+      <c r="AM28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="L28" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P28" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T28" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB28" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI28" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ28" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN28" t="n">
-        <v>3</v>
-      </c>
       <c r="AS28" t="n">
         <v>3</v>
       </c>
@@ -15086,141 +15189,67 @@
         <v>3</v>
       </c>
       <c r="AU28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA28" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB28" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BC28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BD28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="79" t="n">
-        <v>14</v>
-      </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BF29)</f>
+        <f>SUM(G29:BH29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BF29),1)</f>
-        <v/>
-      </c>
-      <c r="U29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X29" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB29" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK29" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G29:BH29),1)</f>
+        <v/>
       </c>
       <c r="AM29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AP29" t="n">
         <v>3</v>
       </c>
+      <c r="AS29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>2</v>
+      </c>
       <c r="AY29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AZ29" t="n">
         <v>2</v>
       </c>
-      <c r="BA29" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD29" t="n">
-        <v>3</v>
-      </c>
       <c r="BE29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF29" t="inlineStr">
         <is>
@@ -15231,24 +15260,24 @@
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>LucFir3</t>
+          <t>Amazonie</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BF30)</f>
+        <f>SUM(G30:BH30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BF30),1)</f>
+        <f>ROUND(AVERAGE(G30:BH30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15258,12 +15287,10 @@
         <v>3</v>
       </c>
       <c r="AO30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>2</v>
       </c>
       <c r="AS30" t="n">
         <v>3</v>
@@ -15272,69 +15299,89 @@
         <v>3</v>
       </c>
       <c r="AU30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV30" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>3</v>
       </c>
       <c r="BC30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BD30" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="BE30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BF31)</f>
+        <f>SUM(G31:BH31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BF31),1)</f>
+        <f>ROUND(AVERAGE(G31:BH31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AO31" t="n">
         <v>3</v>
       </c>
       <c r="AP31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT31" t="n">
-        <v>2</v>
-      </c>
-      <c r="AY31" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ31" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE31" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF31" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BA31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BB31" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15343,7 +15390,7 @@
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>Amazonie</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
@@ -15356,15 +15403,15 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BF32)</f>
+        <f>SUM(G32:BH32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BF32),1)</f>
+        <f>ROUND(AVERAGE(G32:BH32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN32" t="n">
         <v>3</v>
@@ -15373,16 +15420,16 @@
         <v>3</v>
       </c>
       <c r="AP32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AV32" t="n">
         <v>3</v>
@@ -15391,31 +15438,31 @@
         <v>3</v>
       </c>
       <c r="AZ32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BA32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BB32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BC32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BD32" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE32" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH32" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>terracrom</t>
+          <t>Dasters79</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
@@ -15425,73 +15472,51 @@
         <v>0</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BF33)</f>
+        <f>SUM(G33:BH33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BF33),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G33:BH33),1)</f>
+        <v/>
+      </c>
+      <c r="BE33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>VERRETHERULER</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C34" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BF34)</f>
+        <f>SUM(G34:BH34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BF34),1)</f>
-        <v/>
-      </c>
-      <c r="AM34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO34" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP34" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT34" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G34:BH34),1)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>GGfresco_08</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
@@ -15501,63 +15526,27 @@
         <v>0</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BF35)</f>
+        <f>SUM(G35:BH35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BF35),1)</f>
-        <v/>
-      </c>
-      <c r="AM35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU35" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY35" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ35" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G35:BH35),1)</f>
+        <v/>
       </c>
       <c r="BA35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BB35" t="n">
-        <v>2</v>
-      </c>
-      <c r="BC35" t="n">
-        <v>1</v>
-      </c>
-      <c r="BD35" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>Dasters79</t>
+          <t>PESCARA MANZIA</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
@@ -15567,140 +15556,188 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BF36)</f>
+        <f>SUM(G36:BH36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BF36),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G36:BH36),1)</f>
+        <v/>
+      </c>
+      <c r="BA36" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB36" t="n">
+        <v>2</v>
       </c>
       <c r="BE36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>VERRETHERULER</t>
+          <t>BigGiurz08</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BF37)</f>
+        <f>SUM(G37:BH37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BF37),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G37:BH37),1)</f>
+        <v/>
+      </c>
+      <c r="BE37" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF37" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BG37" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH37" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>GGfresco_08</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BF38)</f>
+        <f>SUM(G38:BH38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BF38),1)</f>
-        <v/>
-      </c>
-      <c r="BA38" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB38" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G38:BH38),1)</f>
+        <v/>
+      </c>
+      <c r="BC38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BG38" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH38" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>PESCARA MANZIA</t>
+          <t>StepanYT Ita Uk</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C39" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="79" t="n">
         <v>2</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BF39)</f>
+        <f>SUM(G39:BH39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BF39),1)</f>
-        <v/>
-      </c>
-      <c r="BA39" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB39" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE39" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF39" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G39:BH39),1)</f>
+        <v/>
+      </c>
+      <c r="BC39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BD39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BG39" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>BigGiurz08</t>
+          <t>omar</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BF40)</f>
+        <f>SUM(G40:BH40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BF40),1)</f>
+        <f>ROUND(AVERAGE(G40:BH40),1)</f>
         <v/>
       </c>
       <c r="BE40" t="n">
-        <v>2</v>
-      </c>
-      <c r="BF40" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="BF40" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BH40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15709,45 +15746,31 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Alessio9797</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C41" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BF41)</f>
+        <f>SUM(G41:BH41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BF41),1)</f>
-        <v/>
-      </c>
-      <c r="BC41" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD41" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE41" t="n">
-        <v>1</v>
-      </c>
-      <c r="BF41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G41:BH41),1)</f>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>StepanYT Ita Uk</t>
+          <t>Mario</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
@@ -15760,11 +15783,11 @@
         <v>1</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BF42)</f>
+        <f>SUM(G42:BH42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BF42),1)</f>
+        <f>ROUND(AVERAGE(G42:BH42),1)</f>
         <v/>
       </c>
       <c r="BC42" t="inlineStr">
@@ -15781,7 +15804,7 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>omar</t>
+          <t>papi</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -15791,27 +15814,21 @@
         <v>0</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BF43)</f>
+        <f>SUM(G43:BH43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BF43),1)</f>
-        <v/>
-      </c>
-      <c r="BE43" t="n">
-        <v>1</v>
-      </c>
-      <c r="BF43" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G43:BH43),1)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>Alessio9797</t>
+          <t>jacopo</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -15824,52 +15841,42 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BF44)</f>
+        <f>SUM(G44:BH44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BF44),1)</f>
+        <f>ROUND(AVERAGE(G44:BH44),1)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>king</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BF45)</f>
+        <f>SUM(G45:BH45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BF45),1)</f>
-        <v/>
-      </c>
-      <c r="BC45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BD45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G45:BH45),1)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>papi</t>
+          <t>antony</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -15882,18 +15889,18 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BF46)</f>
+        <f>SUM(G46:BH46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BF46),1)</f>
+        <f>ROUND(AVERAGE(G46:BH46),1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>Samu-Nighix</t>
+          <t>Fra</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -15906,18 +15913,18 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BF47)</f>
+        <f>SUM(G47:BH47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BF47),1)</f>
+        <f>ROUND(AVERAGE(G47:BH47),1)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>jacopo</t>
+          <t>Spiderman</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -15930,18 +15937,18 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BF48)</f>
+        <f>SUM(G48:BH48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BF48),1)</f>
+        <f>ROUND(AVERAGE(G48:BH48),1)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Marchi™</t>
+          <t>perte</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -15954,35 +15961,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BF49)</f>
+        <f>SUM(G49:BH49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BF49),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>Ernis</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:BF50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BF50),1)</f>
+        <f>ROUND(AVERAGE(G49:BH49),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-20
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12456,7 +12456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI49"/>
+  <dimension ref="A1:CI51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -12817,12 +12817,12 @@
       </c>
       <c r="BI1" s="109" t="inlineStr">
         <is>
-          <t>Colonna61</t>
+          <t>WAR-28 (1)</t>
         </is>
       </c>
       <c r="BJ1" s="109" t="inlineStr">
         <is>
-          <t>Colonna62</t>
+          <t>WAR-28 (2)</t>
         </is>
       </c>
       <c r="BK1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BH2)</f>
+        <f>SUM(G2:BJ2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BH2),1)</f>
+        <f>ROUND(AVERAGE(G2:BJ2),1)</f>
         <v/>
       </c>
     </row>
@@ -12991,11 +12991,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BH3)</f>
+        <f>SUM(G3:BJ3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BH3),1)</f>
+        <f>ROUND(AVERAGE(G3:BJ3),1)</f>
         <v/>
       </c>
       <c r="AO3" t="n">
@@ -13036,14 +13036,14 @@
         <v>5</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BH4)</f>
+        <f>SUM(G4:BJ4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BH4),1)</f>
+        <f>ROUND(AVERAGE(G4:BJ4),1)</f>
         <v/>
       </c>
       <c r="G4" s="79" t="n">
@@ -13180,6 +13180,12 @@
         <v>2</v>
       </c>
       <c r="BF4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13199,11 +13205,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BH5)</f>
+        <f>SUM(G5:BJ5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BH5),1)</f>
+        <f>ROUND(AVERAGE(G5:BJ5),1)</f>
         <v/>
       </c>
       <c r="K5" s="79" t="n">
@@ -13277,11 +13283,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BH6)</f>
+        <f>SUM(G6:BJ6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BH6),1)</f>
+        <f>ROUND(AVERAGE(G6:BJ6),1)</f>
         <v/>
       </c>
       <c r="BA6" t="n">
@@ -13309,11 +13315,11 @@
         <v>16</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BH7)</f>
+        <f>SUM(G7:BJ7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BH7),1)</f>
+        <f>ROUND(AVERAGE(G7:BJ7),1)</f>
         <v/>
       </c>
       <c r="G7" s="79" t="n">
@@ -13437,11 +13443,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BH8)</f>
+        <f>SUM(G8:BJ8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BH8),1)</f>
+        <f>ROUND(AVERAGE(G8:BJ8),1)</f>
         <v/>
       </c>
     </row>
@@ -13461,11 +13467,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BH9)</f>
+        <f>SUM(G9:BJ9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BH9),1)</f>
+        <f>ROUND(AVERAGE(G9:BJ9),1)</f>
         <v/>
       </c>
       <c r="I9" s="79" t="n">
@@ -13535,11 +13541,11 @@
         <v>7</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BH10)</f>
+        <f>SUM(G10:BJ10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BH10),1)</f>
+        <f>ROUND(AVERAGE(G10:BJ10),1)</f>
         <v/>
       </c>
       <c r="Q10" s="79" t="n">
@@ -13598,20 +13604,20 @@
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BH11)</f>
+        <f>SUM(G11:BJ11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BH11),1)</f>
+        <f>ROUND(AVERAGE(G11:BJ11),1)</f>
         <v/>
       </c>
       <c r="G11" s="79" t="n">
@@ -13691,6 +13697,14 @@
       </c>
       <c r="BH11" t="n">
         <v>1</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -13706,14 +13720,14 @@
         <v>1</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BH12)</f>
+        <f>SUM(G12:BJ12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BH12),1)</f>
+        <f>ROUND(AVERAGE(G12:BJ12),1)</f>
         <v/>
       </c>
       <c r="I12" s="79" t="n">
@@ -13824,6 +13838,12 @@
         <v>3</v>
       </c>
       <c r="BD12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ12" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13843,11 +13863,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BH13)</f>
+        <f>SUM(G13:BJ13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BH13),1)</f>
+        <f>ROUND(AVERAGE(G13:BJ13),1)</f>
         <v/>
       </c>
       <c r="S13" s="79" t="n">
@@ -13931,11 +13951,11 @@
         <v>8</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BH14)</f>
+        <f>SUM(G14:BJ14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BH14),1)</f>
+        <f>ROUND(AVERAGE(G14:BJ14),1)</f>
         <v/>
       </c>
       <c r="G14" s="79" t="n">
@@ -14002,14 +14022,14 @@
         <v>0</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BH15)</f>
+        <f>SUM(G15:BJ15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BH15),1)</f>
+        <f>ROUND(AVERAGE(G15:BJ15),1)</f>
         <v/>
       </c>
       <c r="AE15" s="79" t="n">
@@ -14023,6 +14043,12 @@
       </c>
       <c r="BB15" t="n">
         <v>2</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -14041,11 +14067,11 @@
         <v>12</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BH16)</f>
+        <f>SUM(G16:BJ16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BH16),1)</f>
+        <f>ROUND(AVERAGE(G16:BJ16),1)</f>
         <v/>
       </c>
       <c r="I16" s="79" t="n">
@@ -14141,11 +14167,11 @@
         <v>14</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BH17)</f>
+        <f>SUM(G17:BJ17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BH17),1)</f>
+        <f>ROUND(AVERAGE(G17:BJ17),1)</f>
         <v/>
       </c>
       <c r="G17" s="79" t="n">
@@ -14267,11 +14293,11 @@
         <v>12</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BH18)</f>
+        <f>SUM(G18:BJ18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BH18),1)</f>
+        <f>ROUND(AVERAGE(G18:BJ18),1)</f>
         <v/>
       </c>
       <c r="G18" s="79" t="n">
@@ -14367,11 +14393,11 @@
         <v>9</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BH19)</f>
+        <f>SUM(G19:BJ19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BH19),1)</f>
+        <f>ROUND(AVERAGE(G19:BJ19),1)</f>
         <v/>
       </c>
       <c r="I19" s="79" t="n">
@@ -14455,11 +14481,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BH20)</f>
+        <f>SUM(G20:BJ20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BH20),1)</f>
+        <f>ROUND(AVERAGE(G20:BJ20),1)</f>
         <v/>
       </c>
       <c r="Y20" s="79" t="n">
@@ -14490,20 +14516,20 @@
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C21" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BH21)</f>
+        <f>SUM(G21:BJ21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BH21),1)</f>
+        <f>ROUND(AVERAGE(G21:BJ21),1)</f>
         <v/>
       </c>
       <c r="S21" s="79" t="n">
@@ -14569,6 +14595,16 @@
       </c>
       <c r="BD21" t="n">
         <v>2</v>
+      </c>
+      <c r="BI21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -14587,11 +14623,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BH22)</f>
+        <f>SUM(G22:BJ22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BH22),1)</f>
+        <f>ROUND(AVERAGE(G22:BJ22),1)</f>
         <v/>
       </c>
       <c r="I22" s="79" t="inlineStr">
@@ -14685,11 +14721,11 @@
         <v>8</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BH23)</f>
+        <f>SUM(G23:BJ23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BH23),1)</f>
+        <f>ROUND(AVERAGE(G23:BJ23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
@@ -14761,11 +14797,11 @@
         <v>12</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BH24)</f>
+        <f>SUM(G24:BJ24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BH24),1)</f>
+        <f>ROUND(AVERAGE(G24:BJ24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -14867,11 +14903,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BH25)</f>
+        <f>SUM(G25:BJ25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BH25),1)</f>
+        <f>ROUND(AVERAGE(G25:BJ25),1)</f>
         <v/>
       </c>
       <c r="AS25" t="n">
@@ -14897,11 +14933,11 @@
         <v>19</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BH26)</f>
+        <f>SUM(G26:BJ26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BH26),1)</f>
+        <f>ROUND(AVERAGE(G26:BJ26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -15043,11 +15079,11 @@
         <v>14</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BH27)</f>
+        <f>SUM(G27:BJ27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BH27),1)</f>
+        <f>ROUND(AVERAGE(G27:BJ27),1)</f>
         <v/>
       </c>
       <c r="U27" s="79" t="n">
@@ -15161,11 +15197,11 @@
         <v>5</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BH28)</f>
+        <f>SUM(G28:BJ28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BH28),1)</f>
+        <f>ROUND(AVERAGE(G28:BJ28),1)</f>
         <v/>
       </c>
       <c r="AM28" t="n">
@@ -15217,11 +15253,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BH29)</f>
+        <f>SUM(G29:BJ29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BH29),1)</f>
+        <f>ROUND(AVERAGE(G29:BJ29),1)</f>
         <v/>
       </c>
       <c r="AM29" t="n">
@@ -15273,11 +15309,11 @@
         <v>9</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BH30)</f>
+        <f>SUM(G30:BJ30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BH30),1)</f>
+        <f>ROUND(AVERAGE(G30:BJ30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15351,11 +15387,11 @@
         <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BH31)</f>
+        <f>SUM(G31:BJ31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BH31),1)</f>
+        <f>ROUND(AVERAGE(G31:BJ31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
@@ -15403,11 +15439,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BH32)</f>
+        <f>SUM(G32:BJ32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BH32),1)</f>
+        <f>ROUND(AVERAGE(G32:BJ32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
@@ -15475,11 +15511,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BH33)</f>
+        <f>SUM(G33:BJ33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BH33),1)</f>
+        <f>ROUND(AVERAGE(G33:BJ33),1)</f>
         <v/>
       </c>
       <c r="BE33" t="n">
@@ -15505,11 +15541,11 @@
         <v>0</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BH34)</f>
+        <f>SUM(G34:BJ34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BH34),1)</f>
+        <f>ROUND(AVERAGE(G34:BJ34),1)</f>
         <v/>
       </c>
     </row>
@@ -15529,11 +15565,11 @@
         <v>1</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BH35)</f>
+        <f>SUM(G35:BJ35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BH35),1)</f>
+        <f>ROUND(AVERAGE(G35:BJ35),1)</f>
         <v/>
       </c>
       <c r="BA35" t="n">
@@ -15550,20 +15586,20 @@
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BH36)</f>
+        <f>SUM(G36:BJ36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BH36),1)</f>
+        <f>ROUND(AVERAGE(G36:BJ36),1)</f>
         <v/>
       </c>
       <c r="BA36" t="n">
@@ -15577,6 +15613,14 @@
       </c>
       <c r="BF36" t="n">
         <v>2</v>
+      </c>
+      <c r="BI36" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -15595,11 +15639,11 @@
         <v>2</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BH37)</f>
+        <f>SUM(G37:BJ37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BH37),1)</f>
+        <f>ROUND(AVERAGE(G37:BJ37),1)</f>
         <v/>
       </c>
       <c r="BE37" t="n">
@@ -15630,14 +15674,14 @@
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BH38)</f>
+        <f>SUM(G38:BJ38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BH38),1)</f>
+        <f>ROUND(AVERAGE(G38:BJ38),1)</f>
         <v/>
       </c>
       <c r="BC38" t="n">
@@ -15659,6 +15703,12 @@
       </c>
       <c r="BH38" t="n">
         <v>2</v>
+      </c>
+      <c r="BI38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ38" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -15668,20 +15718,20 @@
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BH39)</f>
+        <f>SUM(G39:BJ39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BH39),1)</f>
+        <f>ROUND(AVERAGE(G39:BJ39),1)</f>
         <v/>
       </c>
       <c r="BC39" t="inlineStr">
@@ -15698,6 +15748,14 @@
         <v>2</v>
       </c>
       <c r="BH39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BI39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ39" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15719,11 +15777,11 @@
         <v>2</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BH40)</f>
+        <f>SUM(G40:BJ40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BH40),1)</f>
+        <f>ROUND(AVERAGE(G40:BJ40),1)</f>
         <v/>
       </c>
       <c r="BE40" t="n">
@@ -15759,11 +15817,11 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BH41)</f>
+        <f>SUM(G41:BJ41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BH41),1)</f>
+        <f>ROUND(AVERAGE(G41:BJ41),1)</f>
         <v/>
       </c>
     </row>
@@ -15783,11 +15841,11 @@
         <v>1</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BH42)</f>
+        <f>SUM(G42:BJ42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BH42),1)</f>
+        <f>ROUND(AVERAGE(G42:BJ42),1)</f>
         <v/>
       </c>
       <c r="BC42" t="inlineStr">
@@ -15817,11 +15875,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BH43)</f>
+        <f>SUM(G43:BJ43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BH43),1)</f>
+        <f>ROUND(AVERAGE(G43:BJ43),1)</f>
         <v/>
       </c>
     </row>
@@ -15841,18 +15899,18 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BH44)</f>
+        <f>SUM(G44:BJ44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BH44),1)</f>
+        <f>ROUND(AVERAGE(G44:BJ44),1)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>king</t>
+          <t>antony</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -15862,21 +15920,27 @@
         <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BH45)</f>
+        <f>SUM(G45:BJ45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BH45),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G45:BJ45),1)</f>
+        <v/>
+      </c>
+      <c r="BI45" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ45" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>antony</t>
+          <t>Fra</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -15889,18 +15953,18 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BH46)</f>
+        <f>SUM(G46:BJ46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BH46),1)</f>
+        <f>ROUND(AVERAGE(G46:BJ46),1)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>Fra</t>
+          <t>Spiderman</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -15913,18 +15977,18 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BH47)</f>
+        <f>SUM(G47:BJ47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BH47),1)</f>
+        <f>ROUND(AVERAGE(G47:BJ47),1)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>Spiderman</t>
+          <t>perte</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -15937,18 +16001,18 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BH48)</f>
+        <f>SUM(G48:BJ48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BH48),1)</f>
+        <f>ROUND(AVERAGE(G48:BJ48),1)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>perte</t>
+          <t>EMANUELE</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -15961,11 +16025,69 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BH49)</f>
+        <f>SUM(G49:BJ49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BH49),1)</f>
+        <f>ROUND(AVERAGE(G49:BJ49),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>micky</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:BJ50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:BJ50),1)</f>
+        <v/>
+      </c>
+      <c r="BI50" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BJ50" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>TaifTuff</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="68">
+        <f>SUM(G51:BJ51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="68">
+        <f>ROUND(AVERAGE(G51:BJ51),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-22
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12827,12 +12827,12 @@
       </c>
       <c r="BK1" s="109" t="inlineStr">
         <is>
-          <t>Colonna63</t>
+          <t>WAR-29 (1)</t>
         </is>
       </c>
       <c r="BL1" s="109" t="inlineStr">
         <is>
-          <t>Colonna64</t>
+          <t>WAR-29 (2)</t>
         </is>
       </c>
       <c r="BM1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BJ2)</f>
+        <f>SUM(G2:BL2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BJ2),1)</f>
+        <f>ROUND(AVERAGE(G2:BL2),1)</f>
         <v/>
       </c>
     </row>
@@ -12991,11 +12991,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BJ3)</f>
+        <f>SUM(G3:BL3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BJ3),1)</f>
+        <f>ROUND(AVERAGE(G3:BL3),1)</f>
         <v/>
       </c>
       <c r="AO3" t="n">
@@ -13036,14 +13036,14 @@
         <v>5</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BJ4)</f>
+        <f>SUM(G4:BL4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BJ4),1)</f>
+        <f>ROUND(AVERAGE(G4:BL4),1)</f>
         <v/>
       </c>
       <c r="G4" s="79" t="n">
@@ -13187,6 +13187,12 @@
       </c>
       <c r="BJ4" t="n">
         <v>3</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -13205,11 +13211,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BJ5)</f>
+        <f>SUM(G5:BL5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BJ5),1)</f>
+        <f>ROUND(AVERAGE(G5:BL5),1)</f>
         <v/>
       </c>
       <c r="K5" s="79" t="n">
@@ -13283,11 +13289,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BJ6)</f>
+        <f>SUM(G6:BL6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BJ6),1)</f>
+        <f>ROUND(AVERAGE(G6:BL6),1)</f>
         <v/>
       </c>
       <c r="BA6" t="n">
@@ -13315,11 +13321,11 @@
         <v>16</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BJ7)</f>
+        <f>SUM(G7:BL7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BJ7),1)</f>
+        <f>ROUND(AVERAGE(G7:BL7),1)</f>
         <v/>
       </c>
       <c r="G7" s="79" t="n">
@@ -13443,11 +13449,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BJ8)</f>
+        <f>SUM(G8:BL8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BJ8),1)</f>
+        <f>ROUND(AVERAGE(G8:BL8),1)</f>
         <v/>
       </c>
     </row>
@@ -13467,11 +13473,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BJ9)</f>
+        <f>SUM(G9:BL9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BJ9),1)</f>
+        <f>ROUND(AVERAGE(G9:BL9),1)</f>
         <v/>
       </c>
       <c r="I9" s="79" t="n">
@@ -13532,20 +13538,20 @@
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BJ10)</f>
+        <f>SUM(G10:BL10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BJ10),1)</f>
+        <f>ROUND(AVERAGE(G10:BL10),1)</f>
         <v/>
       </c>
       <c r="Q10" s="79" t="n">
@@ -13592,6 +13598,16 @@
         </is>
       </c>
       <c r="AZ10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13610,14 +13626,14 @@
         <v>0</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BJ11)</f>
+        <f>SUM(G11:BL11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BJ11),1)</f>
+        <f>ROUND(AVERAGE(G11:BL11),1)</f>
         <v/>
       </c>
       <c r="G11" s="79" t="n">
@@ -13705,6 +13721,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BK11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -13714,20 +13736,20 @@
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BJ12)</f>
+        <f>SUM(G12:BL12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BJ12),1)</f>
+        <f>ROUND(AVERAGE(G12:BL12),1)</f>
         <v/>
       </c>
       <c r="I12" s="79" t="n">
@@ -13845,6 +13867,14 @@
       </c>
       <c r="BJ12" t="n">
         <v>3</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -13863,11 +13893,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BJ13)</f>
+        <f>SUM(G13:BL13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BJ13),1)</f>
+        <f>ROUND(AVERAGE(G13:BL13),1)</f>
         <v/>
       </c>
       <c r="S13" s="79" t="n">
@@ -13951,11 +13981,11 @@
         <v>8</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BJ14)</f>
+        <f>SUM(G14:BL14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BJ14),1)</f>
+        <f>ROUND(AVERAGE(G14:BL14),1)</f>
         <v/>
       </c>
       <c r="G14" s="79" t="n">
@@ -14025,11 +14055,11 @@
         <v>3</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BJ15)</f>
+        <f>SUM(G15:BL15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BJ15),1)</f>
+        <f>ROUND(AVERAGE(G15:BL15),1)</f>
         <v/>
       </c>
       <c r="AE15" s="79" t="n">
@@ -14064,14 +14094,14 @@
         <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BJ16)</f>
+        <f>SUM(G16:BL16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BJ16),1)</f>
+        <f>ROUND(AVERAGE(G16:BL16),1)</f>
         <v/>
       </c>
       <c r="I16" s="79" t="n">
@@ -14149,6 +14179,12 @@
       </c>
       <c r="BH16" t="n">
         <v>3</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -14158,20 +14194,20 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BJ17)</f>
+        <f>SUM(G17:BL17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BJ17),1)</f>
+        <f>ROUND(AVERAGE(G17:BL17),1)</f>
         <v/>
       </c>
       <c r="G17" s="79" t="n">
@@ -14275,6 +14311,14 @@
       </c>
       <c r="BH17" t="n">
         <v>3</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -14290,14 +14334,14 @@
         <v>1</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BJ18)</f>
+        <f>SUM(G18:BL18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BJ18),1)</f>
+        <f>ROUND(AVERAGE(G18:BL18),1)</f>
         <v/>
       </c>
       <c r="G18" s="79" t="n">
@@ -14374,6 +14418,12 @@
         <v>3</v>
       </c>
       <c r="BB18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14393,11 +14443,11 @@
         <v>9</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BJ19)</f>
+        <f>SUM(G19:BL19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BJ19),1)</f>
+        <f>ROUND(AVERAGE(G19:BL19),1)</f>
         <v/>
       </c>
       <c r="I19" s="79" t="n">
@@ -14481,11 +14531,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BJ20)</f>
+        <f>SUM(G20:BL20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BJ20),1)</f>
+        <f>ROUND(AVERAGE(G20:BL20),1)</f>
         <v/>
       </c>
       <c r="Y20" s="79" t="n">
@@ -14525,11 +14575,11 @@
         <v>10</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BJ21)</f>
+        <f>SUM(G21:BL21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BJ21),1)</f>
+        <f>ROUND(AVERAGE(G21:BL21),1)</f>
         <v/>
       </c>
       <c r="S21" s="79" t="n">
@@ -14623,11 +14673,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BJ22)</f>
+        <f>SUM(G22:BL22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BJ22),1)</f>
+        <f>ROUND(AVERAGE(G22:BL22),1)</f>
         <v/>
       </c>
       <c r="I22" s="79" t="inlineStr">
@@ -14721,11 +14771,11 @@
         <v>8</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BJ23)</f>
+        <f>SUM(G23:BL23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BJ23),1)</f>
+        <f>ROUND(AVERAGE(G23:BL23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
@@ -14797,11 +14847,11 @@
         <v>12</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BJ24)</f>
+        <f>SUM(G24:BL24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BJ24),1)</f>
+        <f>ROUND(AVERAGE(G24:BL24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -14903,11 +14953,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BJ25)</f>
+        <f>SUM(G25:BL25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BJ25),1)</f>
+        <f>ROUND(AVERAGE(G25:BL25),1)</f>
         <v/>
       </c>
       <c r="AS25" t="n">
@@ -14930,14 +14980,14 @@
         <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BJ26)</f>
+        <f>SUM(G26:BL26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BJ26),1)</f>
+        <f>ROUND(AVERAGE(G26:BL26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -15061,6 +15111,12 @@
       </c>
       <c r="BH26" t="n">
         <v>3</v>
+      </c>
+      <c r="BK26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL26" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -15079,11 +15135,11 @@
         <v>14</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BJ27)</f>
+        <f>SUM(G27:BL27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BJ27),1)</f>
+        <f>ROUND(AVERAGE(G27:BL27),1)</f>
         <v/>
       </c>
       <c r="U27" s="79" t="n">
@@ -15197,11 +15253,11 @@
         <v>5</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BJ28)</f>
+        <f>SUM(G28:BL28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BJ28),1)</f>
+        <f>ROUND(AVERAGE(G28:BL28),1)</f>
         <v/>
       </c>
       <c r="AM28" t="n">
@@ -15253,11 +15309,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BJ29)</f>
+        <f>SUM(G29:BL29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BJ29),1)</f>
+        <f>ROUND(AVERAGE(G29:BL29),1)</f>
         <v/>
       </c>
       <c r="AM29" t="n">
@@ -15309,11 +15365,11 @@
         <v>9</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BJ30)</f>
+        <f>SUM(G30:BL30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BJ30),1)</f>
+        <f>ROUND(AVERAGE(G30:BL30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15387,11 +15443,11 @@
         <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BJ31)</f>
+        <f>SUM(G31:BL31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BJ31),1)</f>
+        <f>ROUND(AVERAGE(G31:BL31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
@@ -15436,14 +15492,14 @@
         <v>0</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BJ32)</f>
+        <f>SUM(G32:BL32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BJ32),1)</f>
+        <f>ROUND(AVERAGE(G32:BL32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
@@ -15492,6 +15548,12 @@
         <v>3</v>
       </c>
       <c r="BH32" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK32" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL32" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15511,11 +15573,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BJ33)</f>
+        <f>SUM(G33:BL33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BJ33),1)</f>
+        <f>ROUND(AVERAGE(G33:BL33),1)</f>
         <v/>
       </c>
       <c r="BE33" t="n">
@@ -15541,11 +15603,11 @@
         <v>0</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BJ34)</f>
+        <f>SUM(G34:BL34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BJ34),1)</f>
+        <f>ROUND(AVERAGE(G34:BL34),1)</f>
         <v/>
       </c>
     </row>
@@ -15565,11 +15627,11 @@
         <v>1</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BJ35)</f>
+        <f>SUM(G35:BL35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BJ35),1)</f>
+        <f>ROUND(AVERAGE(G35:BL35),1)</f>
         <v/>
       </c>
       <c r="BA35" t="n">
@@ -15586,20 +15648,20 @@
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BJ36)</f>
+        <f>SUM(G36:BL36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BJ36),1)</f>
+        <f>ROUND(AVERAGE(G36:BL36),1)</f>
         <v/>
       </c>
       <c r="BA36" t="n">
@@ -15618,6 +15680,14 @@
         <v>2</v>
       </c>
       <c r="BJ36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL36" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15639,11 +15709,11 @@
         <v>2</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BJ37)</f>
+        <f>SUM(G37:BL37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BJ37),1)</f>
+        <f>ROUND(AVERAGE(G37:BL37),1)</f>
         <v/>
       </c>
       <c r="BE37" t="n">
@@ -15674,14 +15744,14 @@
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BJ38)</f>
+        <f>SUM(G38:BL38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BJ38),1)</f>
+        <f>ROUND(AVERAGE(G38:BL38),1)</f>
         <v/>
       </c>
       <c r="BC38" t="n">
@@ -15709,6 +15779,12 @@
       </c>
       <c r="BJ38" t="n">
         <v>1</v>
+      </c>
+      <c r="BK38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL38" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -15718,20 +15794,20 @@
         </is>
       </c>
       <c r="B39" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="79" t="n">
         <v>4</v>
       </c>
-      <c r="C39" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="79" t="n">
-        <v>3</v>
-      </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BJ39)</f>
+        <f>SUM(G39:BL39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BJ39),1)</f>
+        <f>ROUND(AVERAGE(G39:BL39),1)</f>
         <v/>
       </c>
       <c r="BC39" t="inlineStr">
@@ -15756,6 +15832,14 @@
         <v>1</v>
       </c>
       <c r="BJ39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK39" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL39" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15768,20 +15852,20 @@
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C40" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BJ40)</f>
+        <f>SUM(G40:BL40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BJ40),1)</f>
+        <f>ROUND(AVERAGE(G40:BL40),1)</f>
         <v/>
       </c>
       <c r="BE40" t="n">
@@ -15796,6 +15880,14 @@
         </is>
       </c>
       <c r="BH40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15817,11 +15909,11 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BJ41)</f>
+        <f>SUM(G41:BL41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BJ41),1)</f>
+        <f>ROUND(AVERAGE(G41:BL41),1)</f>
         <v/>
       </c>
     </row>
@@ -15841,11 +15933,11 @@
         <v>1</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BJ42)</f>
+        <f>SUM(G42:BL42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BJ42),1)</f>
+        <f>ROUND(AVERAGE(G42:BL42),1)</f>
         <v/>
       </c>
       <c r="BC42" t="inlineStr">
@@ -15875,11 +15967,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BJ43)</f>
+        <f>SUM(G43:BL43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BJ43),1)</f>
+        <f>ROUND(AVERAGE(G43:BL43),1)</f>
         <v/>
       </c>
     </row>
@@ -15899,11 +15991,11 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BJ44)</f>
+        <f>SUM(G44:BL44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BJ44),1)</f>
+        <f>ROUND(AVERAGE(G44:BL44),1)</f>
         <v/>
       </c>
     </row>
@@ -15920,20 +16012,26 @@
         <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BJ45)</f>
+        <f>SUM(G45:BL45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BJ45),1)</f>
+        <f>ROUND(AVERAGE(G45:BL45),1)</f>
         <v/>
       </c>
       <c r="BI45" t="n">
         <v>3</v>
       </c>
       <c r="BJ45" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK45" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL45" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15953,11 +16051,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BJ46)</f>
+        <f>SUM(G46:BL46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BJ46),1)</f>
+        <f>ROUND(AVERAGE(G46:BL46),1)</f>
         <v/>
       </c>
     </row>
@@ -15977,11 +16075,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BJ47)</f>
+        <f>SUM(G47:BL47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BJ47),1)</f>
+        <f>ROUND(AVERAGE(G47:BL47),1)</f>
         <v/>
       </c>
     </row>
@@ -16001,11 +16099,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BJ48)</f>
+        <f>SUM(G48:BL48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BJ48),1)</f>
+        <f>ROUND(AVERAGE(G48:BL48),1)</f>
         <v/>
       </c>
     </row>
@@ -16025,11 +16123,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BJ49)</f>
+        <f>SUM(G49:BL49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BJ49),1)</f>
+        <f>ROUND(AVERAGE(G49:BL49),1)</f>
         <v/>
       </c>
     </row>
@@ -16040,20 +16138,20 @@
         </is>
       </c>
       <c r="B50" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C50" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50" s="68">
-        <f>SUM(G50:BJ50)</f>
+        <f>SUM(G50:BL50)</f>
         <v/>
       </c>
       <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BJ50),1)</f>
+        <f>ROUND(AVERAGE(G50:BL50),1)</f>
         <v/>
       </c>
       <c r="BI50" t="inlineStr">
@@ -16062,6 +16160,16 @@
         </is>
       </c>
       <c r="BJ50" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK50" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BL50" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16083,11 +16191,11 @@
         <v>0</v>
       </c>
       <c r="E51" s="68">
-        <f>SUM(G51:BJ51)</f>
+        <f>SUM(G51:BL51)</f>
         <v/>
       </c>
       <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:BJ51),1)</f>
+        <f>ROUND(AVERAGE(G51:BL51),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-24
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12837,12 +12837,12 @@
       </c>
       <c r="BM1" s="109" t="inlineStr">
         <is>
-          <t>Colonna65</t>
+          <t>WAR-30 (1)</t>
         </is>
       </c>
       <c r="BN1" s="109" t="inlineStr">
         <is>
-          <t>Colonna66</t>
+          <t>WAR-30 (2)</t>
         </is>
       </c>
       <c r="BO1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BL2)</f>
+        <f>SUM(G2:BN2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BL2),1)</f>
+        <f>ROUND(AVERAGE(G2:BN2),1)</f>
         <v/>
       </c>
     </row>
@@ -12991,11 +12991,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BL3)</f>
+        <f>SUM(G3:BN3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BL3),1)</f>
+        <f>ROUND(AVERAGE(G3:BN3),1)</f>
         <v/>
       </c>
       <c r="AO3" t="n">
@@ -13039,11 +13039,11 @@
         <v>20</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BL4)</f>
+        <f>SUM(G4:BN4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BL4),1)</f>
+        <f>ROUND(AVERAGE(G4:BN4),1)</f>
         <v/>
       </c>
       <c r="G4" s="79" t="n">
@@ -13211,11 +13211,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BL5)</f>
+        <f>SUM(G5:BN5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BL5),1)</f>
+        <f>ROUND(AVERAGE(G5:BN5),1)</f>
         <v/>
       </c>
       <c r="K5" s="79" t="n">
@@ -13289,11 +13289,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BL6)</f>
+        <f>SUM(G6:BN6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BL6),1)</f>
+        <f>ROUND(AVERAGE(G6:BN6),1)</f>
         <v/>
       </c>
       <c r="BA6" t="n">
@@ -13312,20 +13312,20 @@
         </is>
       </c>
       <c r="B7" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C7" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BL7)</f>
+        <f>SUM(G7:BN7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BL7),1)</f>
+        <f>ROUND(AVERAGE(G7:BN7),1)</f>
         <v/>
       </c>
       <c r="G7" s="79" t="n">
@@ -13428,6 +13428,16 @@
         </is>
       </c>
       <c r="BH7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BN7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13449,11 +13459,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BL8)</f>
+        <f>SUM(G8:BN8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BL8),1)</f>
+        <f>ROUND(AVERAGE(G8:BN8),1)</f>
         <v/>
       </c>
     </row>
@@ -13473,11 +13483,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BL9)</f>
+        <f>SUM(G9:BN9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BL9),1)</f>
+        <f>ROUND(AVERAGE(G9:BN9),1)</f>
         <v/>
       </c>
       <c r="I9" s="79" t="n">
@@ -13547,11 +13557,11 @@
         <v>8</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BL10)</f>
+        <f>SUM(G10:BN10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BL10),1)</f>
+        <f>ROUND(AVERAGE(G10:BN10),1)</f>
         <v/>
       </c>
       <c r="Q10" s="79" t="n">
@@ -13620,20 +13630,20 @@
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BL11)</f>
+        <f>SUM(G11:BN11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BL11),1)</f>
+        <f>ROUND(AVERAGE(G11:BN11),1)</f>
         <v/>
       </c>
       <c r="G11" s="79" t="n">
@@ -13727,6 +13737,16 @@
       </c>
       <c r="BL11" t="n">
         <v>3</v>
+      </c>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -13745,11 +13765,11 @@
         <v>19</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BL12)</f>
+        <f>SUM(G12:BN12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BL12),1)</f>
+        <f>ROUND(AVERAGE(G12:BN12),1)</f>
         <v/>
       </c>
       <c r="I12" s="79" t="n">
@@ -13893,11 +13913,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BL13)</f>
+        <f>SUM(G13:BN13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BL13),1)</f>
+        <f>ROUND(AVERAGE(G13:BN13),1)</f>
         <v/>
       </c>
       <c r="S13" s="79" t="n">
@@ -13981,11 +14001,11 @@
         <v>8</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BL14)</f>
+        <f>SUM(G14:BN14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BL14),1)</f>
+        <f>ROUND(AVERAGE(G14:BN14),1)</f>
         <v/>
       </c>
       <c r="G14" s="79" t="n">
@@ -14055,11 +14075,11 @@
         <v>3</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BL15)</f>
+        <f>SUM(G15:BN15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BL15),1)</f>
+        <f>ROUND(AVERAGE(G15:BN15),1)</f>
         <v/>
       </c>
       <c r="AE15" s="79" t="n">
@@ -14097,11 +14117,11 @@
         <v>13</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BL16)</f>
+        <f>SUM(G16:BN16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BL16),1)</f>
+        <f>ROUND(AVERAGE(G16:BN16),1)</f>
         <v/>
       </c>
       <c r="I16" s="79" t="n">
@@ -14203,11 +14223,11 @@
         <v>15</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BL17)</f>
+        <f>SUM(G17:BN17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BL17),1)</f>
+        <f>ROUND(AVERAGE(G17:BN17),1)</f>
         <v/>
       </c>
       <c r="G17" s="79" t="n">
@@ -14334,14 +14354,14 @@
         <v>1</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BL18)</f>
+        <f>SUM(G18:BN18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BL18),1)</f>
+        <f>ROUND(AVERAGE(G18:BN18),1)</f>
         <v/>
       </c>
       <c r="G18" s="79" t="n">
@@ -14424,6 +14444,12 @@
         <v>3</v>
       </c>
       <c r="BL18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14443,11 +14469,11 @@
         <v>9</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BL19)</f>
+        <f>SUM(G19:BN19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BL19),1)</f>
+        <f>ROUND(AVERAGE(G19:BN19),1)</f>
         <v/>
       </c>
       <c r="I19" s="79" t="n">
@@ -14531,11 +14557,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BL20)</f>
+        <f>SUM(G20:BN20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BL20),1)</f>
+        <f>ROUND(AVERAGE(G20:BN20),1)</f>
         <v/>
       </c>
       <c r="Y20" s="79" t="n">
@@ -14572,14 +14598,14 @@
         <v>3</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BL21)</f>
+        <f>SUM(G21:BN21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BL21),1)</f>
+        <f>ROUND(AVERAGE(G21:BN21),1)</f>
         <v/>
       </c>
       <c r="S21" s="79" t="n">
@@ -14655,6 +14681,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BM21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -14673,11 +14705,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BL22)</f>
+        <f>SUM(G22:BN22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BL22),1)</f>
+        <f>ROUND(AVERAGE(G22:BN22),1)</f>
         <v/>
       </c>
       <c r="I22" s="79" t="inlineStr">
@@ -14771,11 +14803,11 @@
         <v>8</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BL23)</f>
+        <f>SUM(G23:BN23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BL23),1)</f>
+        <f>ROUND(AVERAGE(G23:BN23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
@@ -14844,14 +14876,14 @@
         <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BL24)</f>
+        <f>SUM(G24:BN24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BL24),1)</f>
+        <f>ROUND(AVERAGE(G24:BN24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -14935,6 +14967,12 @@
       </c>
       <c r="AT24" t="n">
         <v>3</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -14953,11 +14991,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BL25)</f>
+        <f>SUM(G25:BN25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BL25),1)</f>
+        <f>ROUND(AVERAGE(G25:BN25),1)</f>
         <v/>
       </c>
       <c r="AS25" t="n">
@@ -14980,14 +15018,14 @@
         <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BL26)</f>
+        <f>SUM(G26:BN26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BL26),1)</f>
+        <f>ROUND(AVERAGE(G26:BN26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -15117,6 +15155,12 @@
       </c>
       <c r="BL26" t="n">
         <v>2</v>
+      </c>
+      <c r="BM26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN26" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -15135,11 +15179,11 @@
         <v>14</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BL27)</f>
+        <f>SUM(G27:BN27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BL27),1)</f>
+        <f>ROUND(AVERAGE(G27:BN27),1)</f>
         <v/>
       </c>
       <c r="U27" s="79" t="n">
@@ -15253,11 +15297,11 @@
         <v>5</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BL28)</f>
+        <f>SUM(G28:BN28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BL28),1)</f>
+        <f>ROUND(AVERAGE(G28:BN28),1)</f>
         <v/>
       </c>
       <c r="AM28" t="n">
@@ -15309,11 +15353,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BL29)</f>
+        <f>SUM(G29:BN29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BL29),1)</f>
+        <f>ROUND(AVERAGE(G29:BN29),1)</f>
         <v/>
       </c>
       <c r="AM29" t="n">
@@ -15365,11 +15409,11 @@
         <v>9</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BL30)</f>
+        <f>SUM(G30:BN30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BL30),1)</f>
+        <f>ROUND(AVERAGE(G30:BN30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15443,11 +15487,11 @@
         <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BL31)</f>
+        <f>SUM(G31:BN31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BL31),1)</f>
+        <f>ROUND(AVERAGE(G31:BN31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
@@ -15495,11 +15539,11 @@
         <v>9</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BL32)</f>
+        <f>SUM(G32:BN32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BL32),1)</f>
+        <f>ROUND(AVERAGE(G32:BN32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
@@ -15573,11 +15617,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BL33)</f>
+        <f>SUM(G33:BN33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BL33),1)</f>
+        <f>ROUND(AVERAGE(G33:BN33),1)</f>
         <v/>
       </c>
       <c r="BE33" t="n">
@@ -15603,11 +15647,11 @@
         <v>0</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BL34)</f>
+        <f>SUM(G34:BN34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BL34),1)</f>
+        <f>ROUND(AVERAGE(G34:BN34),1)</f>
         <v/>
       </c>
     </row>
@@ -15627,11 +15671,11 @@
         <v>1</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BL35)</f>
+        <f>SUM(G35:BN35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BL35),1)</f>
+        <f>ROUND(AVERAGE(G35:BN35),1)</f>
         <v/>
       </c>
       <c r="BA35" t="n">
@@ -15654,14 +15698,14 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BL36)</f>
+        <f>SUM(G36:BN36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BL36),1)</f>
+        <f>ROUND(AVERAGE(G36:BN36),1)</f>
         <v/>
       </c>
       <c r="BA36" t="n">
@@ -15691,6 +15735,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BM36" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN36" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -15709,11 +15759,11 @@
         <v>2</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BL37)</f>
+        <f>SUM(G37:BN37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BL37),1)</f>
+        <f>ROUND(AVERAGE(G37:BN37),1)</f>
         <v/>
       </c>
       <c r="BE37" t="n">
@@ -15747,11 +15797,11 @@
         <v>5</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BL38)</f>
+        <f>SUM(G38:BN38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BL38),1)</f>
+        <f>ROUND(AVERAGE(G38:BN38),1)</f>
         <v/>
       </c>
       <c r="BC38" t="n">
@@ -15794,20 +15844,20 @@
         </is>
       </c>
       <c r="B39" s="79" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="C39" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="79" t="n">
-        <v>4</v>
-      </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BL39)</f>
+        <f>SUM(G39:BN39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BL39),1)</f>
+        <f>ROUND(AVERAGE(G39:BN39),1)</f>
         <v/>
       </c>
       <c r="BC39" t="inlineStr">
@@ -15840,6 +15890,14 @@
         <v>2</v>
       </c>
       <c r="BL39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BM39" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN39" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15852,20 +15910,20 @@
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BL40)</f>
+        <f>SUM(G40:BN40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BL40),1)</f>
+        <f>ROUND(AVERAGE(G40:BN40),1)</f>
         <v/>
       </c>
       <c r="BE40" t="n">
@@ -15888,6 +15946,16 @@
         <v>0</v>
       </c>
       <c r="BL40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BM40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BN40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15909,11 +15977,11 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BL41)</f>
+        <f>SUM(G41:BN41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BL41),1)</f>
+        <f>ROUND(AVERAGE(G41:BN41),1)</f>
         <v/>
       </c>
     </row>
@@ -15924,20 +15992,20 @@
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C42" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BL42)</f>
+        <f>SUM(G42:BN42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BL42),1)</f>
+        <f>ROUND(AVERAGE(G42:BN42),1)</f>
         <v/>
       </c>
       <c r="BC42" t="inlineStr">
@@ -15946,6 +16014,14 @@
         </is>
       </c>
       <c r="BD42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BM42" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN42" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15967,11 +16043,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BL43)</f>
+        <f>SUM(G43:BN43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BL43),1)</f>
+        <f>ROUND(AVERAGE(G43:BN43),1)</f>
         <v/>
       </c>
     </row>
@@ -15991,11 +16067,11 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BL44)</f>
+        <f>SUM(G44:BN44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BL44),1)</f>
+        <f>ROUND(AVERAGE(G44:BN44),1)</f>
         <v/>
       </c>
     </row>
@@ -16015,11 +16091,11 @@
         <v>2</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BL45)</f>
+        <f>SUM(G45:BN45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BL45),1)</f>
+        <f>ROUND(AVERAGE(G45:BN45),1)</f>
         <v/>
       </c>
       <c r="BI45" t="n">
@@ -16051,11 +16127,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BL46)</f>
+        <f>SUM(G46:BN46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BL46),1)</f>
+        <f>ROUND(AVERAGE(G46:BN46),1)</f>
         <v/>
       </c>
     </row>
@@ -16075,18 +16151,18 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BL47)</f>
+        <f>SUM(G47:BN47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BL47),1)</f>
+        <f>ROUND(AVERAGE(G47:BN47),1)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>perte</t>
+          <t>EMANUELE</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -16099,86 +16175,86 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BL48)</f>
+        <f>SUM(G48:BN48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BL48),1)</f>
+        <f>ROUND(AVERAGE(G48:BN48),1)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>EMANUELE</t>
+          <t>micky</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C49" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D49" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BL49)</f>
+        <f>SUM(G49:BN49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BL49),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G49:BN49),1)</f>
+        <v/>
+      </c>
+      <c r="BI49" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BJ49" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK49" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BL49" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="79" t="inlineStr">
         <is>
-          <t>micky</t>
+          <t>salvo24</t>
         </is>
       </c>
       <c r="B50" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C50" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D50" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E50" s="68">
-        <f>SUM(G50:BL50)</f>
+        <f>SUM(G50:BN50)</f>
         <v/>
       </c>
       <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BL50),1)</f>
-        <v/>
-      </c>
-      <c r="BI50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BJ50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BK50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BL50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G50:BN50),1)</f>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="79" t="inlineStr">
         <is>
-          <t>TaifTuff</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B51" s="79" t="n">
@@ -16191,11 +16267,11 @@
         <v>0</v>
       </c>
       <c r="E51" s="68">
-        <f>SUM(G51:BL51)</f>
+        <f>SUM(G51:BN51)</f>
         <v/>
       </c>
       <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:BL51),1)</f>
+        <f>ROUND(AVERAGE(G51:BN51),1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-26
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12847,12 +12847,12 @@
       </c>
       <c r="BO1" s="109" t="inlineStr">
         <is>
-          <t>Colonna67</t>
+          <t>WAR-31 (1)</t>
         </is>
       </c>
       <c r="BP1" s="109" t="inlineStr">
         <is>
-          <t>Colonna68</t>
+          <t>WAR-31 (2)</t>
         </is>
       </c>
       <c r="BQ1" s="109" t="inlineStr">
@@ -12967,11 +12967,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BN2)</f>
+        <f>SUM(G2:BP2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BN2),1)</f>
+        <f>ROUND(AVERAGE(G2:BP2),1)</f>
         <v/>
       </c>
     </row>
@@ -12991,11 +12991,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BN3)</f>
+        <f>SUM(G3:BP3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BN3),1)</f>
+        <f>ROUND(AVERAGE(G3:BP3),1)</f>
         <v/>
       </c>
       <c r="AO3" t="n">
@@ -13036,14 +13036,14 @@
         <v>5</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BN4)</f>
+        <f>SUM(G4:BP4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BN4),1)</f>
+        <f>ROUND(AVERAGE(G4:BP4),1)</f>
         <v/>
       </c>
       <c r="G4" s="79" t="n">
@@ -13192,6 +13192,12 @@
         <v>3</v>
       </c>
       <c r="BL4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13211,11 +13217,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BN5)</f>
+        <f>SUM(G5:BP5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BN5),1)</f>
+        <f>ROUND(AVERAGE(G5:BP5),1)</f>
         <v/>
       </c>
       <c r="K5" s="79" t="n">
@@ -13289,11 +13295,11 @@
         <v>1</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BN6)</f>
+        <f>SUM(G6:BP6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BN6),1)</f>
+        <f>ROUND(AVERAGE(G6:BP6),1)</f>
         <v/>
       </c>
       <c r="BA6" t="n">
@@ -13321,11 +13327,11 @@
         <v>17</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BN7)</f>
+        <f>SUM(G7:BP7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BN7),1)</f>
+        <f>ROUND(AVERAGE(G7:BP7),1)</f>
         <v/>
       </c>
       <c r="G7" s="79" t="n">
@@ -13459,11 +13465,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BN8)</f>
+        <f>SUM(G8:BP8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BN8),1)</f>
+        <f>ROUND(AVERAGE(G8:BP8),1)</f>
         <v/>
       </c>
     </row>
@@ -13483,11 +13489,11 @@
         <v>6</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BN9)</f>
+        <f>SUM(G9:BP9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BN9),1)</f>
+        <f>ROUND(AVERAGE(G9:BP9),1)</f>
         <v/>
       </c>
       <c r="I9" s="79" t="n">
@@ -13548,20 +13554,20 @@
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BN10)</f>
+        <f>SUM(G10:BP10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BN10),1)</f>
+        <f>ROUND(AVERAGE(G10:BP10),1)</f>
         <v/>
       </c>
       <c r="Q10" s="79" t="n">
@@ -13618,6 +13624,14 @@
         </is>
       </c>
       <c r="BL10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13639,11 +13653,11 @@
         <v>16</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BN11)</f>
+        <f>SUM(G11:BP11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BN11),1)</f>
+        <f>ROUND(AVERAGE(G11:BP11),1)</f>
         <v/>
       </c>
       <c r="G11" s="79" t="n">
@@ -13762,14 +13776,14 @@
         <v>1</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BN12)</f>
+        <f>SUM(G12:BP12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BN12),1)</f>
+        <f>ROUND(AVERAGE(G12:BP12),1)</f>
         <v/>
       </c>
       <c r="I12" s="79" t="n">
@@ -13895,6 +13909,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BO12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -13913,11 +13933,11 @@
         <v>10</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BN13)</f>
+        <f>SUM(G13:BP13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BN13),1)</f>
+        <f>ROUND(AVERAGE(G13:BP13),1)</f>
         <v/>
       </c>
       <c r="S13" s="79" t="n">
@@ -14001,11 +14021,11 @@
         <v>8</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BN14)</f>
+        <f>SUM(G14:BP14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BN14),1)</f>
+        <f>ROUND(AVERAGE(G14:BP14),1)</f>
         <v/>
       </c>
       <c r="G14" s="79" t="n">
@@ -14072,14 +14092,14 @@
         <v>0</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BN15)</f>
+        <f>SUM(G15:BP15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BN15),1)</f>
+        <f>ROUND(AVERAGE(G15:BP15),1)</f>
         <v/>
       </c>
       <c r="AE15" s="79" t="n">
@@ -14098,6 +14118,12 @@
         <v>3</v>
       </c>
       <c r="BJ15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP15" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14114,14 +14140,14 @@
         <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BN16)</f>
+        <f>SUM(G16:BP16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BN16),1)</f>
+        <f>ROUND(AVERAGE(G16:BP16),1)</f>
         <v/>
       </c>
       <c r="I16" s="79" t="n">
@@ -14205,6 +14231,12 @@
       </c>
       <c r="BL16" t="n">
         <v>2</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -14220,14 +14252,14 @@
         <v>1</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BN17)</f>
+        <f>SUM(G17:BP17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BN17),1)</f>
+        <f>ROUND(AVERAGE(G17:BP17),1)</f>
         <v/>
       </c>
       <c r="G17" s="79" t="n">
@@ -14339,6 +14371,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BO17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -14357,11 +14395,11 @@
         <v>14</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BN18)</f>
+        <f>SUM(G18:BP18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BN18),1)</f>
+        <f>ROUND(AVERAGE(G18:BP18),1)</f>
         <v/>
       </c>
       <c r="G18" s="79" t="n">
@@ -14469,11 +14507,11 @@
         <v>9</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BN19)</f>
+        <f>SUM(G19:BP19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BN19),1)</f>
+        <f>ROUND(AVERAGE(G19:BP19),1)</f>
         <v/>
       </c>
       <c r="I19" s="79" t="n">
@@ -14557,11 +14595,11 @@
         <v>3</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BN20)</f>
+        <f>SUM(G20:BP20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BN20),1)</f>
+        <f>ROUND(AVERAGE(G20:BP20),1)</f>
         <v/>
       </c>
       <c r="Y20" s="79" t="n">
@@ -14598,14 +14636,14 @@
         <v>3</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BN21)</f>
+        <f>SUM(G21:BP21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BN21),1)</f>
+        <f>ROUND(AVERAGE(G21:BP21),1)</f>
         <v/>
       </c>
       <c r="S21" s="79" t="n">
@@ -14687,6 +14725,12 @@
       </c>
       <c r="BN21" t="n">
         <v>3</v>
+      </c>
+      <c r="BO21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -14702,14 +14746,14 @@
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BN22)</f>
+        <f>SUM(G22:BP22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BN22),1)</f>
+        <f>ROUND(AVERAGE(G22:BP22),1)</f>
         <v/>
       </c>
       <c r="I22" s="79" t="inlineStr">
@@ -14785,6 +14829,12 @@
       </c>
       <c r="AN22" t="n">
         <v>2</v>
+      </c>
+      <c r="BO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP22" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -14803,11 +14853,11 @@
         <v>8</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BN23)</f>
+        <f>SUM(G23:BP23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BN23),1)</f>
+        <f>ROUND(AVERAGE(G23:BP23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
@@ -14876,14 +14926,14 @@
         <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BN24)</f>
+        <f>SUM(G24:BP24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BN24),1)</f>
+        <f>ROUND(AVERAGE(G24:BP24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -14972,6 +15022,12 @@
         <v>3</v>
       </c>
       <c r="BN24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14991,11 +15047,11 @@
         <v>1</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BN25)</f>
+        <f>SUM(G25:BP25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BN25),1)</f>
+        <f>ROUND(AVERAGE(G25:BP25),1)</f>
         <v/>
       </c>
       <c r="AS25" t="n">
@@ -15018,14 +15074,14 @@
         <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BN26)</f>
+        <f>SUM(G26:BP26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BN26),1)</f>
+        <f>ROUND(AVERAGE(G26:BP26),1)</f>
         <v/>
       </c>
       <c r="G26" s="79" t="n">
@@ -15160,6 +15216,12 @@
         <v>3</v>
       </c>
       <c r="BN26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP26" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15179,11 +15241,11 @@
         <v>14</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BN27)</f>
+        <f>SUM(G27:BP27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BN27),1)</f>
+        <f>ROUND(AVERAGE(G27:BP27),1)</f>
         <v/>
       </c>
       <c r="U27" s="79" t="n">
@@ -15297,11 +15359,11 @@
         <v>5</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BN28)</f>
+        <f>SUM(G28:BP28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BN28),1)</f>
+        <f>ROUND(AVERAGE(G28:BP28),1)</f>
         <v/>
       </c>
       <c r="AM28" t="n">
@@ -15353,11 +15415,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BN29)</f>
+        <f>SUM(G29:BP29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BN29),1)</f>
+        <f>ROUND(AVERAGE(G29:BP29),1)</f>
         <v/>
       </c>
       <c r="AM29" t="n">
@@ -15409,11 +15471,11 @@
         <v>9</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BN30)</f>
+        <f>SUM(G30:BP30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BN30),1)</f>
+        <f>ROUND(AVERAGE(G30:BP30),1)</f>
         <v/>
       </c>
       <c r="AM30" t="n">
@@ -15487,11 +15549,11 @@
         <v>4</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BN31)</f>
+        <f>SUM(G31:BP31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BN31),1)</f>
+        <f>ROUND(AVERAGE(G31:BP31),1)</f>
         <v/>
       </c>
       <c r="AM31" t="n">
@@ -15539,11 +15601,11 @@
         <v>9</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BN32)</f>
+        <f>SUM(G32:BP32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BN32),1)</f>
+        <f>ROUND(AVERAGE(G32:BP32),1)</f>
         <v/>
       </c>
       <c r="AM32" t="n">
@@ -15617,11 +15679,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BN33)</f>
+        <f>SUM(G33:BP33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BN33),1)</f>
+        <f>ROUND(AVERAGE(G33:BP33),1)</f>
         <v/>
       </c>
       <c r="BE33" t="n">
@@ -15647,11 +15709,11 @@
         <v>0</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BN34)</f>
+        <f>SUM(G34:BP34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BN34),1)</f>
+        <f>ROUND(AVERAGE(G34:BP34),1)</f>
         <v/>
       </c>
     </row>
@@ -15671,11 +15733,11 @@
         <v>1</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BN35)</f>
+        <f>SUM(G35:BP35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BN35),1)</f>
+        <f>ROUND(AVERAGE(G35:BP35),1)</f>
         <v/>
       </c>
       <c r="BA35" t="n">
@@ -15698,14 +15760,14 @@
         <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BN36)</f>
+        <f>SUM(G36:BP36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BN36),1)</f>
+        <f>ROUND(AVERAGE(G36:BP36),1)</f>
         <v/>
       </c>
       <c r="BA36" t="n">
@@ -15741,6 +15803,12 @@
       </c>
       <c r="BN36" t="n">
         <v>2</v>
+      </c>
+      <c r="BO36" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP36" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -15759,11 +15827,11 @@
         <v>2</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BN37)</f>
+        <f>SUM(G37:BP37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BN37),1)</f>
+        <f>ROUND(AVERAGE(G37:BP37),1)</f>
         <v/>
       </c>
       <c r="BE37" t="n">
@@ -15797,11 +15865,11 @@
         <v>5</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BN38)</f>
+        <f>SUM(G38:BP38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BN38),1)</f>
+        <f>ROUND(AVERAGE(G38:BP38),1)</f>
         <v/>
       </c>
       <c r="BC38" t="n">
@@ -15844,20 +15912,20 @@
         </is>
       </c>
       <c r="B39" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="79" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="79" t="n">
-        <v>5</v>
-      </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BN39)</f>
+        <f>SUM(G39:BP39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BN39),1)</f>
+        <f>ROUND(AVERAGE(G39:BP39),1)</f>
         <v/>
       </c>
       <c r="BC39" t="inlineStr">
@@ -15898,6 +15966,14 @@
         <v>3</v>
       </c>
       <c r="BN39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO39" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP39" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15910,20 +15986,20 @@
         </is>
       </c>
       <c r="B40" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="C40" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="79" t="n">
-        <v>4</v>
-      </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BN40)</f>
+        <f>SUM(G40:BP40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BN40),1)</f>
+        <f>ROUND(AVERAGE(G40:BP40),1)</f>
         <v/>
       </c>
       <c r="BE40" t="n">
@@ -15956,6 +16032,16 @@
         </is>
       </c>
       <c r="BN40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BP40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15977,11 +16063,11 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BN41)</f>
+        <f>SUM(G41:BP41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BN41),1)</f>
+        <f>ROUND(AVERAGE(G41:BP41),1)</f>
         <v/>
       </c>
     </row>
@@ -16001,11 +16087,11 @@
         <v>2</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BN42)</f>
+        <f>SUM(G42:BP42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BN42),1)</f>
+        <f>ROUND(AVERAGE(G42:BP42),1)</f>
         <v/>
       </c>
       <c r="BC42" t="inlineStr">
@@ -16043,11 +16129,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BN43)</f>
+        <f>SUM(G43:BP43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BN43),1)</f>
+        <f>ROUND(AVERAGE(G43:BP43),1)</f>
         <v/>
       </c>
     </row>
@@ -16067,11 +16153,11 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BN44)</f>
+        <f>SUM(G44:BP44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BN44),1)</f>
+        <f>ROUND(AVERAGE(G44:BP44),1)</f>
         <v/>
       </c>
     </row>
@@ -16088,14 +16174,14 @@
         <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BN45)</f>
+        <f>SUM(G45:BP45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BN45),1)</f>
+        <f>ROUND(AVERAGE(G45:BP45),1)</f>
         <v/>
       </c>
       <c r="BI45" t="n">
@@ -16108,6 +16194,12 @@
         <v>2</v>
       </c>
       <c r="BL45" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO45" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP45" t="n">
         <v>3</v>
       </c>
     </row>
@@ -16127,11 +16219,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BN46)</f>
+        <f>SUM(G46:BP46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BN46),1)</f>
+        <f>ROUND(AVERAGE(G46:BP46),1)</f>
         <v/>
       </c>
     </row>
@@ -16151,11 +16243,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BN47)</f>
+        <f>SUM(G47:BP47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BN47),1)</f>
+        <f>ROUND(AVERAGE(G47:BP47),1)</f>
         <v/>
       </c>
     </row>
@@ -16175,11 +16267,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BN48)</f>
+        <f>SUM(G48:BP48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BN48),1)</f>
+        <f>ROUND(AVERAGE(G48:BP48),1)</f>
         <v/>
       </c>
     </row>
@@ -16199,11 +16291,11 @@
         <v>2</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BN49)</f>
+        <f>SUM(G49:BP49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BN49),1)</f>
+        <f>ROUND(AVERAGE(G49:BP49),1)</f>
         <v/>
       </c>
       <c r="BI49" t="inlineStr">
@@ -16243,11 +16335,11 @@
         <v>0</v>
       </c>
       <c r="E50" s="68">
-        <f>SUM(G50:BN50)</f>
+        <f>SUM(G50:BP50)</f>
         <v/>
       </c>
       <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BN50),1)</f>
+        <f>ROUND(AVERAGE(G50:BP50),1)</f>
         <v/>
       </c>
     </row>
@@ -16264,15 +16356,21 @@
         <v>0</v>
       </c>
       <c r="D51" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" s="68">
-        <f>SUM(G51:BN51)</f>
+        <f>SUM(G51:BP51)</f>
         <v/>
       </c>
       <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:BN51),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G51:BP51),1)</f>
+        <v/>
+      </c>
+      <c r="BO51" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP51" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update WAR data - 2026-03-31
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12475,7 +12475,6 @@
         </is>
       </c>
       <c r="S29" s="78" t="n"/>
-      <c r="X29" t="inlineStr"/>
       <c r="AD29" s="79" t="inlineStr">
         <is>
           <t>LucFir3</t>
@@ -12690,7 +12689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI50"/>
+  <dimension ref="A1:CI51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13101,12 +13100,12 @@
       </c>
       <c r="BS1" s="109" t="inlineStr">
         <is>
-          <t>Colonna71</t>
+          <t>WAR-33 (1)</t>
         </is>
       </c>
       <c r="BT1" s="109" t="inlineStr">
         <is>
-          <t>Colonna72</t>
+          <t>WAR-33 (2)</t>
         </is>
       </c>
       <c r="BU1" s="109" t="inlineStr">
@@ -13201,11 +13200,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="125">
-        <f>SUM(G2:BR2)</f>
+        <f>SUM(G2:BT2)</f>
         <v/>
       </c>
       <c r="F2" s="125">
-        <f>ROUND(AVERAGE(G2:BR2),1)</f>
+        <f>ROUND(AVERAGE(G2:BT2),1)</f>
         <v/>
       </c>
     </row>
@@ -13225,11 +13224,11 @@
         <v>0</v>
       </c>
       <c r="E3" s="125">
-        <f>SUM(G3:BR3)</f>
+        <f>SUM(G3:BT3)</f>
         <v/>
       </c>
       <c r="F3" s="125">
-        <f>ROUND(AVERAGE(G3:BR3),1)</f>
+        <f>ROUND(AVERAGE(G3:BT3),1)</f>
         <v/>
       </c>
       <c r="AO3" s="125" t="n"/>
@@ -13251,11 +13250,11 @@
         <v>3</v>
       </c>
       <c r="E4" s="125">
-        <f>SUM(G4:BR4)</f>
+        <f>SUM(G4:BT4)</f>
         <v/>
       </c>
       <c r="F4" s="125">
-        <f>ROUND(AVERAGE(G4:BR4),1)</f>
+        <f>ROUND(AVERAGE(G4:BT4),1)</f>
         <v/>
       </c>
       <c r="AI4" s="125" t="n"/>
@@ -13304,14 +13303,14 @@
         <v>0</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="125">
-        <f>SUM(G5:BR5)</f>
+        <f>SUM(G5:BT5)</f>
         <v/>
       </c>
       <c r="F5" s="125">
-        <f>ROUND(AVERAGE(G5:BR5),1)</f>
+        <f>ROUND(AVERAGE(G5:BT5),1)</f>
         <v/>
       </c>
       <c r="AM5" t="n">
@@ -13372,6 +13371,12 @@
         <v>3</v>
       </c>
       <c r="BR5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13391,11 +13396,11 @@
         <v>4</v>
       </c>
       <c r="E6" s="125">
-        <f>SUM(G6:BR6)</f>
+        <f>SUM(G6:BT6)</f>
         <v/>
       </c>
       <c r="F6" s="125">
-        <f>ROUND(AVERAGE(G6:BR6),1)</f>
+        <f>ROUND(AVERAGE(G6:BT6),1)</f>
         <v/>
       </c>
       <c r="BI6" t="n">
@@ -13439,11 +13444,11 @@
         <v>2</v>
       </c>
       <c r="E7" s="125">
-        <f>SUM(G7:BR7)</f>
+        <f>SUM(G7:BT7)</f>
         <v/>
       </c>
       <c r="F7" s="125">
-        <f>ROUND(AVERAGE(G7:BR7),1)</f>
+        <f>ROUND(AVERAGE(G7:BT7),1)</f>
         <v/>
       </c>
       <c r="AM7" s="125" t="n"/>
@@ -13481,11 +13486,11 @@
         <v>22</v>
       </c>
       <c r="E8" s="125">
-        <f>SUM(G8:BR8)</f>
+        <f>SUM(G8:BT8)</f>
         <v/>
       </c>
       <c r="F8" s="125">
-        <f>ROUND(AVERAGE(G8:BR8),1)</f>
+        <f>ROUND(AVERAGE(G8:BT8),1)</f>
         <v/>
       </c>
       <c r="G8" s="79" t="n">
@@ -13667,11 +13672,11 @@
         <v>9</v>
       </c>
       <c r="E9" s="125">
-        <f>SUM(G9:BR9)</f>
+        <f>SUM(G9:BT9)</f>
         <v/>
       </c>
       <c r="F9" s="125">
-        <f>ROUND(AVERAGE(G9:BR9),1)</f>
+        <f>ROUND(AVERAGE(G9:BT9),1)</f>
         <v/>
       </c>
       <c r="K9" s="79" t="n">
@@ -13749,11 +13754,11 @@
         <v>1</v>
       </c>
       <c r="E10" s="125">
-        <f>SUM(G10:BR10)</f>
+        <f>SUM(G10:BT10)</f>
         <v/>
       </c>
       <c r="F10" s="125">
-        <f>ROUND(AVERAGE(G10:BR10),1)</f>
+        <f>ROUND(AVERAGE(G10:BT10),1)</f>
         <v/>
       </c>
       <c r="AS10" s="125" t="n"/>
@@ -13780,14 +13785,14 @@
         <v>0</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E11" s="125">
-        <f>SUM(G11:BR11)</f>
+        <f>SUM(G11:BT11)</f>
         <v/>
       </c>
       <c r="F11" s="125">
-        <f>ROUND(AVERAGE(G11:BR11),1)</f>
+        <f>ROUND(AVERAGE(G11:BT11),1)</f>
         <v/>
       </c>
       <c r="AM11" t="n">
@@ -13848,6 +13853,12 @@
         <v>3</v>
       </c>
       <c r="BR11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13867,11 +13878,11 @@
         <v>18</v>
       </c>
       <c r="E12" s="125">
-        <f>SUM(G12:BR12)</f>
+        <f>SUM(G12:BT12)</f>
         <v/>
       </c>
       <c r="F12" s="125">
-        <f>ROUND(AVERAGE(G12:BR12),1)</f>
+        <f>ROUND(AVERAGE(G12:BT12),1)</f>
         <v/>
       </c>
       <c r="G12" s="79" t="n">
@@ -14019,11 +14030,11 @@
         <v>1</v>
       </c>
       <c r="E13" s="125">
-        <f>SUM(G13:BR13)</f>
+        <f>SUM(G13:BT13)</f>
         <v/>
       </c>
       <c r="F13" s="125">
-        <f>ROUND(AVERAGE(G13:BR13),1)</f>
+        <f>ROUND(AVERAGE(G13:BT13),1)</f>
         <v/>
       </c>
       <c r="AI13" s="125" t="n"/>
@@ -14048,20 +14059,20 @@
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="125" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="125">
-        <f>SUM(G14:BR14)</f>
+        <f>SUM(G14:BT14)</f>
         <v/>
       </c>
       <c r="F14" s="125">
-        <f>ROUND(AVERAGE(G14:BR14),1)</f>
+        <f>ROUND(AVERAGE(G14:BT14),1)</f>
         <v/>
       </c>
       <c r="BO14" t="n">
@@ -14074,6 +14085,14 @@
         <v>1</v>
       </c>
       <c r="BR14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -14095,11 +14114,11 @@
         <v>0</v>
       </c>
       <c r="E15" s="125">
-        <f>SUM(G15:BR15)</f>
+        <f>SUM(G15:BT15)</f>
         <v/>
       </c>
       <c r="F15" s="125">
-        <f>ROUND(AVERAGE(G15:BR15),1)</f>
+        <f>ROUND(AVERAGE(G15:BT15),1)</f>
         <v/>
       </c>
     </row>
@@ -14119,11 +14138,11 @@
         <v>6</v>
       </c>
       <c r="E16" s="125">
-        <f>SUM(G16:BR16)</f>
+        <f>SUM(G16:BT16)</f>
         <v/>
       </c>
       <c r="F16" s="125">
-        <f>ROUND(AVERAGE(G16:BR16),1)</f>
+        <f>ROUND(AVERAGE(G16:BT16),1)</f>
         <v/>
       </c>
       <c r="I16" s="79" t="n">
@@ -14197,11 +14216,11 @@
         <v>10</v>
       </c>
       <c r="E17" s="125">
-        <f>SUM(G17:BR17)</f>
+        <f>SUM(G17:BT17)</f>
         <v/>
       </c>
       <c r="F17" s="125">
-        <f>ROUND(AVERAGE(G17:BR17),1)</f>
+        <f>ROUND(AVERAGE(G17:BT17),1)</f>
         <v/>
       </c>
       <c r="Q17" s="79" t="n">
@@ -14297,11 +14316,11 @@
         <v>1</v>
       </c>
       <c r="E18" s="125">
-        <f>SUM(G18:BR18)</f>
+        <f>SUM(G18:BT18)</f>
         <v/>
       </c>
       <c r="F18" s="125">
-        <f>ROUND(AVERAGE(G18:BR18),1)</f>
+        <f>ROUND(AVERAGE(G18:BT18),1)</f>
         <v/>
       </c>
       <c r="BA18" t="n">
@@ -14327,11 +14346,11 @@
         <v>16</v>
       </c>
       <c r="E19" s="125">
-        <f>SUM(G19:BR19)</f>
+        <f>SUM(G19:BT19)</f>
         <v/>
       </c>
       <c r="F19" s="125">
-        <f>ROUND(AVERAGE(G19:BR19),1)</f>
+        <f>ROUND(AVERAGE(G19:BT19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14457,11 +14476,11 @@
         <v>20</v>
       </c>
       <c r="E20" s="125">
-        <f>SUM(G20:BR20)</f>
+        <f>SUM(G20:BT20)</f>
         <v/>
       </c>
       <c r="F20" s="125">
-        <f>ROUND(AVERAGE(G20:BR20),1)</f>
+        <f>ROUND(AVERAGE(G20:BT20),1)</f>
         <v/>
       </c>
       <c r="I20" s="79" t="n">
@@ -14608,14 +14627,14 @@
         <v>1</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" s="125">
-        <f>SUM(G21:BR21)</f>
+        <f>SUM(G21:BT21)</f>
         <v/>
       </c>
       <c r="F21" s="125">
-        <f>ROUND(AVERAGE(G21:BR21),1)</f>
+        <f>ROUND(AVERAGE(G21:BT21),1)</f>
         <v/>
       </c>
       <c r="S21" s="79" t="n">
@@ -14686,6 +14705,12 @@
         <v>3</v>
       </c>
       <c r="BR21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14705,11 +14730,11 @@
         <v>8</v>
       </c>
       <c r="E22" s="125">
-        <f>SUM(G22:BR22)</f>
+        <f>SUM(G22:BT22)</f>
         <v/>
       </c>
       <c r="F22" s="125">
-        <f>ROUND(AVERAGE(G22:BR22),1)</f>
+        <f>ROUND(AVERAGE(G22:BT22),1)</f>
         <v/>
       </c>
       <c r="G22" s="79" t="n">
@@ -14784,14 +14809,14 @@
         <v>0</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E23" s="125">
-        <f>SUM(G23:BR23)</f>
+        <f>SUM(G23:BT23)</f>
         <v/>
       </c>
       <c r="F23" s="125">
-        <f>ROUND(AVERAGE(G23:BR23),1)</f>
+        <f>ROUND(AVERAGE(G23:BT23),1)</f>
         <v/>
       </c>
       <c r="AI23" s="125" t="n"/>
@@ -14832,6 +14857,12 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BS23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT23" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
@@ -14849,11 +14880,11 @@
         <v>5</v>
       </c>
       <c r="E24" s="125">
-        <f>SUM(G24:BR24)</f>
+        <f>SUM(G24:BT24)</f>
         <v/>
       </c>
       <c r="F24" s="125">
-        <f>ROUND(AVERAGE(G24:BR24),1)</f>
+        <f>ROUND(AVERAGE(G24:BT24),1)</f>
         <v/>
       </c>
       <c r="AE24" s="79" t="n">
@@ -14911,11 +14942,11 @@
         <v>6</v>
       </c>
       <c r="E25" s="125">
-        <f>SUM(G25:BR25)</f>
+        <f>SUM(G25:BT25)</f>
         <v/>
       </c>
       <c r="F25" s="125">
-        <f>ROUND(AVERAGE(G25:BR25),1)</f>
+        <f>ROUND(AVERAGE(G25:BT25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="125" t="n"/>
@@ -14981,11 +15012,11 @@
         <v>5</v>
       </c>
       <c r="E26" s="125">
-        <f>SUM(G26:BR26)</f>
+        <f>SUM(G26:BT26)</f>
         <v/>
       </c>
       <c r="F26" s="125">
-        <f>ROUND(AVERAGE(G26:BR26),1)</f>
+        <f>ROUND(AVERAGE(G26:BT26),1)</f>
         <v/>
       </c>
       <c r="AM26" t="n">
@@ -15034,14 +15065,14 @@
         <v>0</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="125">
-        <f>SUM(G27:BR27)</f>
+        <f>SUM(G27:BT27)</f>
         <v/>
       </c>
       <c r="F27" s="125">
-        <f>ROUND(AVERAGE(G27:BR27),1)</f>
+        <f>ROUND(AVERAGE(G27:BT27),1)</f>
         <v/>
       </c>
       <c r="I27" s="79" t="n">
@@ -15136,6 +15167,12 @@
       <c r="BP27" t="n">
         <v>3</v>
       </c>
+      <c r="BS27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT27" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
@@ -15153,11 +15190,11 @@
         <v>16</v>
       </c>
       <c r="E28" s="125">
-        <f>SUM(G28:BR28)</f>
+        <f>SUM(G28:BT28)</f>
         <v/>
       </c>
       <c r="F28" s="125">
-        <f>ROUND(AVERAGE(G28:BR28),1)</f>
+        <f>ROUND(AVERAGE(G28:BT28),1)</f>
         <v/>
       </c>
       <c r="G28" s="79" t="n">
@@ -15286,20 +15323,20 @@
         </is>
       </c>
       <c r="B29" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="79" t="n">
         <v>4</v>
       </c>
-      <c r="C29" s="125" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="79" t="n">
-        <v>3</v>
-      </c>
       <c r="E29" s="125">
-        <f>SUM(G29:BR29)</f>
+        <f>SUM(G29:BT29)</f>
         <v/>
       </c>
       <c r="F29" s="125">
-        <f>ROUND(AVERAGE(G29:BR29),1)</f>
+        <f>ROUND(AVERAGE(G29:BT29),1)</f>
         <v/>
       </c>
       <c r="AM29" s="125" t="n"/>
@@ -15336,6 +15373,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BS29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
@@ -15353,11 +15398,11 @@
         <v>4</v>
       </c>
       <c r="E30" s="125">
-        <f>SUM(G30:BR30)</f>
+        <f>SUM(G30:BT30)</f>
         <v/>
       </c>
       <c r="F30" s="125">
-        <f>ROUND(AVERAGE(G30:BR30),1)</f>
+        <f>ROUND(AVERAGE(G30:BT30),1)</f>
         <v/>
       </c>
       <c r="AM30" s="124" t="n">
@@ -15405,11 +15450,11 @@
         <v>6</v>
       </c>
       <c r="E31" s="125">
-        <f>SUM(G31:BR31)</f>
+        <f>SUM(G31:BT31)</f>
         <v/>
       </c>
       <c r="F31" s="125">
-        <f>ROUND(AVERAGE(G31:BR31),1)</f>
+        <f>ROUND(AVERAGE(G31:BT31),1)</f>
         <v/>
       </c>
       <c r="BE31" t="n">
@@ -15483,11 +15528,11 @@
         <v>0</v>
       </c>
       <c r="E32" s="125">
-        <f>SUM(G32:BR32)</f>
+        <f>SUM(G32:BT32)</f>
         <v/>
       </c>
       <c r="F32" s="125">
-        <f>ROUND(AVERAGE(G32:BR32),1)</f>
+        <f>ROUND(AVERAGE(G32:BT32),1)</f>
         <v/>
       </c>
     </row>
@@ -15504,14 +15549,14 @@
         <v>0</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E33" s="125">
-        <f>SUM(G33:BR33)</f>
+        <f>SUM(G33:BT33)</f>
         <v/>
       </c>
       <c r="F33" s="125">
-        <f>ROUND(AVERAGE(G33:BR33),1)</f>
+        <f>ROUND(AVERAGE(G33:BT33),1)</f>
         <v/>
       </c>
       <c r="BA33" t="n">
@@ -15552,6 +15597,12 @@
         <v>2</v>
       </c>
       <c r="BP33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT33" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15568,14 +15619,14 @@
         <v>1</v>
       </c>
       <c r="D34" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E34" s="125">
-        <f>SUM(G34:BR34)</f>
+        <f>SUM(G34:BT34)</f>
         <v/>
       </c>
       <c r="F34" s="125">
-        <f>ROUND(AVERAGE(G34:BR34),1)</f>
+        <f>ROUND(AVERAGE(G34:BT34),1)</f>
         <v/>
       </c>
       <c r="G34" s="79" t="n">
@@ -15671,6 +15722,12 @@
       </c>
       <c r="BR34" t="n">
         <v>3</v>
+      </c>
+      <c r="BS34" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT34" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -15686,14 +15743,14 @@
         <v>1</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E35" s="125">
-        <f>SUM(G35:BR35)</f>
+        <f>SUM(G35:BT35)</f>
         <v/>
       </c>
       <c r="F35" s="125">
-        <f>ROUND(AVERAGE(G35:BR35),1)</f>
+        <f>ROUND(AVERAGE(G35:BT35),1)</f>
         <v/>
       </c>
       <c r="I35" s="79" t="n">
@@ -15764,6 +15821,12 @@
         <v>2</v>
       </c>
       <c r="BR35" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS35" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT35" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15783,11 +15846,11 @@
         <v>3</v>
       </c>
       <c r="E36" s="125">
-        <f>SUM(G36:BR36)</f>
+        <f>SUM(G36:BT36)</f>
         <v/>
       </c>
       <c r="F36" s="125">
-        <f>ROUND(AVERAGE(G36:BR36),1)</f>
+        <f>ROUND(AVERAGE(G36:BT36),1)</f>
         <v/>
       </c>
       <c r="Y36" s="79" t="n">
@@ -15827,11 +15890,11 @@
         <v>13</v>
       </c>
       <c r="E37" s="125">
-        <f>SUM(G37:BR37)</f>
+        <f>SUM(G37:BT37)</f>
         <v/>
       </c>
       <c r="F37" s="125">
-        <f>ROUND(AVERAGE(G37:BR37),1)</f>
+        <f>ROUND(AVERAGE(G37:BT37),1)</f>
         <v/>
       </c>
       <c r="S37" s="79" t="n">
@@ -15943,11 +16006,11 @@
         <v>12</v>
       </c>
       <c r="E38" s="125">
-        <f>SUM(G38:BR38)</f>
+        <f>SUM(G38:BT38)</f>
         <v/>
       </c>
       <c r="F38" s="125">
-        <f>ROUND(AVERAGE(G38:BR38),1)</f>
+        <f>ROUND(AVERAGE(G38:BT38),1)</f>
         <v/>
       </c>
       <c r="I38" s="79" t="inlineStr">
@@ -16053,11 +16116,11 @@
         <v>8</v>
       </c>
       <c r="E39" s="125">
-        <f>SUM(G39:BR39)</f>
+        <f>SUM(G39:BT39)</f>
         <v/>
       </c>
       <c r="F39" s="125">
-        <f>ROUND(AVERAGE(G39:BR39),1)</f>
+        <f>ROUND(AVERAGE(G39:BT39),1)</f>
         <v/>
       </c>
       <c r="G39" s="79" t="n">
@@ -16126,14 +16189,14 @@
         <v>1</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E40" s="125">
-        <f>SUM(G40:BR40)</f>
+        <f>SUM(G40:BT40)</f>
         <v/>
       </c>
       <c r="F40" s="125">
-        <f>ROUND(AVERAGE(G40:BR40),1)</f>
+        <f>ROUND(AVERAGE(G40:BT40),1)</f>
         <v/>
       </c>
       <c r="G40" s="79" t="n">
@@ -16229,6 +16292,12 @@
       </c>
       <c r="BP40" t="n">
         <v>1</v>
+      </c>
+      <c r="BS40" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT40" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -16238,20 +16307,20 @@
         </is>
       </c>
       <c r="B41" s="79" t="n">
+        <v>9</v>
+      </c>
+      <c r="C41" s="125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="79" t="n">
         <v>8</v>
       </c>
-      <c r="C41" s="125" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="79" t="n">
-        <v>7</v>
-      </c>
       <c r="E41" s="125">
-        <f>SUM(G41:BR41)</f>
+        <f>SUM(G41:BT41)</f>
         <v/>
       </c>
       <c r="F41" s="125">
-        <f>ROUND(AVERAGE(G41:BR41),1)</f>
+        <f>ROUND(AVERAGE(G41:BT41),1)</f>
         <v/>
       </c>
       <c r="BC41" t="inlineStr">
@@ -16308,6 +16377,14 @@
         <v>2</v>
       </c>
       <c r="BR41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS41" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT41" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16329,11 +16406,11 @@
         <v>1</v>
       </c>
       <c r="E42" s="125">
-        <f>SUM(G42:BR42)</f>
+        <f>SUM(G42:BT42)</f>
         <v/>
       </c>
       <c r="F42" s="125">
-        <f>ROUND(AVERAGE(G42:BR42),1)</f>
+        <f>ROUND(AVERAGE(G42:BT42),1)</f>
         <v/>
       </c>
       <c r="AS42" s="124" t="n">
@@ -16350,20 +16427,20 @@
         </is>
       </c>
       <c r="B43" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C43" s="125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E43" s="125">
-        <f>SUM(G43:BR43)</f>
+        <f>SUM(G43:BT43)</f>
         <v/>
       </c>
       <c r="F43" s="125">
-        <f>ROUND(AVERAGE(G43:BR43),1)</f>
+        <f>ROUND(AVERAGE(G43:BT43),1)</f>
         <v/>
       </c>
       <c r="G43" s="79" t="n">
@@ -16512,6 +16589,16 @@
         </is>
       </c>
       <c r="BR43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT43" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16533,11 +16620,11 @@
         <v>15</v>
       </c>
       <c r="E44" s="125">
-        <f>SUM(G44:BR44)</f>
+        <f>SUM(G44:BT44)</f>
         <v/>
       </c>
       <c r="F44" s="125">
-        <f>ROUND(AVERAGE(G44:BR44),1)</f>
+        <f>ROUND(AVERAGE(G44:BT44),1)</f>
         <v/>
       </c>
       <c r="U44" s="79" t="n">
@@ -16648,7 +16735,7 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Er Caciotta</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -16661,11 +16748,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="125">
-        <f>SUM(G45:BR45)</f>
+        <f>SUM(G45:BT45)</f>
         <v/>
       </c>
       <c r="F45" s="125">
-        <f>ROUND(AVERAGE(G45:BR45),1)</f>
+        <f>ROUND(AVERAGE(G45:BT45),1)</f>
         <v/>
       </c>
       <c r="U45" s="79" t="n"/>
@@ -16692,24 +16779,24 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>er samu</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C46" s="125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="125">
-        <f>SUM(G46:BR46)</f>
+        <f>SUM(G46:BT46)</f>
         <v/>
       </c>
       <c r="F46" s="125">
-        <f>ROUND(AVERAGE(G46:BR46),1)</f>
+        <f>ROUND(AVERAGE(G46:BT46),1)</f>
         <v/>
       </c>
       <c r="U46" s="79" t="n"/>
@@ -16732,11 +16819,21 @@
       <c r="AN46" s="126" t="n"/>
       <c r="AO46" s="124" t="n"/>
       <c r="AP46" s="126" t="n"/>
+      <c r="BS46" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT46" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>er samu</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -16749,11 +16846,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="125">
-        <f>SUM(G47:BR47)</f>
+        <f>SUM(G47:BT47)</f>
         <v/>
       </c>
       <c r="F47" s="125">
-        <f>ROUND(AVERAGE(G47:BR47),1)</f>
+        <f>ROUND(AVERAGE(G47:BT47),1)</f>
         <v/>
       </c>
       <c r="U47" s="79" t="n"/>
@@ -16780,7 +16877,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>salvuz11</t>
+          <t>krigohard</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -16793,11 +16890,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="125">
-        <f>SUM(G48:BR48)</f>
+        <f>SUM(G48:BT48)</f>
         <v/>
       </c>
       <c r="F48" s="125">
-        <f>ROUND(AVERAGE(G48:BR48),1)</f>
+        <f>ROUND(AVERAGE(G48:BT48),1)</f>
         <v/>
       </c>
       <c r="U48" s="79" t="n"/>
@@ -16824,7 +16921,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>_loris_yt</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -16837,11 +16934,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="125">
-        <f>SUM(G49:BR49)</f>
+        <f>SUM(G49:BT49)</f>
         <v/>
       </c>
       <c r="F49" s="125">
-        <f>ROUND(AVERAGE(G49:BR49),1)</f>
+        <f>ROUND(AVERAGE(G49:BT49),1)</f>
         <v/>
       </c>
       <c r="U49" s="79" t="n"/>
@@ -16868,7 +16965,7 @@
     <row r="50">
       <c r="A50" s="79" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>cactus</t>
         </is>
       </c>
       <c r="B50" s="79" t="n">
@@ -16881,11 +16978,11 @@
         <v>0</v>
       </c>
       <c r="E50" s="125">
-        <f>SUM(G50:BR50)</f>
+        <f>SUM(G50:BT50)</f>
         <v/>
       </c>
       <c r="F50" s="125">
-        <f>ROUND(AVERAGE(G50:BR50),1)</f>
+        <f>ROUND(AVERAGE(G50:BT50),1)</f>
         <v/>
       </c>
       <c r="U50" s="79" t="n"/>
@@ -16909,6 +17006,50 @@
       <c r="AO50" s="124" t="n"/>
       <c r="AP50" s="126" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>Steninja:)</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="125">
+        <f>SUM(G51:BT51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="125">
+        <f>ROUND(AVERAGE(G51:BT51),1)</f>
+        <v/>
+      </c>
+      <c r="U51" s="79" t="n"/>
+      <c r="V51" s="80" t="n"/>
+      <c r="W51" s="79" t="n"/>
+      <c r="X51" s="80" t="n"/>
+      <c r="Y51" s="79" t="n"/>
+      <c r="Z51" s="80" t="n"/>
+      <c r="AA51" s="79" t="n"/>
+      <c r="AB51" s="80" t="n"/>
+      <c r="AC51" s="79" t="n"/>
+      <c r="AD51" s="80" t="n"/>
+      <c r="AE51" s="79" t="n"/>
+      <c r="AF51" s="80" t="n"/>
+      <c r="AI51" s="124" t="n"/>
+      <c r="AJ51" s="126" t="n"/>
+      <c r="AK51" s="124" t="n"/>
+      <c r="AL51" s="126" t="n"/>
+      <c r="AM51" s="124" t="n"/>
+      <c r="AN51" s="126" t="n"/>
+      <c r="AO51" s="124" t="n"/>
+      <c r="AP51" s="126" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:CL1">
     <sortState ref="A2:CL51">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-16
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -11289,7 +11289,7 @@
   <dimension ref="A1:AH49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col hidden="1" min="9" max="27"/>
+    <col hidden="1" width="13" customWidth="1" min="9" max="27"/>
     <col width="16.5703125" customWidth="1" min="28" max="28"/>
     <col width="15.7109375" customWidth="1" min="33" max="33"/>
   </cols>
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI51"/>
+  <dimension ref="A1:CI49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13151,12 +13151,12 @@
       </c>
       <c r="BW1" s="109" t="inlineStr">
         <is>
-          <t>Colonna75</t>
+          <t>WAR-35 (1)</t>
         </is>
       </c>
       <c r="BX1" s="109" t="inlineStr">
         <is>
-          <t>Colonna76</t>
+          <t>WAR-35 (2)</t>
         </is>
       </c>
       <c r="BY1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BV2)</f>
+        <f>SUM(G2:BX2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BV2),1)</f>
+        <f>ROUND(AVERAGE(G2:BX2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BV3)</f>
+        <f>SUM(G3:BX3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BV3),1)</f>
+        <f>ROUND(AVERAGE(G3:BX3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13302,20 +13302,20 @@
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BV4)</f>
+        <f>SUM(G4:BX4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BV4),1)</f>
+        <f>ROUND(AVERAGE(G4:BX4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13389,6 +13389,16 @@
       </c>
       <c r="BV4" t="n">
         <v>3</v>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -13398,20 +13408,20 @@
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C5" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BV5)</f>
+        <f>SUM(G5:BX5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BV5),1)</f>
+        <f>ROUND(AVERAGE(G5:BX5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13444,6 +13454,16 @@
         </is>
       </c>
       <c r="BV5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX5" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13456,20 +13476,20 @@
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" s="68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BV6)</f>
+        <f>SUM(G6:BX6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BV6),1)</f>
+        <f>ROUND(AVERAGE(G6:BX6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13638,6 +13658,16 @@
         <v>1</v>
       </c>
       <c r="BV6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13659,11 +13689,11 @@
         <v>10</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BV7)</f>
+        <f>SUM(G7:BX7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BV7),1)</f>
+        <f>ROUND(AVERAGE(G7:BX7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13747,11 +13777,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BV8)</f>
+        <f>SUM(G8:BX8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BV8),1)</f>
+        <f>ROUND(AVERAGE(G8:BX8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13772,20 +13802,20 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BV9)</f>
+        <f>SUM(G9:BX9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BV9),1)</f>
+        <f>ROUND(AVERAGE(G9:BX9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13859,6 +13889,16 @@
       </c>
       <c r="BV9" t="n">
         <v>3</v>
+      </c>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -13877,11 +13917,11 @@
         <v>19</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BV10)</f>
+        <f>SUM(G10:BX10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BV10),1)</f>
+        <f>ROUND(AVERAGE(G10:BX10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14035,11 +14075,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BV11)</f>
+        <f>SUM(G11:BX11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BV11),1)</f>
+        <f>ROUND(AVERAGE(G11:BX11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14073,11 +14113,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BV12)</f>
+        <f>SUM(G12:BX12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BV12),1)</f>
+        <f>ROUND(AVERAGE(G12:BX12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14125,11 +14165,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BV13)</f>
+        <f>SUM(G13:BX13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BV13),1)</f>
+        <f>ROUND(AVERAGE(G13:BX13),1)</f>
         <v/>
       </c>
     </row>
@@ -14140,20 +14180,20 @@
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C14" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BV14)</f>
+        <f>SUM(G14:BX14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BV14),1)</f>
+        <f>ROUND(AVERAGE(G14:BX14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14238,6 +14278,16 @@
       <c r="BV14" t="n">
         <v>1</v>
       </c>
+      <c r="BW14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
@@ -14255,11 +14305,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BV15)</f>
+        <f>SUM(G15:BX15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BV15),1)</f>
+        <f>ROUND(AVERAGE(G15:BX15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14285,11 +14335,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BV16)</f>
+        <f>SUM(G16:BX16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BV16),1)</f>
+        <f>ROUND(AVERAGE(G16:BX16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14406,20 +14456,20 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BV17)</f>
+        <f>SUM(G17:BX17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BV17),1)</f>
+        <f>ROUND(AVERAGE(G17:BX17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14557,6 +14607,16 @@
       </c>
       <c r="BV17" t="n">
         <v>3</v>
+      </c>
+      <c r="BW17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -14566,20 +14626,20 @@
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C18" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BV18)</f>
+        <f>SUM(G18:BX18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BV18),1)</f>
+        <f>ROUND(AVERAGE(G18:BX18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14663,6 +14723,16 @@
       </c>
       <c r="BV18" t="n">
         <v>3</v>
+      </c>
+      <c r="BW18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -14681,11 +14751,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BV19)</f>
+        <f>SUM(G19:BX19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BV19),1)</f>
+        <f>ROUND(AVERAGE(G19:BX19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14763,11 +14833,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BV20)</f>
+        <f>SUM(G20:BX20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BV20),1)</f>
+        <f>ROUND(AVERAGE(G20:BX20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -14831,11 +14901,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BV21)</f>
+        <f>SUM(G21:BX21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BV21),1)</f>
+        <f>ROUND(AVERAGE(G21:BX21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -14884,20 +14954,20 @@
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BV22)</f>
+        <f>SUM(G22:BX22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BV22),1)</f>
+        <f>ROUND(AVERAGE(G22:BX22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -14952,6 +15022,16 @@
       <c r="BV22" t="n">
         <v>3</v>
       </c>
+      <c r="BW22" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX22" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
@@ -14969,11 +15049,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BV23)</f>
+        <f>SUM(G23:BX23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BV23),1)</f>
+        <f>ROUND(AVERAGE(G23:BX23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15082,20 +15162,20 @@
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C24" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BV24)</f>
+        <f>SUM(G24:BX24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BV24),1)</f>
+        <f>ROUND(AVERAGE(G24:BX24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15224,6 +15304,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BW24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
@@ -15232,20 +15322,20 @@
         </is>
       </c>
       <c r="B25" s="79" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="79" t="n">
         <v>6</v>
       </c>
-      <c r="C25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="79" t="n">
-        <v>5</v>
-      </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BV25)</f>
+        <f>SUM(G25:BX25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BV25),1)</f>
+        <f>ROUND(AVERAGE(G25:BX25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15298,6 +15388,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BW25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
@@ -15315,11 +15415,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BV26)</f>
+        <f>SUM(G26:BX26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BV26),1)</f>
+        <f>ROUND(AVERAGE(G26:BX26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15358,20 +15458,20 @@
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BV27)</f>
+        <f>SUM(G27:BX27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BV27),1)</f>
+        <f>ROUND(AVERAGE(G27:BX27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15479,6 +15579,16 @@
       </c>
       <c r="BV27" t="n">
         <v>2</v>
+      </c>
+      <c r="BW27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -15488,20 +15598,20 @@
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BV28)</f>
+        <f>SUM(G28:BX28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BV28),1)</f>
+        <f>ROUND(AVERAGE(G28:BX28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -15579,6 +15689,16 @@
       </c>
       <c r="BT28" t="n">
         <v>3</v>
+      </c>
+      <c r="BW28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -15597,11 +15717,11 @@
         <v>4</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BV29)</f>
+        <f>SUM(G29:BX29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BV29),1)</f>
+        <f>ROUND(AVERAGE(G29:BX29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -15647,11 +15767,11 @@
         <v>14</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BV30)</f>
+        <f>SUM(G30:BX30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BV30),1)</f>
+        <f>ROUND(AVERAGE(G30:BX30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -15769,11 +15889,11 @@
         <v>13</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BV31)</f>
+        <f>SUM(G31:BX31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BV31),1)</f>
+        <f>ROUND(AVERAGE(G31:BX31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -15889,11 +16009,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BV32)</f>
+        <f>SUM(G32:BX32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BV32),1)</f>
+        <f>ROUND(AVERAGE(G32:BX32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -15965,11 +16085,11 @@
         <v>15</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BV33)</f>
+        <f>SUM(G33:BX33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BV33),1)</f>
+        <f>ROUND(AVERAGE(G33:BX33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16089,11 +16209,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BV34)</f>
+        <f>SUM(G34:BX34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BV34),1)</f>
+        <f>ROUND(AVERAGE(G34:BX34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16119,11 +16239,11 @@
         <v>25</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BV35)</f>
+        <f>SUM(G35:BX35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BV35),1)</f>
+        <f>ROUND(AVERAGE(G35:BX35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16309,11 +16429,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BV36)</f>
+        <f>SUM(G36:BX36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BV36),1)</f>
+        <f>ROUND(AVERAGE(G36:BX36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16437,11 +16557,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BV37)</f>
+        <f>SUM(G37:BX37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BV37),1)</f>
+        <f>ROUND(AVERAGE(G37:BX37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16469,11 +16589,11 @@
         <v>0</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BV38)</f>
+        <f>SUM(G38:BX38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BV38),1)</f>
+        <f>ROUND(AVERAGE(G38:BX38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16501,11 +16621,11 @@
         <v>0</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BV39)</f>
+        <f>SUM(G39:BX39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BV39),1)</f>
+        <f>ROUND(AVERAGE(G39:BX39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16533,11 +16653,11 @@
         <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BV40)</f>
+        <f>SUM(G40:BX40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BV40),1)</f>
+        <f>ROUND(AVERAGE(G40:BX40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -16565,11 +16685,11 @@
         <v>1</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BV41)</f>
+        <f>SUM(G41:BX41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BV41),1)</f>
+        <f>ROUND(AVERAGE(G41:BX41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -16607,11 +16727,11 @@
         <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BV42)</f>
+        <f>SUM(G42:BX42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BV42),1)</f>
+        <f>ROUND(AVERAGE(G42:BX42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -16630,20 +16750,20 @@
         </is>
       </c>
       <c r="B43" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C43" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BV43)</f>
+        <f>SUM(G43:BX43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BV43),1)</f>
+        <f>ROUND(AVERAGE(G43:BX43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -16654,11 +16774,21 @@
       <c r="AN43" s="121" t="n"/>
       <c r="AO43" s="120" t="n"/>
       <c r="AP43" s="121" t="n"/>
+      <c r="BW43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>MRCOMPLEX</t>
+          <t>color052</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -16671,11 +16801,11 @@
         <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BV44)</f>
+        <f>SUM(G44:BX44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BV44),1)</f>
+        <f>ROUND(AVERAGE(G44:BX44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -16690,24 +16820,24 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Ascanio3</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BV45)</f>
+        <f>SUM(G45:BX45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BV45),1)</f>
+        <f>ROUND(AVERAGE(G45:BX45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -16718,11 +16848,21 @@
       <c r="AN45" s="121" t="n"/>
       <c r="AO45" s="120" t="n"/>
       <c r="AP45" s="121" t="n"/>
+      <c r="BW45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>color052</t>
+          <t>Michele</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -16735,11 +16875,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BV46)</f>
+        <f>SUM(G46:BX46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BV46),1)</f>
+        <f>ROUND(AVERAGE(G46:BX46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -16754,24 +16894,24 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>ggvitotmm</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BV47)</f>
+        <f>SUM(G47:BX47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BV47),1)</f>
+        <f>ROUND(AVERAGE(G47:BX47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -16782,11 +16922,31 @@
       <c r="AN47" s="121" t="n"/>
       <c r="AO47" s="120" t="n"/>
       <c r="AP47" s="121" t="n"/>
+      <c r="BU47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BV47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BW47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>toxic</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -16799,11 +16959,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BV48)</f>
+        <f>SUM(G48:BX48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BV48),1)</f>
+        <f>ROUND(AVERAGE(G48:BX48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -16818,7 +16978,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>gamer</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -16831,11 +16991,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BV49)</f>
+        <f>SUM(G49:BX49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BV49),1)</f>
+        <f>ROUND(AVERAGE(G49:BX49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>
@@ -16846,80 +17006,6 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>ggvitotmm</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:BV50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BV50),1)</f>
-        <v/>
-      </c>
-      <c r="AI50" s="120" t="n"/>
-      <c r="AJ50" s="121" t="n"/>
-      <c r="AK50" s="120" t="n"/>
-      <c r="AL50" s="121" t="n"/>
-      <c r="AM50" s="120" t="n"/>
-      <c r="AN50" s="121" t="n"/>
-      <c r="AO50" s="120" t="n"/>
-      <c r="AP50" s="121" t="n"/>
-      <c r="BU50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV50" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="79" t="inlineStr">
-        <is>
-          <t>toxic</t>
-        </is>
-      </c>
-      <c r="B51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="68">
-        <f>SUM(G51:BV51)</f>
-        <v/>
-      </c>
-      <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:BV51),1)</f>
-        <v/>
-      </c>
-      <c r="AI51" s="120" t="n"/>
-      <c r="AJ51" s="121" t="n"/>
-      <c r="AK51" s="120" t="n"/>
-      <c r="AL51" s="121" t="n"/>
-      <c r="AM51" s="120" t="n"/>
-      <c r="AN51" s="121" t="n"/>
-      <c r="AO51" s="120" t="n"/>
-      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-18
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI49"/>
+  <dimension ref="A1:CI50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13161,12 +13161,12 @@
       </c>
       <c r="BY1" s="109" t="inlineStr">
         <is>
-          <t>Colonna77</t>
+          <t>WAR-36 (1)</t>
         </is>
       </c>
       <c r="BZ1" s="109" t="inlineStr">
         <is>
-          <t>Colonna78</t>
+          <t>WAR-36 (2)</t>
         </is>
       </c>
       <c r="CA1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BX2)</f>
+        <f>SUM(G2:BZ2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BX2),1)</f>
+        <f>ROUND(AVERAGE(G2:BZ2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BX3)</f>
+        <f>SUM(G3:BZ3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BX3),1)</f>
+        <f>ROUND(AVERAGE(G3:BZ3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13308,14 +13308,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BX4)</f>
+        <f>SUM(G4:BZ4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BX4),1)</f>
+        <f>ROUND(AVERAGE(G4:BZ4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13399,6 +13399,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -13408,20 +13414,20 @@
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BX5)</f>
+        <f>SUM(G5:BZ5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BX5),1)</f>
+        <f>ROUND(AVERAGE(G5:BZ5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13464,6 +13470,16 @@
         </is>
       </c>
       <c r="BX5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BZ5" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13476,20 +13492,20 @@
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="68" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BX6)</f>
+        <f>SUM(G6:BZ6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BX6),1)</f>
+        <f>ROUND(AVERAGE(G6:BZ6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13668,6 +13684,14 @@
         </is>
       </c>
       <c r="BX6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -13689,11 +13713,11 @@
         <v>10</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BX7)</f>
+        <f>SUM(G7:BZ7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BX7),1)</f>
+        <f>ROUND(AVERAGE(G7:BZ7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13777,11 +13801,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BX8)</f>
+        <f>SUM(G8:BZ8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BX8),1)</f>
+        <f>ROUND(AVERAGE(G8:BZ8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13808,14 +13832,14 @@
         <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BX9)</f>
+        <f>SUM(G9:BZ9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BX9),1)</f>
+        <f>ROUND(AVERAGE(G9:BZ9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13899,6 +13923,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -13917,11 +13947,11 @@
         <v>19</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BX10)</f>
+        <f>SUM(G10:BZ10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BX10),1)</f>
+        <f>ROUND(AVERAGE(G10:BZ10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14075,11 +14105,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BX11)</f>
+        <f>SUM(G11:BZ11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BX11),1)</f>
+        <f>ROUND(AVERAGE(G11:BZ11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14113,11 +14143,11 @@
         <v>4</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BX12)</f>
+        <f>SUM(G12:BZ12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BX12),1)</f>
+        <f>ROUND(AVERAGE(G12:BZ12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14165,11 +14195,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BX13)</f>
+        <f>SUM(G13:BZ13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BX13),1)</f>
+        <f>ROUND(AVERAGE(G13:BZ13),1)</f>
         <v/>
       </c>
     </row>
@@ -14186,14 +14216,14 @@
         <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BX14)</f>
+        <f>SUM(G14:BZ14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BX14),1)</f>
+        <f>ROUND(AVERAGE(G14:BZ14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14288,6 +14318,12 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BY14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
@@ -14305,11 +14341,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BX15)</f>
+        <f>SUM(G15:BZ15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BX15),1)</f>
+        <f>ROUND(AVERAGE(G15:BZ15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14335,11 +14371,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BX16)</f>
+        <f>SUM(G16:BZ16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BX16),1)</f>
+        <f>ROUND(AVERAGE(G16:BZ16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14462,14 +14498,14 @@
         <v>2</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BX17)</f>
+        <f>SUM(G17:BZ17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BX17),1)</f>
+        <f>ROUND(AVERAGE(G17:BZ17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14617,6 +14653,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -14632,14 +14674,14 @@
         <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BX18)</f>
+        <f>SUM(G18:BZ18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BX18),1)</f>
+        <f>ROUND(AVERAGE(G18:BZ18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14733,6 +14775,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY18" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -14751,11 +14799,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BX19)</f>
+        <f>SUM(G19:BZ19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BX19),1)</f>
+        <f>ROUND(AVERAGE(G19:BZ19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14833,11 +14881,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BX20)</f>
+        <f>SUM(G20:BZ20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BX20),1)</f>
+        <f>ROUND(AVERAGE(G20:BZ20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -14901,11 +14949,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BX21)</f>
+        <f>SUM(G21:BZ21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BX21),1)</f>
+        <f>ROUND(AVERAGE(G21:BZ21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -14960,14 +15008,14 @@
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BX22)</f>
+        <f>SUM(G22:BZ22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BX22),1)</f>
+        <f>ROUND(AVERAGE(G22:BZ22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -15032,6 +15080,12 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BY22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ22" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
@@ -15049,11 +15103,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BX23)</f>
+        <f>SUM(G23:BZ23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BX23),1)</f>
+        <f>ROUND(AVERAGE(G23:BZ23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15162,20 +15216,20 @@
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C24" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BX24)</f>
+        <f>SUM(G24:BZ24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BX24),1)</f>
+        <f>ROUND(AVERAGE(G24:BZ24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15314,6 +15368,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BY24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
@@ -15322,20 +15384,20 @@
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BX25)</f>
+        <f>SUM(G25:BZ25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BX25),1)</f>
+        <f>ROUND(AVERAGE(G25:BZ25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15398,6 +15460,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BY25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BZ25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
@@ -15415,11 +15487,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BX26)</f>
+        <f>SUM(G26:BZ26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BX26),1)</f>
+        <f>ROUND(AVERAGE(G26:BZ26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15464,14 +15536,14 @@
         <v>2</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BX27)</f>
+        <f>SUM(G27:BZ27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BX27),1)</f>
+        <f>ROUND(AVERAGE(G27:BZ27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15589,6 +15661,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY27" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ27" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -15604,14 +15682,14 @@
         <v>2</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BX28)</f>
+        <f>SUM(G28:BZ28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BX28),1)</f>
+        <f>ROUND(AVERAGE(G28:BZ28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -15699,6 +15777,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BY28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ28" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -15717,11 +15801,11 @@
         <v>4</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BX29)</f>
+        <f>SUM(G29:BZ29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BX29),1)</f>
+        <f>ROUND(AVERAGE(G29:BZ29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -15767,11 +15851,11 @@
         <v>14</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BX30)</f>
+        <f>SUM(G30:BZ30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BX30),1)</f>
+        <f>ROUND(AVERAGE(G30:BZ30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -15889,11 +15973,11 @@
         <v>13</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BX31)</f>
+        <f>SUM(G31:BZ31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BX31),1)</f>
+        <f>ROUND(AVERAGE(G31:BZ31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -16009,11 +16093,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BX32)</f>
+        <f>SUM(G32:BZ32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BX32),1)</f>
+        <f>ROUND(AVERAGE(G32:BZ32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -16085,11 +16169,11 @@
         <v>15</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BX33)</f>
+        <f>SUM(G33:BZ33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BX33),1)</f>
+        <f>ROUND(AVERAGE(G33:BZ33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16209,11 +16293,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BX34)</f>
+        <f>SUM(G34:BZ34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BX34),1)</f>
+        <f>ROUND(AVERAGE(G34:BZ34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16239,11 +16323,11 @@
         <v>25</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BX35)</f>
+        <f>SUM(G35:BZ35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BX35),1)</f>
+        <f>ROUND(AVERAGE(G35:BZ35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16429,11 +16513,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BX36)</f>
+        <f>SUM(G36:BZ36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BX36),1)</f>
+        <f>ROUND(AVERAGE(G36:BZ36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16557,11 +16641,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BX37)</f>
+        <f>SUM(G37:BZ37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BX37),1)</f>
+        <f>ROUND(AVERAGE(G37:BZ37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16589,11 +16673,11 @@
         <v>0</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BX38)</f>
+        <f>SUM(G38:BZ38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BX38),1)</f>
+        <f>ROUND(AVERAGE(G38:BZ38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16621,11 +16705,11 @@
         <v>0</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BX39)</f>
+        <f>SUM(G39:BZ39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BX39),1)</f>
+        <f>ROUND(AVERAGE(G39:BZ39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16653,11 +16737,11 @@
         <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BX40)</f>
+        <f>SUM(G40:BZ40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BX40),1)</f>
+        <f>ROUND(AVERAGE(G40:BZ40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -16685,11 +16769,11 @@
         <v>1</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BX41)</f>
+        <f>SUM(G41:BZ41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BX41),1)</f>
+        <f>ROUND(AVERAGE(G41:BZ41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -16727,11 +16811,11 @@
         <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BX42)</f>
+        <f>SUM(G42:BZ42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BX42),1)</f>
+        <f>ROUND(AVERAGE(G42:BZ42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -16756,14 +16840,14 @@
         <v>1</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BX43)</f>
+        <f>SUM(G43:BZ43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BX43),1)</f>
+        <f>ROUND(AVERAGE(G43:BZ43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -16784,28 +16868,34 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="BY43" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ43" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>color052</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BX44)</f>
+        <f>SUM(G44:BZ44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BX44),1)</f>
+        <f>ROUND(AVERAGE(G44:BZ44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -16816,28 +16906,44 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
+      <c r="BW44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY44" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ44" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>ggvitotmm</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BX45)</f>
+        <f>SUM(G45:BZ45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BX45),1)</f>
+        <f>ROUND(AVERAGE(G45:BZ45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -16848,12 +16954,32 @@
       <c r="AN45" s="121" t="n"/>
       <c r="AO45" s="120" t="n"/>
       <c r="AP45" s="121" t="n"/>
+      <c r="BU45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BV45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="BW45" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
       <c r="BX45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BZ45" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16862,7 +16988,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>toxic</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -16875,11 +17001,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BX46)</f>
+        <f>SUM(G46:BZ46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BX46),1)</f>
+        <f>ROUND(AVERAGE(G46:BZ46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -16894,24 +17020,24 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>ggvitotmm</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BX47)</f>
+        <f>SUM(G47:BZ47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BX47),1)</f>
+        <f>ROUND(AVERAGE(G47:BZ47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -16922,31 +17048,11 @@
       <c r="AN47" s="121" t="n"/>
       <c r="AO47" s="120" t="n"/>
       <c r="AP47" s="121" t="n"/>
-      <c r="BU47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>toxic</t>
+          <t>andrea</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -16959,11 +17065,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BX48)</f>
+        <f>SUM(G48:BZ48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BX48),1)</f>
+        <f>ROUND(AVERAGE(G48:BZ48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -16978,7 +17084,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>piter</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -16991,11 +17097,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BX49)</f>
+        <f>SUM(G49:BZ49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BX49),1)</f>
+        <f>ROUND(AVERAGE(G49:BZ49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>
@@ -17006,6 +17112,38 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>Anto</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:BZ50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:BZ50),1)</f>
+        <v/>
+      </c>
+      <c r="AI50" s="120" t="n"/>
+      <c r="AJ50" s="121" t="n"/>
+      <c r="AK50" s="120" t="n"/>
+      <c r="AL50" s="121" t="n"/>
+      <c r="AM50" s="120" t="n"/>
+      <c r="AN50" s="121" t="n"/>
+      <c r="AO50" s="120" t="n"/>
+      <c r="AP50" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-20
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI50"/>
+  <dimension ref="A1:CI51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13171,12 +13171,12 @@
       </c>
       <c r="CA1" s="109" t="inlineStr">
         <is>
-          <t>Colonna79</t>
+          <t>WAR-37 (1)</t>
         </is>
       </c>
       <c r="CB1" s="109" t="inlineStr">
         <is>
-          <t>Colonna80</t>
+          <t>WAR-37 (2)</t>
         </is>
       </c>
       <c r="CC1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:BZ2)</f>
+        <f>SUM(G2:CB2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:BZ2),1)</f>
+        <f>ROUND(AVERAGE(G2:CB2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:BZ3)</f>
+        <f>SUM(G3:CB3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:BZ3),1)</f>
+        <f>ROUND(AVERAGE(G3:CB3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13308,14 +13308,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:BZ4)</f>
+        <f>SUM(G4:CB4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:BZ4),1)</f>
+        <f>ROUND(AVERAGE(G4:CB4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13404,6 +13404,12 @@
         <v>3</v>
       </c>
       <c r="BZ4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13420,14 +13426,14 @@
         <v>3</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:BZ5)</f>
+        <f>SUM(G5:CB5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:BZ5),1)</f>
+        <f>ROUND(AVERAGE(G5:CB5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13483,6 +13489,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="CA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -13501,11 +13513,11 @@
         <v>25</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:BZ6)</f>
+        <f>SUM(G6:CB6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:BZ6),1)</f>
+        <f>ROUND(AVERAGE(G6:CB6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13710,14 +13722,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:BZ7)</f>
+        <f>SUM(G7:CB7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:BZ7),1)</f>
+        <f>ROUND(AVERAGE(G7:CB7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13784,6 +13796,12 @@
       <c r="BV7" t="n">
         <v>3</v>
       </c>
+      <c r="CA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
@@ -13801,11 +13819,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:BZ8)</f>
+        <f>SUM(G8:CB8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:BZ8),1)</f>
+        <f>ROUND(AVERAGE(G8:CB8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13835,11 +13853,11 @@
         <v>14</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:BZ9)</f>
+        <f>SUM(G9:CB9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:BZ9),1)</f>
+        <f>ROUND(AVERAGE(G9:CB9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13947,11 +13965,11 @@
         <v>19</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:BZ10)</f>
+        <f>SUM(G10:CB10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:BZ10),1)</f>
+        <f>ROUND(AVERAGE(G10:CB10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14105,11 +14123,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:BZ11)</f>
+        <f>SUM(G11:CB11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:BZ11),1)</f>
+        <f>ROUND(AVERAGE(G11:CB11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14134,20 +14152,20 @@
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:BZ12)</f>
+        <f>SUM(G12:CB12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:BZ12),1)</f>
+        <f>ROUND(AVERAGE(G12:CB12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14177,6 +14195,14 @@
       </c>
       <c r="BV12" t="n">
         <v>3</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -14195,11 +14221,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:BZ13)</f>
+        <f>SUM(G13:CB13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:BZ13),1)</f>
+        <f>ROUND(AVERAGE(G13:CB13),1)</f>
         <v/>
       </c>
     </row>
@@ -14219,11 +14245,11 @@
         <v>13</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:BZ14)</f>
+        <f>SUM(G14:CB14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:BZ14),1)</f>
+        <f>ROUND(AVERAGE(G14:CB14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14341,11 +14367,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:BZ15)</f>
+        <f>SUM(G15:CB15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:BZ15),1)</f>
+        <f>ROUND(AVERAGE(G15:CB15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14371,11 +14397,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:BZ16)</f>
+        <f>SUM(G16:CB16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:BZ16),1)</f>
+        <f>ROUND(AVERAGE(G16:CB16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14501,11 +14527,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:BZ17)</f>
+        <f>SUM(G17:CB17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:BZ17),1)</f>
+        <f>ROUND(AVERAGE(G17:CB17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14674,14 +14700,14 @@
         <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:BZ18)</f>
+        <f>SUM(G18:CB18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:BZ18),1)</f>
+        <f>ROUND(AVERAGE(G18:CB18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14780,6 +14806,12 @@
         <v>3</v>
       </c>
       <c r="BZ18" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA18" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14799,11 +14831,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:BZ19)</f>
+        <f>SUM(G19:CB19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:BZ19),1)</f>
+        <f>ROUND(AVERAGE(G19:CB19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14881,11 +14913,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:BZ20)</f>
+        <f>SUM(G20:CB20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:BZ20),1)</f>
+        <f>ROUND(AVERAGE(G20:CB20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -14949,11 +14981,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:BZ21)</f>
+        <f>SUM(G21:CB21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:BZ21),1)</f>
+        <f>ROUND(AVERAGE(G21:CB21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -15008,14 +15040,14 @@
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:BZ22)</f>
+        <f>SUM(G22:CB22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:BZ22),1)</f>
+        <f>ROUND(AVERAGE(G22:CB22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -15086,6 +15118,12 @@
       <c r="BZ22" t="n">
         <v>3</v>
       </c>
+      <c r="CA22" t="n">
+        <v>2</v>
+      </c>
+      <c r="CB22" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
@@ -15103,11 +15141,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:BZ23)</f>
+        <f>SUM(G23:CB23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:BZ23),1)</f>
+        <f>ROUND(AVERAGE(G23:CB23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15216,20 +15254,20 @@
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C24" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:BZ24)</f>
+        <f>SUM(G24:CB24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:BZ24),1)</f>
+        <f>ROUND(AVERAGE(G24:CB24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15376,6 +15414,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CA24" t="n">
+        <v>2</v>
+      </c>
+      <c r="CB24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
@@ -15384,20 +15430,20 @@
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C25" s="68" t="n">
         <v>3</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:BZ25)</f>
+        <f>SUM(G25:CB25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:BZ25),1)</f>
+        <f>ROUND(AVERAGE(G25:CB25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15470,6 +15516,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CA25" t="n">
+        <v>2</v>
+      </c>
+      <c r="CB25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
@@ -15487,11 +15541,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:BZ26)</f>
+        <f>SUM(G26:CB26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:BZ26),1)</f>
+        <f>ROUND(AVERAGE(G26:CB26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15536,14 +15590,14 @@
         <v>2</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:BZ27)</f>
+        <f>SUM(G27:CB27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:BZ27),1)</f>
+        <f>ROUND(AVERAGE(G27:CB27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15667,6 +15721,12 @@
       </c>
       <c r="BZ27" t="n">
         <v>3</v>
+      </c>
+      <c r="CA27" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB27" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -15685,11 +15745,11 @@
         <v>13</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:BZ28)</f>
+        <f>SUM(G28:CB28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:BZ28),1)</f>
+        <f>ROUND(AVERAGE(G28:CB28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -15801,11 +15861,11 @@
         <v>4</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:BZ29)</f>
+        <f>SUM(G29:CB29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:BZ29),1)</f>
+        <f>ROUND(AVERAGE(G29:CB29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -15848,14 +15908,14 @@
         <v>3</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:BZ30)</f>
+        <f>SUM(G30:CB30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:BZ30),1)</f>
+        <f>ROUND(AVERAGE(G30:CB30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -15954,6 +16014,12 @@
         <v>3</v>
       </c>
       <c r="BV30" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA30" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB30" t="n">
         <v>3</v>
       </c>
     </row>
@@ -15970,14 +16036,14 @@
         <v>2</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:BZ31)</f>
+        <f>SUM(G31:CB31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:BZ31),1)</f>
+        <f>ROUND(AVERAGE(G31:CB31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -16075,6 +16141,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="CA31" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB31" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -16093,11 +16165,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:BZ32)</f>
+        <f>SUM(G32:CB32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:BZ32),1)</f>
+        <f>ROUND(AVERAGE(G32:CB32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -16166,14 +16238,14 @@
         <v>1</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:BZ33)</f>
+        <f>SUM(G33:CB33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:BZ33),1)</f>
+        <f>ROUND(AVERAGE(G33:CB33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16275,6 +16347,12 @@
       </c>
       <c r="BT33" t="n">
         <v>2</v>
+      </c>
+      <c r="CA33" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -16293,11 +16371,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:BZ34)</f>
+        <f>SUM(G34:CB34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:BZ34),1)</f>
+        <f>ROUND(AVERAGE(G34:CB34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16323,11 +16401,11 @@
         <v>25</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:BZ35)</f>
+        <f>SUM(G35:CB35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:BZ35),1)</f>
+        <f>ROUND(AVERAGE(G35:CB35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16513,11 +16591,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:BZ36)</f>
+        <f>SUM(G36:CB36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:BZ36),1)</f>
+        <f>ROUND(AVERAGE(G36:CB36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16641,11 +16719,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:BZ37)</f>
+        <f>SUM(G37:CB37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:BZ37),1)</f>
+        <f>ROUND(AVERAGE(G37:CB37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16673,11 +16751,11 @@
         <v>0</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:BZ38)</f>
+        <f>SUM(G38:CB38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:BZ38),1)</f>
+        <f>ROUND(AVERAGE(G38:CB38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16705,11 +16783,11 @@
         <v>0</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:BZ39)</f>
+        <f>SUM(G39:CB39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:BZ39),1)</f>
+        <f>ROUND(AVERAGE(G39:CB39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16737,11 +16815,11 @@
         <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:BZ40)</f>
+        <f>SUM(G40:CB40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:BZ40),1)</f>
+        <f>ROUND(AVERAGE(G40:CB40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -16769,11 +16847,11 @@
         <v>1</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:BZ41)</f>
+        <f>SUM(G41:CB41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:BZ41),1)</f>
+        <f>ROUND(AVERAGE(G41:CB41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -16798,24 +16876,24 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>samuel</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:BZ42)</f>
+        <f>SUM(G42:CB42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:BZ42),1)</f>
+        <f>ROUND(AVERAGE(G42:CB42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -16826,11 +16904,33 @@
       <c r="AN42" s="121" t="n"/>
       <c r="AO42" s="120" t="n"/>
       <c r="AP42" s="121" t="n"/>
+      <c r="BW42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY42" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ42" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA42" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB42" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -16840,14 +16940,14 @@
         <v>1</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:BZ43)</f>
+        <f>SUM(G43:CB43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:BZ43),1)</f>
+        <f>ROUND(AVERAGE(G43:CB43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -16869,33 +16969,39 @@
         </is>
       </c>
       <c r="BY43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BZ43" t="n">
         <v>3</v>
+      </c>
+      <c r="CA43" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB43" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>ggvitotmm</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:BZ44)</f>
+        <f>SUM(G44:CB44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:BZ44),1)</f>
+        <f>ROUND(AVERAGE(G44:CB44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -16906,6 +17012,16 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
+      <c r="BU44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BV44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="BW44" t="inlineStr">
         <is>
           <t>SKIP</t>
@@ -16916,34 +17032,38 @@
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BY44" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ44" t="n">
-        <v>3</v>
+      <c r="BY44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BZ44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>ggvitotmm</t>
+          <t>toxic</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:BZ45)</f>
+        <f>SUM(G45:CB45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:BZ45),1)</f>
+        <f>ROUND(AVERAGE(G45:CB45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -16954,41 +17074,11 @@
       <c r="AN45" s="121" t="n"/>
       <c r="AO45" s="120" t="n"/>
       <c r="AP45" s="121" t="n"/>
-      <c r="BU45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BZ45" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>toxic</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -17001,11 +17091,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:BZ46)</f>
+        <f>SUM(G46:CB46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:BZ46),1)</f>
+        <f>ROUND(AVERAGE(G46:CB46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17020,7 +17110,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>andrea</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -17033,11 +17123,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:BZ47)</f>
+        <f>SUM(G47:CB47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:BZ47),1)</f>
+        <f>ROUND(AVERAGE(G47:CB47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17052,7 +17142,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>andrea</t>
+          <t>piter</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -17065,11 +17155,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:BZ48)</f>
+        <f>SUM(G48:CB48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:BZ48),1)</f>
+        <f>ROUND(AVERAGE(G48:CB48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17084,7 +17174,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>piter</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -17094,14 +17184,14 @@
         <v>0</v>
       </c>
       <c r="D49" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:BZ49)</f>
+        <f>SUM(G49:CB49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:BZ49),1)</f>
+        <f>ROUND(AVERAGE(G49:CB49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>
@@ -17112,11 +17202,17 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
+      <c r="CA49" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB49" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B50" s="79" t="n">
@@ -17129,11 +17225,11 @@
         <v>0</v>
       </c>
       <c r="E50" s="68">
-        <f>SUM(G50:BZ50)</f>
+        <f>SUM(G50:CB50)</f>
         <v/>
       </c>
       <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:BZ50),1)</f>
+        <f>ROUND(AVERAGE(G50:CB50),1)</f>
         <v/>
       </c>
       <c r="AI50" s="120" t="n"/>
@@ -17144,6 +17240,38 @@
       <c r="AN50" s="121" t="n"/>
       <c r="AO50" s="120" t="n"/>
       <c r="AP50" s="121" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>satana03</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="68">
+        <f>SUM(G51:CB51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="68">
+        <f>ROUND(AVERAGE(G51:CB51),1)</f>
+        <v/>
+      </c>
+      <c r="AI51" s="120" t="n"/>
+      <c r="AJ51" s="121" t="n"/>
+      <c r="AK51" s="120" t="n"/>
+      <c r="AL51" s="121" t="n"/>
+      <c r="AM51" s="120" t="n"/>
+      <c r="AN51" s="121" t="n"/>
+      <c r="AO51" s="120" t="n"/>
+      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-22
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI51"/>
+  <dimension ref="A1:CI49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13181,12 +13181,12 @@
       </c>
       <c r="CC1" s="109" t="inlineStr">
         <is>
-          <t>Colonna81</t>
+          <t>WAR-38 (1)</t>
         </is>
       </c>
       <c r="CD1" s="109" t="inlineStr">
         <is>
-          <t>Colonna82</t>
+          <t>WAR-38 (2)</t>
         </is>
       </c>
       <c r="CE1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:CB2)</f>
+        <f>SUM(G2:CD2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:CB2),1)</f>
+        <f>ROUND(AVERAGE(G2:CD2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:CB3)</f>
+        <f>SUM(G3:CD3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:CB3),1)</f>
+        <f>ROUND(AVERAGE(G3:CD3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13308,14 +13308,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:CB4)</f>
+        <f>SUM(G4:CD4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:CB4),1)</f>
+        <f>ROUND(AVERAGE(G4:CD4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13410,6 +13410,12 @@
         <v>3</v>
       </c>
       <c r="CB4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13426,14 +13432,14 @@
         <v>3</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:CB5)</f>
+        <f>SUM(G5:CD5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:CB5),1)</f>
+        <f>ROUND(AVERAGE(G5:CD5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13495,6 +13501,12 @@
       </c>
       <c r="CB5" t="n">
         <v>3</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -13510,14 +13522,14 @@
         <v>6</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:CB6)</f>
+        <f>SUM(G6:CD6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:CB6),1)</f>
+        <f>ROUND(AVERAGE(G6:CD6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13707,6 +13719,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="CC6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -13722,14 +13740,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:CB7)</f>
+        <f>SUM(G7:CD7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:CB7),1)</f>
+        <f>ROUND(AVERAGE(G7:CD7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13802,6 +13820,12 @@
       <c r="CB7" t="n">
         <v>3</v>
       </c>
+      <c r="CC7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
@@ -13819,11 +13843,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:CB8)</f>
+        <f>SUM(G8:CD8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:CB8),1)</f>
+        <f>ROUND(AVERAGE(G8:CD8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13850,14 +13874,14 @@
         <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:CB9)</f>
+        <f>SUM(G9:CD9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:CB9),1)</f>
+        <f>ROUND(AVERAGE(G9:CD9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13947,6 +13971,12 @@
       </c>
       <c r="BZ9" t="n">
         <v>2</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -13965,11 +13995,11 @@
         <v>19</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:CB10)</f>
+        <f>SUM(G10:CD10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:CB10),1)</f>
+        <f>ROUND(AVERAGE(G10:CD10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14123,11 +14153,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:CB11)</f>
+        <f>SUM(G11:CD11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:CB11),1)</f>
+        <f>ROUND(AVERAGE(G11:CD11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14158,14 +14188,14 @@
         <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:CB12)</f>
+        <f>SUM(G12:CD12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:CB12),1)</f>
+        <f>ROUND(AVERAGE(G12:CD12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14203,6 +14233,12 @@
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="CC12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -14221,11 +14257,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:CB13)</f>
+        <f>SUM(G13:CD13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:CB13),1)</f>
+        <f>ROUND(AVERAGE(G13:CD13),1)</f>
         <v/>
       </c>
     </row>
@@ -14242,14 +14278,14 @@
         <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:CB14)</f>
+        <f>SUM(G14:CD14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:CB14),1)</f>
+        <f>ROUND(AVERAGE(G14:CD14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14350,6 +14386,12 @@
       <c r="BZ14" t="n">
         <v>1</v>
       </c>
+      <c r="CC14" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
@@ -14367,11 +14409,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:CB15)</f>
+        <f>SUM(G15:CD15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:CB15),1)</f>
+        <f>ROUND(AVERAGE(G15:CD15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14397,11 +14439,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:CB16)</f>
+        <f>SUM(G16:CD16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:CB16),1)</f>
+        <f>ROUND(AVERAGE(G16:CD16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14527,11 +14569,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:CB17)</f>
+        <f>SUM(G17:CD17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:CB17),1)</f>
+        <f>ROUND(AVERAGE(G17:CD17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14700,14 +14742,14 @@
         <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:CB18)</f>
+        <f>SUM(G18:CD18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:CB18),1)</f>
+        <f>ROUND(AVERAGE(G18:CD18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14812,6 +14854,12 @@
         <v>3</v>
       </c>
       <c r="CB18" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC18" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14831,11 +14879,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:CB19)</f>
+        <f>SUM(G19:CD19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:CB19),1)</f>
+        <f>ROUND(AVERAGE(G19:CD19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14913,11 +14961,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:CB20)</f>
+        <f>SUM(G20:CD20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:CB20),1)</f>
+        <f>ROUND(AVERAGE(G20:CD20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -14981,11 +15029,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:CB21)</f>
+        <f>SUM(G21:CD21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:CB21),1)</f>
+        <f>ROUND(AVERAGE(G21:CD21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -15043,11 +15091,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:CB22)</f>
+        <f>SUM(G22:CD22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:CB22),1)</f>
+        <f>ROUND(AVERAGE(G22:CD22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -15138,14 +15186,14 @@
         <v>0</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:CB23)</f>
+        <f>SUM(G23:CD23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:CB23),1)</f>
+        <f>ROUND(AVERAGE(G23:CD23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15246,6 +15294,12 @@
       <c r="BT23" t="n">
         <v>3</v>
       </c>
+      <c r="CC23" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD23" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
@@ -15254,20 +15308,20 @@
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C24" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:CB24)</f>
+        <f>SUM(G24:CD24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:CB24),1)</f>
+        <f>ROUND(AVERAGE(G24:CD24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15422,6 +15476,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CC24" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
@@ -15430,20 +15492,20 @@
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:CB25)</f>
+        <f>SUM(G25:CD25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:CB25),1)</f>
+        <f>ROUND(AVERAGE(G25:CD25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15524,6 +15586,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CC25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
@@ -15541,11 +15613,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:CB26)</f>
+        <f>SUM(G26:CD26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:CB26),1)</f>
+        <f>ROUND(AVERAGE(G26:CD26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15590,14 +15662,14 @@
         <v>2</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:CB27)</f>
+        <f>SUM(G27:CD27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:CB27),1)</f>
+        <f>ROUND(AVERAGE(G27:CD27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15727,6 +15799,12 @@
       </c>
       <c r="CB27" t="n">
         <v>2</v>
+      </c>
+      <c r="CC27" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD27" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -15745,11 +15823,11 @@
         <v>13</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:CB28)</f>
+        <f>SUM(G28:CD28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:CB28),1)</f>
+        <f>ROUND(AVERAGE(G28:CD28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -15858,14 +15936,14 @@
         <v>0</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:CB29)</f>
+        <f>SUM(G29:CD29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:CB29),1)</f>
+        <f>ROUND(AVERAGE(G29:CD29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -15892,6 +15970,12 @@
         <v>3</v>
       </c>
       <c r="BV29" t="n">
+        <v>2</v>
+      </c>
+      <c r="CC29" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15902,20 +15986,20 @@
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:CB30)</f>
+        <f>SUM(G30:CD30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:CB30),1)</f>
+        <f>ROUND(AVERAGE(G30:CD30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -16021,6 +16105,16 @@
       </c>
       <c r="CB30" t="n">
         <v>3</v>
+      </c>
+      <c r="CC30" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD30" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -16039,11 +16133,11 @@
         <v>14</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:CB31)</f>
+        <f>SUM(G31:CD31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:CB31),1)</f>
+        <f>ROUND(AVERAGE(G31:CD31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -16165,11 +16259,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:CB32)</f>
+        <f>SUM(G32:CD32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:CB32),1)</f>
+        <f>ROUND(AVERAGE(G32:CD32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -16241,11 +16335,11 @@
         <v>16</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:CB33)</f>
+        <f>SUM(G33:CD33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:CB33),1)</f>
+        <f>ROUND(AVERAGE(G33:CD33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16371,11 +16465,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:CB34)</f>
+        <f>SUM(G34:CD34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:CB34),1)</f>
+        <f>ROUND(AVERAGE(G34:CD34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16392,20 +16486,20 @@
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:CB35)</f>
+        <f>SUM(G35:CD35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:CB35),1)</f>
+        <f>ROUND(AVERAGE(G35:CD35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16573,6 +16667,16 @@
       </c>
       <c r="BV35" t="n">
         <v>1</v>
+      </c>
+      <c r="CC35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -16591,11 +16695,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:CB36)</f>
+        <f>SUM(G36:CD36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:CB36),1)</f>
+        <f>ROUND(AVERAGE(G36:CD36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16719,11 +16823,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:CB37)</f>
+        <f>SUM(G37:CD37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:CB37),1)</f>
+        <f>ROUND(AVERAGE(G37:CD37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16751,11 +16855,11 @@
         <v>0</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:CB38)</f>
+        <f>SUM(G38:CD38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:CB38),1)</f>
+        <f>ROUND(AVERAGE(G38:CD38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16770,7 +16874,7 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>krigohard</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
@@ -16780,14 +16884,14 @@
         <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:CB39)</f>
+        <f>SUM(G39:CD39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:CB39),1)</f>
+        <f>ROUND(AVERAGE(G39:CD39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16798,28 +16902,34 @@
       <c r="AN39" s="121" t="n"/>
       <c r="AO39" s="120" t="n"/>
       <c r="AP39" s="121" t="n"/>
+      <c r="CC39" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD39" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Steninja:)</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:CB40)</f>
+        <f>SUM(G40:CD40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:CB40),1)</f>
+        <f>ROUND(AVERAGE(G40:CD40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -16830,28 +16940,38 @@
       <c r="AN40" s="121" t="n"/>
       <c r="AO40" s="120" t="n"/>
       <c r="AP40" s="121" t="n"/>
+      <c r="BU40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BV40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>IMnotReal</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:CB41)</f>
+        <f>SUM(G41:CD41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:CB41),1)</f>
+        <f>ROUND(AVERAGE(G41:CD41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -16862,12 +16982,34 @@
       <c r="AN41" s="121" t="n"/>
       <c r="AO41" s="120" t="n"/>
       <c r="AP41" s="121" t="n"/>
-      <c r="BU41" t="inlineStr">
+      <c r="BW41" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BV41" t="inlineStr">
+      <c r="BX41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY41" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ41" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA41" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB41" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD41" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16876,7 +17018,7 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
@@ -16886,14 +17028,14 @@
         <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:CB42)</f>
+        <f>SUM(G42:CD42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:CB42),1)</f>
+        <f>ROUND(AVERAGE(G42:CD42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -16915,22 +17057,28 @@
         </is>
       </c>
       <c r="BY42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BZ42" t="n">
         <v>3</v>
       </c>
       <c r="CA42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CB42" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="CC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD42" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -16940,14 +17088,14 @@
         <v>1</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:CB43)</f>
+        <f>SUM(G43:CD43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:CB43),1)</f>
+        <f>ROUND(AVERAGE(G43:CD43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -16958,50 +17106,38 @@
       <c r="AN43" s="121" t="n"/>
       <c r="AO43" s="120" t="n"/>
       <c r="AP43" s="121" t="n"/>
-      <c r="BW43" t="inlineStr">
+      <c r="CC43" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BX43" t="inlineStr">
+      <c r="CD43" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="BY43" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ43" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA43" t="n">
-        <v>1</v>
-      </c>
-      <c r="CB43" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>ggvitotmm</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:CB44)</f>
+        <f>SUM(G44:CD44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:CB44),1)</f>
+        <f>ROUND(AVERAGE(G44:CD44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -17012,41 +17148,23 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
-      <c r="BU44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BZ44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="CA44" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB44" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC44" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD44" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>toxic</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -17059,11 +17177,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:CB45)</f>
+        <f>SUM(G45:CD45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:CB45),1)</f>
+        <f>ROUND(AVERAGE(G45:CD45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -17078,7 +17196,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>satana03</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -17091,11 +17209,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:CB46)</f>
+        <f>SUM(G46:CD46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:CB46),1)</f>
+        <f>ROUND(AVERAGE(G46:CD46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17110,7 +17228,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>andrea</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -17123,11 +17241,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:CB47)</f>
+        <f>SUM(G47:CD47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:CB47),1)</f>
+        <f>ROUND(AVERAGE(G47:CD47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17142,7 +17260,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>piter</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -17155,11 +17273,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:CB48)</f>
+        <f>SUM(G48:CD48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:CB48),1)</f>
+        <f>ROUND(AVERAGE(G48:CD48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17174,7 +17292,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>Diego229</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -17184,14 +17302,14 @@
         <v>0</v>
       </c>
       <c r="D49" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:CB49)</f>
+        <f>SUM(G49:CD49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:CB49),1)</f>
+        <f>ROUND(AVERAGE(G49:CD49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>
@@ -17202,76 +17320,6 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
-      <c r="CA49" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB49" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>Ema alba003</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:CB50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:CB50),1)</f>
-        <v/>
-      </c>
-      <c r="AI50" s="120" t="n"/>
-      <c r="AJ50" s="121" t="n"/>
-      <c r="AK50" s="120" t="n"/>
-      <c r="AL50" s="121" t="n"/>
-      <c r="AM50" s="120" t="n"/>
-      <c r="AN50" s="121" t="n"/>
-      <c r="AO50" s="120" t="n"/>
-      <c r="AP50" s="121" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="79" t="inlineStr">
-        <is>
-          <t>satana03</t>
-        </is>
-      </c>
-      <c r="B51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="68">
-        <f>SUM(G51:CB51)</f>
-        <v/>
-      </c>
-      <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:CB51),1)</f>
-        <v/>
-      </c>
-      <c r="AI51" s="120" t="n"/>
-      <c r="AJ51" s="121" t="n"/>
-      <c r="AK51" s="120" t="n"/>
-      <c r="AL51" s="121" t="n"/>
-      <c r="AM51" s="120" t="n"/>
-      <c r="AN51" s="121" t="n"/>
-      <c r="AO51" s="120" t="n"/>
-      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-25
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -13191,12 +13191,12 @@
       </c>
       <c r="CE1" s="109" t="inlineStr">
         <is>
-          <t>Colonna83</t>
+          <t>WAR-39 (1)</t>
         </is>
       </c>
       <c r="CF1" s="109" t="inlineStr">
         <is>
-          <t>Colonna84</t>
+          <t>WAR-39 (2)</t>
         </is>
       </c>
       <c r="CG1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:CD2)</f>
+        <f>SUM(G2:CF2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:CD2),1)</f>
+        <f>ROUND(AVERAGE(G2:CF2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:CD3)</f>
+        <f>SUM(G3:CF3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:CD3),1)</f>
+        <f>ROUND(AVERAGE(G3:CF3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13308,14 +13308,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:CD4)</f>
+        <f>SUM(G4:CF4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:CD4),1)</f>
+        <f>ROUND(AVERAGE(G4:CF4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13416,6 +13416,12 @@
         <v>3</v>
       </c>
       <c r="CD4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13435,11 +13441,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:CD5)</f>
+        <f>SUM(G5:CF5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:CD5),1)</f>
+        <f>ROUND(AVERAGE(G5:CF5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13516,20 +13522,20 @@
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="68" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:CD6)</f>
+        <f>SUM(G6:CF6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:CD6),1)</f>
+        <f>ROUND(AVERAGE(G6:CF6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13725,6 +13731,14 @@
       </c>
       <c r="CD6" t="n">
         <v>3</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -13740,14 +13754,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:CD7)</f>
+        <f>SUM(G7:CF7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:CD7),1)</f>
+        <f>ROUND(AVERAGE(G7:CF7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13826,6 +13840,12 @@
       <c r="CD7" t="n">
         <v>3</v>
       </c>
+      <c r="CE7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
@@ -13843,11 +13863,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:CD8)</f>
+        <f>SUM(G8:CF8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:CD8),1)</f>
+        <f>ROUND(AVERAGE(G8:CF8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13877,11 +13897,11 @@
         <v>15</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:CD9)</f>
+        <f>SUM(G9:CF9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:CD9),1)</f>
+        <f>ROUND(AVERAGE(G9:CF9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13986,20 +14006,20 @@
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:CD10)</f>
+        <f>SUM(G10:CF10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:CD10),1)</f>
+        <f>ROUND(AVERAGE(G10:CF10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14136,6 +14156,16 @@
       <c r="BV10" t="n">
         <v>2</v>
       </c>
+      <c r="CE10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
@@ -14153,11 +14183,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:CD11)</f>
+        <f>SUM(G11:CF11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:CD11),1)</f>
+        <f>ROUND(AVERAGE(G11:CF11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14191,11 +14221,11 @@
         <v>6</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:CD12)</f>
+        <f>SUM(G12:CF12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:CD12),1)</f>
+        <f>ROUND(AVERAGE(G12:CF12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14257,11 +14287,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:CD13)</f>
+        <f>SUM(G13:CF13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:CD13),1)</f>
+        <f>ROUND(AVERAGE(G13:CF13),1)</f>
         <v/>
       </c>
     </row>
@@ -14272,20 +14302,20 @@
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="68" t="n">
         <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:CD14)</f>
+        <f>SUM(G14:CF14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:CD14),1)</f>
+        <f>ROUND(AVERAGE(G14:CF14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14392,6 +14422,14 @@
       <c r="CD14" t="n">
         <v>3</v>
       </c>
+      <c r="CE14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
@@ -14409,11 +14447,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:CD15)</f>
+        <f>SUM(G15:CF15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:CD15),1)</f>
+        <f>ROUND(AVERAGE(G15:CF15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14439,11 +14477,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:CD16)</f>
+        <f>SUM(G16:CF16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:CD16),1)</f>
+        <f>ROUND(AVERAGE(G16:CF16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14569,11 +14607,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:CD17)</f>
+        <f>SUM(G17:CF17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:CD17),1)</f>
+        <f>ROUND(AVERAGE(G17:CF17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14742,14 +14780,14 @@
         <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:CD18)</f>
+        <f>SUM(G18:CF18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:CD18),1)</f>
+        <f>ROUND(AVERAGE(G18:CF18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14861,6 +14899,12 @@
       </c>
       <c r="CD18" t="n">
         <v>3</v>
+      </c>
+      <c r="CE18" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF18" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -14879,11 +14923,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:CD19)</f>
+        <f>SUM(G19:CF19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:CD19),1)</f>
+        <f>ROUND(AVERAGE(G19:CF19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -14961,11 +15005,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:CD20)</f>
+        <f>SUM(G20:CF20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:CD20),1)</f>
+        <f>ROUND(AVERAGE(G20:CF20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -15029,11 +15073,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:CD21)</f>
+        <f>SUM(G21:CF21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:CD21),1)</f>
+        <f>ROUND(AVERAGE(G21:CF21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -15091,11 +15135,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:CD22)</f>
+        <f>SUM(G22:CF22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:CD22),1)</f>
+        <f>ROUND(AVERAGE(G22:CF22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -15180,20 +15224,20 @@
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:CD23)</f>
+        <f>SUM(G23:CF23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:CD23),1)</f>
+        <f>ROUND(AVERAGE(G23:CF23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15300,6 +15344,16 @@
       <c r="CD23" t="n">
         <v>3</v>
       </c>
+      <c r="CE23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
@@ -15308,20 +15362,20 @@
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:CD24)</f>
+        <f>SUM(G24:CF24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:CD24),1)</f>
+        <f>ROUND(AVERAGE(G24:CF24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15484,6 +15538,14 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CE24" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
@@ -15492,20 +15554,20 @@
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:CD25)</f>
+        <f>SUM(G25:CF25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:CD25),1)</f>
+        <f>ROUND(AVERAGE(G25:CF25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15596,6 +15658,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CE25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF25" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
@@ -15613,11 +15685,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:CD26)</f>
+        <f>SUM(G26:CF26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:CD26),1)</f>
+        <f>ROUND(AVERAGE(G26:CF26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15662,14 +15734,14 @@
         <v>2</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:CD27)</f>
+        <f>SUM(G27:CF27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:CD27),1)</f>
+        <f>ROUND(AVERAGE(G27:CF27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15805,6 +15877,12 @@
       </c>
       <c r="CD27" t="n">
         <v>3</v>
+      </c>
+      <c r="CE27" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF27" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -15823,11 +15901,11 @@
         <v>13</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:CD28)</f>
+        <f>SUM(G28:CF28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:CD28),1)</f>
+        <f>ROUND(AVERAGE(G28:CF28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -15939,11 +16017,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:CD29)</f>
+        <f>SUM(G29:CF29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:CD29),1)</f>
+        <f>ROUND(AVERAGE(G29:CF29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -15995,11 +16073,11 @@
         <v>16</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:CD30)</f>
+        <f>SUM(G30:CF30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:CD30),1)</f>
+        <f>ROUND(AVERAGE(G30:CF30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -16133,11 +16211,11 @@
         <v>14</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:CD31)</f>
+        <f>SUM(G31:CF31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:CD31),1)</f>
+        <f>ROUND(AVERAGE(G31:CF31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -16259,11 +16337,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:CD32)</f>
+        <f>SUM(G32:CF32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:CD32),1)</f>
+        <f>ROUND(AVERAGE(G32:CF32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -16335,11 +16413,11 @@
         <v>16</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:CD33)</f>
+        <f>SUM(G33:CF33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:CD33),1)</f>
+        <f>ROUND(AVERAGE(G33:CF33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16465,11 +16543,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:CD34)</f>
+        <f>SUM(G34:CF34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:CD34),1)</f>
+        <f>ROUND(AVERAGE(G34:CF34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16486,20 +16564,20 @@
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:CD35)</f>
+        <f>SUM(G35:CF35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:CD35),1)</f>
+        <f>ROUND(AVERAGE(G35:CF35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16674,6 +16752,16 @@
         </is>
       </c>
       <c r="CD35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF35" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16695,11 +16783,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:CD36)</f>
+        <f>SUM(G36:CF36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:CD36),1)</f>
+        <f>ROUND(AVERAGE(G36:CF36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16823,11 +16911,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:CD37)</f>
+        <f>SUM(G37:CF37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:CD37),1)</f>
+        <f>ROUND(AVERAGE(G37:CF37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16846,20 +16934,20 @@
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:CD38)</f>
+        <f>SUM(G38:CF38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:CD38),1)</f>
+        <f>ROUND(AVERAGE(G38:CF38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16870,6 +16958,16 @@
       <c r="AN38" s="121" t="n"/>
       <c r="AO38" s="120" t="n"/>
       <c r="AP38" s="121" t="n"/>
+      <c r="CE38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
@@ -16887,11 +16985,11 @@
         <v>1</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:CD39)</f>
+        <f>SUM(G39:CF39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:CD39),1)</f>
+        <f>ROUND(AVERAGE(G39:CF39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16925,11 +17023,11 @@
         <v>1</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:CD40)</f>
+        <f>SUM(G40:CF40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:CD40),1)</f>
+        <f>ROUND(AVERAGE(G40:CF40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -16958,20 +17056,20 @@
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:CD41)</f>
+        <f>SUM(G41:CF41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:CD41),1)</f>
+        <f>ROUND(AVERAGE(G41:CF41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -17014,6 +17112,16 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CE41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
@@ -17028,14 +17136,14 @@
         <v>1</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:CD42)</f>
+        <f>SUM(G42:CF42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:CD42),1)</f>
+        <f>ROUND(AVERAGE(G42:CF42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -17074,6 +17182,12 @@
       <c r="CD42" t="n">
         <v>1</v>
       </c>
+      <c r="CE42" t="n">
+        <v>2</v>
+      </c>
+      <c r="CF42" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
@@ -17091,11 +17205,11 @@
         <v>1</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:CD43)</f>
+        <f>SUM(G43:CF43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:CD43),1)</f>
+        <f>ROUND(AVERAGE(G43:CF43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -17130,14 +17244,14 @@
         <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:CD44)</f>
+        <f>SUM(G44:CF44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:CD44),1)</f>
+        <f>ROUND(AVERAGE(G44:CF44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -17160,6 +17274,12 @@
       <c r="CD44" t="n">
         <v>1</v>
       </c>
+      <c r="CE44" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF44" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
@@ -17177,11 +17297,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:CD45)</f>
+        <f>SUM(G45:CF45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:CD45),1)</f>
+        <f>ROUND(AVERAGE(G45:CF45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -17209,11 +17329,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:CD46)</f>
+        <f>SUM(G46:CF46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:CD46),1)</f>
+        <f>ROUND(AVERAGE(G46:CF46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17241,11 +17361,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:CD47)</f>
+        <f>SUM(G47:CF47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:CD47),1)</f>
+        <f>ROUND(AVERAGE(G47:CF47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17273,11 +17393,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:CD48)</f>
+        <f>SUM(G48:CF48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:CD48),1)</f>
+        <f>ROUND(AVERAGE(G48:CF48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17305,11 +17425,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:CD49)</f>
+        <f>SUM(G49:CF49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:CD49),1)</f>
+        <f>ROUND(AVERAGE(G49:CF49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>

</xml_diff>

<commit_message>
Update WAR data - 2026-04-28
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI49"/>
+  <dimension ref="A1:CI50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13201,12 +13201,12 @@
       </c>
       <c r="CG1" s="109" t="inlineStr">
         <is>
-          <t>Colonna85</t>
+          <t>WAR-40 (1)</t>
         </is>
       </c>
       <c r="CH1" s="109" t="inlineStr">
         <is>
-          <t>Colonna86</t>
+          <t>WAR-40 (2)</t>
         </is>
       </c>
       <c r="CI1" s="109" t="inlineStr">
@@ -13231,11 +13231,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:CF2)</f>
+        <f>SUM(G2:CH2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:CF2),1)</f>
+        <f>ROUND(AVERAGE(G2:CH2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13255,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:CF3)</f>
+        <f>SUM(G3:CH3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:CF3),1)</f>
+        <f>ROUND(AVERAGE(G3:CH3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13311,11 +13311,11 @@
         <v>17</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:CF4)</f>
+        <f>SUM(G4:CH4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:CF4),1)</f>
+        <f>ROUND(AVERAGE(G4:CH4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13441,11 +13441,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:CF5)</f>
+        <f>SUM(G5:CH5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:CF5),1)</f>
+        <f>ROUND(AVERAGE(G5:CH5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13531,11 +13531,11 @@
         <v>27</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:CF6)</f>
+        <f>SUM(G6:CH6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:CF6),1)</f>
+        <f>ROUND(AVERAGE(G6:CH6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13757,11 +13757,11 @@
         <v>13</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:CF7)</f>
+        <f>SUM(G7:CH7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:CF7),1)</f>
+        <f>ROUND(AVERAGE(G7:CH7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13863,11 +13863,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:CF8)</f>
+        <f>SUM(G8:CH8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:CF8),1)</f>
+        <f>ROUND(AVERAGE(G8:CH8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13897,11 +13897,11 @@
         <v>15</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:CF9)</f>
+        <f>SUM(G9:CH9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:CF9),1)</f>
+        <f>ROUND(AVERAGE(G9:CH9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -14015,11 +14015,11 @@
         <v>20</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:CF10)</f>
+        <f>SUM(G10:CH10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:CF10),1)</f>
+        <f>ROUND(AVERAGE(G10:CH10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14183,11 +14183,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:CF11)</f>
+        <f>SUM(G11:CH11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:CF11),1)</f>
+        <f>ROUND(AVERAGE(G11:CH11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14221,11 +14221,11 @@
         <v>6</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:CF12)</f>
+        <f>SUM(G12:CH12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:CF12),1)</f>
+        <f>ROUND(AVERAGE(G12:CH12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14287,11 +14287,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:CF13)</f>
+        <f>SUM(G13:CH13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:CF13),1)</f>
+        <f>ROUND(AVERAGE(G13:CH13),1)</f>
         <v/>
       </c>
     </row>
@@ -14311,11 +14311,11 @@
         <v>15</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:CF14)</f>
+        <f>SUM(G14:CH14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:CF14),1)</f>
+        <f>ROUND(AVERAGE(G14:CH14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14447,11 +14447,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:CF15)</f>
+        <f>SUM(G15:CH15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:CF15),1)</f>
+        <f>ROUND(AVERAGE(G15:CH15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14477,11 +14477,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:CF16)</f>
+        <f>SUM(G16:CH16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:CF16),1)</f>
+        <f>ROUND(AVERAGE(G16:CH16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14607,11 +14607,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:CF17)</f>
+        <f>SUM(G17:CH17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:CF17),1)</f>
+        <f>ROUND(AVERAGE(G17:CH17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14783,11 +14783,11 @@
         <v>18</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:CF18)</f>
+        <f>SUM(G18:CH18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:CF18),1)</f>
+        <f>ROUND(AVERAGE(G18:CH18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14923,11 +14923,11 @@
         <v>8</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:CF19)</f>
+        <f>SUM(G19:CH19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:CF19),1)</f>
+        <f>ROUND(AVERAGE(G19:CH19),1)</f>
         <v/>
       </c>
       <c r="G19" s="79" t="n">
@@ -15005,11 +15005,11 @@
         <v>6</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:CF20)</f>
+        <f>SUM(G20:CH20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:CF20),1)</f>
+        <f>ROUND(AVERAGE(G20:CH20),1)</f>
         <v/>
       </c>
       <c r="AI20" s="68" t="n"/>
@@ -15073,11 +15073,11 @@
         <v>5</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:CF21)</f>
+        <f>SUM(G21:CH21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:CF21),1)</f>
+        <f>ROUND(AVERAGE(G21:CH21),1)</f>
         <v/>
       </c>
       <c r="AE21" s="79" t="n">
@@ -15135,11 +15135,11 @@
         <v>10</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:CF22)</f>
+        <f>SUM(G22:CH22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:CF22),1)</f>
+        <f>ROUND(AVERAGE(G22:CH22),1)</f>
         <v/>
       </c>
       <c r="AM22" s="68" t="n"/>
@@ -15233,11 +15233,11 @@
         <v>17</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:CF23)</f>
+        <f>SUM(G23:CH23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:CF23),1)</f>
+        <f>ROUND(AVERAGE(G23:CH23),1)</f>
         <v/>
       </c>
       <c r="I23" s="79" t="n">
@@ -15371,11 +15371,11 @@
         <v>22</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:CF24)</f>
+        <f>SUM(G24:CH24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:CF24),1)</f>
+        <f>ROUND(AVERAGE(G24:CH24),1)</f>
         <v/>
       </c>
       <c r="G24" s="79" t="n">
@@ -15563,11 +15563,11 @@
         <v>10</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:CF25)</f>
+        <f>SUM(G25:CH25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:CF25),1)</f>
+        <f>ROUND(AVERAGE(G25:CH25),1)</f>
         <v/>
       </c>
       <c r="AM25" s="68" t="n"/>
@@ -15685,11 +15685,11 @@
         <v>4</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:CF26)</f>
+        <f>SUM(G26:CH26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:CF26),1)</f>
+        <f>ROUND(AVERAGE(G26:CH26),1)</f>
         <v/>
       </c>
       <c r="AM26" s="120" t="n">
@@ -15737,11 +15737,11 @@
         <v>22</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:CF27)</f>
+        <f>SUM(G27:CH27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:CF27),1)</f>
+        <f>ROUND(AVERAGE(G27:CH27),1)</f>
         <v/>
       </c>
       <c r="G27" s="79" t="n">
@@ -15901,11 +15901,11 @@
         <v>13</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:CF28)</f>
+        <f>SUM(G28:CH28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:CF28),1)</f>
+        <f>ROUND(AVERAGE(G28:CH28),1)</f>
         <v/>
       </c>
       <c r="I28" s="79" t="n">
@@ -16017,11 +16017,11 @@
         <v>5</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:CF29)</f>
+        <f>SUM(G29:CH29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:CF29),1)</f>
+        <f>ROUND(AVERAGE(G29:CH29),1)</f>
         <v/>
       </c>
       <c r="Y29" s="79" t="n">
@@ -16073,11 +16073,11 @@
         <v>16</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:CF30)</f>
+        <f>SUM(G30:CH30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:CF30),1)</f>
+        <f>ROUND(AVERAGE(G30:CH30),1)</f>
         <v/>
       </c>
       <c r="S30" s="79" t="n">
@@ -16211,11 +16211,11 @@
         <v>14</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:CF31)</f>
+        <f>SUM(G31:CH31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:CF31),1)</f>
+        <f>ROUND(AVERAGE(G31:CH31),1)</f>
         <v/>
       </c>
       <c r="I31" s="79" t="inlineStr">
@@ -16337,11 +16337,11 @@
         <v>8</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:CF32)</f>
+        <f>SUM(G32:CH32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:CF32),1)</f>
+        <f>ROUND(AVERAGE(G32:CH32),1)</f>
         <v/>
       </c>
       <c r="G32" s="79" t="n">
@@ -16413,11 +16413,11 @@
         <v>16</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:CF33)</f>
+        <f>SUM(G33:CH33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:CF33),1)</f>
+        <f>ROUND(AVERAGE(G33:CH33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16543,11 +16543,11 @@
         <v>1</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:CF34)</f>
+        <f>SUM(G34:CH34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:CF34),1)</f>
+        <f>ROUND(AVERAGE(G34:CH34),1)</f>
         <v/>
       </c>
       <c r="AS34" s="120" t="n">
@@ -16573,11 +16573,11 @@
         <v>27</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:CF35)</f>
+        <f>SUM(G35:CH35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:CF35),1)</f>
+        <f>ROUND(AVERAGE(G35:CH35),1)</f>
         <v/>
       </c>
       <c r="G35" s="79" t="n">
@@ -16783,11 +16783,11 @@
         <v>15</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:CF36)</f>
+        <f>SUM(G36:CH36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:CF36),1)</f>
+        <f>ROUND(AVERAGE(G36:CH36),1)</f>
         <v/>
       </c>
       <c r="U36" s="79" t="n">
@@ -16911,11 +16911,11 @@
         <v>0</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:CF37)</f>
+        <f>SUM(G37:CH37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:CF37),1)</f>
+        <f>ROUND(AVERAGE(G37:CH37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16943,11 +16943,11 @@
         <v>1</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:CF38)</f>
+        <f>SUM(G38:CH38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:CF38),1)</f>
+        <f>ROUND(AVERAGE(G38:CH38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16972,24 +16972,24 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>matty</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C39" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:CF39)</f>
+        <f>SUM(G39:CH39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:CF39),1)</f>
+        <f>ROUND(AVERAGE(G39:CH39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -17000,17 +17000,45 @@
       <c r="AN39" s="121" t="n"/>
       <c r="AO39" s="120" t="n"/>
       <c r="AP39" s="121" t="n"/>
+      <c r="BW39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY39" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ39" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA39" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB39" t="n">
+        <v>1</v>
+      </c>
       <c r="CC39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="CD39" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE39" t="n">
+        <v>2</v>
+      </c>
+      <c r="CF39" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>Steninja:)</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
@@ -17023,11 +17051,11 @@
         <v>1</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:CF40)</f>
+        <f>SUM(G40:CH40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:CF40),1)</f>
+        <f>ROUND(AVERAGE(G40:CH40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -17038,12 +17066,12 @@
       <c r="AN40" s="121" t="n"/>
       <c r="AO40" s="120" t="n"/>
       <c r="AP40" s="121" t="n"/>
-      <c r="BU40" t="inlineStr">
+      <c r="CC40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BV40" t="inlineStr">
+      <c r="CD40" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -17052,24 +17080,24 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>IMnotReal</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:CF41)</f>
+        <f>SUM(G41:CH41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:CF41),1)</f>
+        <f>ROUND(AVERAGE(G41:CH41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -17080,70 +17108,46 @@
       <c r="AN41" s="121" t="n"/>
       <c r="AO41" s="120" t="n"/>
       <c r="AP41" s="121" t="n"/>
-      <c r="BW41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY41" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ41" t="n">
-        <v>3</v>
-      </c>
       <c r="CA41" t="n">
         <v>3</v>
       </c>
       <c r="CB41" t="n">
         <v>3</v>
       </c>
-      <c r="CC41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="CC41" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE41" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF41" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:CF42)</f>
+        <f>SUM(G42:CH42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:CF42),1)</f>
+        <f>ROUND(AVERAGE(G42:CH42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -17154,62 +17158,28 @@
       <c r="AN42" s="121" t="n"/>
       <c r="AO42" s="120" t="n"/>
       <c r="AP42" s="121" t="n"/>
-      <c r="BW42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY42" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ42" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA42" t="n">
-        <v>1</v>
-      </c>
-      <c r="CB42" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC42" t="n">
-        <v>0</v>
-      </c>
-      <c r="CD42" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE42" t="n">
-        <v>2</v>
-      </c>
-      <c r="CF42" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C43" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:CF43)</f>
+        <f>SUM(G43:CH43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:CF43),1)</f>
+        <f>ROUND(AVERAGE(G43:CH43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -17220,21 +17190,11 @@
       <c r="AN43" s="121" t="n"/>
       <c r="AO43" s="120" t="n"/>
       <c r="AP43" s="121" t="n"/>
-      <c r="CC43" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD43" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -17244,14 +17204,14 @@
         <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:CF44)</f>
+        <f>SUM(G44:CH44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:CF44),1)</f>
+        <f>ROUND(AVERAGE(G44:CH44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -17262,29 +17222,11 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
-      <c r="CA44" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB44" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC44" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD44" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE44" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF44" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>Dade_Aca_03</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -17297,11 +17239,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:CF45)</f>
+        <f>SUM(G45:CH45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:CF45),1)</f>
+        <f>ROUND(AVERAGE(G45:CH45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -17316,7 +17258,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>satana03</t>
+          <t>AnT0x</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -17329,11 +17271,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:CF46)</f>
+        <f>SUM(G46:CH46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:CF46),1)</f>
+        <f>ROUND(AVERAGE(G46:CH46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17348,7 +17290,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>ldl</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -17361,11 +17303,11 @@
         <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:CF47)</f>
+        <f>SUM(G47:CH47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:CF47),1)</f>
+        <f>ROUND(AVERAGE(G47:CH47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17380,7 +17322,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>Tropical</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -17393,11 +17335,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:CF48)</f>
+        <f>SUM(G48:CH48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:CF48),1)</f>
+        <f>ROUND(AVERAGE(G48:CH48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17412,7 +17354,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Diego229</t>
+          <t>-WOLF-</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -17425,11 +17367,11 @@
         <v>0</v>
       </c>
       <c r="E49" s="68">
-        <f>SUM(G49:CF49)</f>
+        <f>SUM(G49:CH49)</f>
         <v/>
       </c>
       <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:CF49),1)</f>
+        <f>ROUND(AVERAGE(G49:CH49),1)</f>
         <v/>
       </c>
       <c r="AI49" s="120" t="n"/>
@@ -17440,6 +17382,38 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>-_HORROR_-</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:CH50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:CH50),1)</f>
+        <v/>
+      </c>
+      <c r="AI50" s="120" t="n"/>
+      <c r="AJ50" s="121" t="n"/>
+      <c r="AK50" s="120" t="n"/>
+      <c r="AL50" s="121" t="n"/>
+      <c r="AM50" s="120" t="n"/>
+      <c r="AN50" s="121" t="n"/>
+      <c r="AO50" s="120" t="n"/>
+      <c r="AP50" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-04-30
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI50"/>
+  <dimension ref="A1:CJ48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13211,7 +13211,12 @@
       </c>
       <c r="CI1" s="109" t="inlineStr">
         <is>
-          <t>Colonna87</t>
+          <t>WAR-41 (1)</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>WAR-41 (2)</t>
         </is>
       </c>
     </row>
@@ -13231,11 +13236,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:CH2)</f>
+        <f>SUM(G2:CJ2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:CH2),1)</f>
+        <f>ROUND(AVERAGE(G2:CJ2),1)</f>
         <v/>
       </c>
     </row>
@@ -13255,11 +13260,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:CH3)</f>
+        <f>SUM(G3:CJ3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:CH3),1)</f>
+        <f>ROUND(AVERAGE(G3:CJ3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13308,14 +13313,14 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:CH4)</f>
+        <f>SUM(G4:CJ4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:CH4),1)</f>
+        <f>ROUND(AVERAGE(G4:CJ4),1)</f>
         <v/>
       </c>
       <c r="AM4" t="n">
@@ -13422,6 +13427,12 @@
         <v>3</v>
       </c>
       <c r="CF4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -13441,11 +13452,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:CH5)</f>
+        <f>SUM(G5:CJ5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:CH5),1)</f>
+        <f>ROUND(AVERAGE(G5:CJ5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13531,11 +13542,11 @@
         <v>27</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:CH6)</f>
+        <f>SUM(G6:CJ6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:CH6),1)</f>
+        <f>ROUND(AVERAGE(G6:CJ6),1)</f>
         <v/>
       </c>
       <c r="G6" s="79" t="n">
@@ -13757,11 +13768,11 @@
         <v>13</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:CH7)</f>
+        <f>SUM(G7:CJ7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:CH7),1)</f>
+        <f>ROUND(AVERAGE(G7:CJ7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13863,11 +13874,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:CH8)</f>
+        <f>SUM(G8:CJ8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:CH8),1)</f>
+        <f>ROUND(AVERAGE(G8:CJ8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13894,14 +13905,14 @@
         <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:CH9)</f>
+        <f>SUM(G9:CJ9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:CH9),1)</f>
+        <f>ROUND(AVERAGE(G9:CJ9),1)</f>
         <v/>
       </c>
       <c r="AM9" t="n">
@@ -13996,6 +14007,12 @@
         <v>3</v>
       </c>
       <c r="CD9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -14012,14 +14029,14 @@
         <v>4</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:CH10)</f>
+        <f>SUM(G10:CJ10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:CH10),1)</f>
+        <f>ROUND(AVERAGE(G10:CJ10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14166,6 +14183,12 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CI10" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
@@ -14183,11 +14206,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:CH11)</f>
+        <f>SUM(G11:CJ11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:CH11),1)</f>
+        <f>ROUND(AVERAGE(G11:CJ11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14218,14 +14241,14 @@
         <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:CH12)</f>
+        <f>SUM(G12:CJ12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:CH12),1)</f>
+        <f>ROUND(AVERAGE(G12:CJ12),1)</f>
         <v/>
       </c>
       <c r="BO12" t="n">
@@ -14269,6 +14292,12 @@
       </c>
       <c r="CD12" t="n">
         <v>3</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -14287,11 +14316,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:CH13)</f>
+        <f>SUM(G13:CJ13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:CH13),1)</f>
+        <f>ROUND(AVERAGE(G13:CJ13),1)</f>
         <v/>
       </c>
     </row>
@@ -14308,14 +14337,14 @@
         <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:CH14)</f>
+        <f>SUM(G14:CJ14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:CH14),1)</f>
+        <f>ROUND(AVERAGE(G14:CJ14),1)</f>
         <v/>
       </c>
       <c r="Q14" s="79" t="n">
@@ -14430,6 +14459,12 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CI14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
@@ -14447,11 +14482,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:CH15)</f>
+        <f>SUM(G15:CJ15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:CH15),1)</f>
+        <f>ROUND(AVERAGE(G15:CJ15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14477,11 +14512,11 @@
         <v>16</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:CH16)</f>
+        <f>SUM(G16:CJ16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:CH16),1)</f>
+        <f>ROUND(AVERAGE(G16:CJ16),1)</f>
         <v/>
       </c>
       <c r="G16" s="79" t="n">
@@ -14607,11 +14642,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:CH17)</f>
+        <f>SUM(G17:CJ17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:CH17),1)</f>
+        <f>ROUND(AVERAGE(G17:CJ17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14783,11 +14818,11 @@
         <v>18</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:CH18)</f>
+        <f>SUM(G18:CJ18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:CH18),1)</f>
+        <f>ROUND(AVERAGE(G18:CJ18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14910,7 +14945,7 @@
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>HikariNoRob</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B19" s="79" t="n">
@@ -14920,356 +14955,424 @@
         <v>0</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:CH19)</f>
+        <f>SUM(G19:CJ19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:CH19),1)</f>
-        <v/>
-      </c>
-      <c r="G19" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="I19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z19" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G19:CJ19),1)</f>
+        <v/>
       </c>
       <c r="AI19" s="68" t="n"/>
       <c r="AJ19" s="68" t="n"/>
       <c r="AK19" s="68" t="n"/>
       <c r="AL19" s="68" t="n"/>
-      <c r="AM19" s="68" t="n"/>
-      <c r="AN19" s="68" t="n"/>
-      <c r="AS19" s="68" t="n"/>
-      <c r="AT19" s="68" t="n"/>
+      <c r="AM19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO19" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP19" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU19" s="68" t="n"/>
+      <c r="AV19" s="68" t="n"/>
       <c r="AY19" t="n">
         <v>3</v>
       </c>
       <c r="AZ19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BE19" t="n">
         <v>3</v>
       </c>
-      <c r="BF19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH19" t="inlineStr">
+      <c r="BF19" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BS19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT19" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>leo</t>
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:CH20)</f>
+        <f>SUM(G20:CJ20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:CH20),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G20:CJ20),1)</f>
+        <v/>
+      </c>
+      <c r="AE20" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF20" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="AI20" s="68" t="n"/>
       <c r="AJ20" s="68" t="n"/>
       <c r="AK20" s="68" t="n"/>
       <c r="AL20" s="68" t="n"/>
-      <c r="AM20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO20" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP20" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU20" s="68" t="n"/>
-      <c r="AV20" s="68" t="n"/>
-      <c r="AY20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ20" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BS20" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT20" t="n">
+      <c r="AM20" s="68" t="n"/>
+      <c r="AN20" s="68" t="n"/>
+      <c r="AO20" s="68" t="n"/>
+      <c r="AP20" s="68" t="n"/>
+      <c r="BA20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR20" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>leo</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C21" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:CH21)</f>
+        <f>SUM(G21:CJ21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:CH21),1)</f>
-        <v/>
-      </c>
-      <c r="AE21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF21" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI21" s="68" t="n"/>
-      <c r="AJ21" s="68" t="n"/>
-      <c r="AK21" s="68" t="n"/>
-      <c r="AL21" s="68" t="n"/>
+        <f>ROUND(AVERAGE(G21:CJ21),1)</f>
+        <v/>
+      </c>
       <c r="AM21" s="68" t="n"/>
       <c r="AN21" s="68" t="n"/>
       <c r="AO21" s="68" t="n"/>
       <c r="AP21" s="68" t="n"/>
-      <c r="BA21" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB21" t="n">
+      <c r="AS21" s="68" t="n"/>
+      <c r="AT21" s="68" t="n"/>
+      <c r="AU21" s="68" t="n"/>
+      <c r="AV21" s="68" t="n"/>
+      <c r="BC21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BG21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH21" t="n">
         <v>2</v>
       </c>
       <c r="BI21" t="n">
         <v>3</v>
       </c>
       <c r="BJ21" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO21" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL21" t="n">
         <v>3</v>
       </c>
       <c r="BQ21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BR21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX21" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ21" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA21" t="n">
+        <v>2</v>
+      </c>
+      <c r="CB21" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI21" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ21" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:CH22)</f>
+        <f>SUM(G22:CJ22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:CH22),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G22:CJ22),1)</f>
+        <v/>
+      </c>
+      <c r="I22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="M22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P22" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R22" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X22" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA22" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB22" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC22" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD22" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="AM22" s="68" t="n"/>
       <c r="AN22" s="68" t="n"/>
-      <c r="AO22" s="68" t="n"/>
-      <c r="AP22" s="68" t="n"/>
+      <c r="AO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>1</v>
+      </c>
       <c r="AS22" s="68" t="n"/>
       <c r="AT22" s="68" t="n"/>
-      <c r="AU22" s="68" t="n"/>
-      <c r="AV22" s="68" t="n"/>
-      <c r="BC22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BF22" t="inlineStr">
+      <c r="AU22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP22" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT22" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC22" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD22" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BG22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BI22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW22" t="inlineStr">
+      <c r="CF22" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BX22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ22" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA22" t="n">
-        <v>2</v>
-      </c>
-      <c r="CB22" t="n">
+      <c r="CI22" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ22" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:CH23)</f>
+        <f>SUM(G23:CJ23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:CH23),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G23:CJ23),1)</f>
+        <v/>
+      </c>
+      <c r="G23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="I23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" s="80" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="J23" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="M23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R23" s="80" t="inlineStr">
+      <c r="S23" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T23" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
       <c r="W23" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X23" s="80" t="n">
         <v>2</v>
@@ -15277,45 +15380,69 @@
       <c r="AA23" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="AB23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD23" s="80" t="n">
+      <c r="AB23" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AE23" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF23" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI23" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ23" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK23" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL23" s="121" t="n">
         <v>3</v>
       </c>
       <c r="AM23" s="68" t="n"/>
       <c r="AN23" s="68" t="n"/>
       <c r="AO23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS23" s="68" t="n"/>
-      <c r="AT23" s="68" t="n"/>
-      <c r="AU23" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV23" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY23" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ23" t="n">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AS23" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>2</v>
       </c>
       <c r="BA23" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB23" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BE23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BG23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BH23" t="n">
         <v>3</v>
@@ -15323,33 +15450,71 @@
       <c r="BK23" t="n">
         <v>3</v>
       </c>
-      <c r="BL23" t="n">
-        <v>2</v>
+      <c r="BL23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BO23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BP23" t="n">
         <v>3</v>
       </c>
-      <c r="BS23" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT23" t="n">
-        <v>3</v>
+      <c r="BU23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BW23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY23" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CA23" t="n">
+        <v>2</v>
+      </c>
+      <c r="CB23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="CC23" t="n">
         <v>3</v>
       </c>
-      <c r="CD23" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE23" t="inlineStr">
+      <c r="CD23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
+      <c r="CE23" t="n">
+        <v>3</v>
+      </c>
       <c r="CF23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI23" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ23" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15358,190 +15523,50 @@
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>MIRIAM MIRIAM</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C24" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:CH24)</f>
+        <f>SUM(G24:CJ24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:CH24),1)</f>
-        <v/>
-      </c>
-      <c r="G24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P24" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G24:CJ24),1)</f>
+        <v/>
+      </c>
+      <c r="AM24" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN24" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO24" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP24" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS24" s="120" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT24" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="S24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X24" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI24" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ24" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK24" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL24" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM24" s="68" t="n"/>
-      <c r="AN24" s="68" t="n"/>
-      <c r="AO24" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AS24" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT24" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>3</v>
-      </c>
       <c r="BB24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BE24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BG24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BO24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CA24" t="n">
-        <v>2</v>
-      </c>
-      <c r="CB24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CC24" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE24" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF24" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -15550,387 +15575,383 @@
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>Mario</t>
+          <t>piegian99</t>
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:CH25)</f>
+        <f>SUM(G25:CJ25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:CH25),1)</f>
-        <v/>
-      </c>
-      <c r="AM25" s="68" t="n"/>
-      <c r="AN25" s="68" t="n"/>
-      <c r="AO25" s="68" t="n"/>
-      <c r="AP25" s="68" t="n"/>
-      <c r="AS25" s="68" t="n"/>
-      <c r="AT25" s="68" t="n"/>
-      <c r="AU25" s="68" t="n"/>
-      <c r="AV25" s="68" t="n"/>
-      <c r="BC25" t="inlineStr">
+        <f>ROUND(AVERAGE(G25:CJ25),1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M25" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="N25" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="T25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V25" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE25" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF25" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI25" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BD25" t="inlineStr">
+      <c r="AJ25" s="121" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
+      <c r="AK25" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL25" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL25" t="n">
+        <v>3</v>
+      </c>
       <c r="BM25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BN25" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BN25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BW25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BQ25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BR25" t="inlineStr">
+      <c r="BX25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BS25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BU25" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BZ25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="BY25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ25" t="n">
+        <v>3</v>
       </c>
       <c r="CA25" t="n">
-        <v>2</v>
-      </c>
-      <c r="CB25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CC25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="CB25" t="n">
+        <v>2</v>
+      </c>
+      <c r="CC25" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD25" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE25" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF25" t="n">
+        <v>2</v>
+      </c>
+      <c r="CI25" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ25" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>MIRIAM MIRIAM</t>
+          <t>pigiamone99</t>
         </is>
       </c>
       <c r="B26" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C26" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:CH26)</f>
+        <f>SUM(G26:CJ26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:CH26),1)</f>
-        <v/>
-      </c>
-      <c r="AM26" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN26" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO26" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP26" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS26" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT26" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA26" t="inlineStr">
+        <f>ROUND(AVERAGE(G26:CJ26),1)</f>
+        <v/>
+      </c>
+      <c r="I26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE26" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF26" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI26" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BB26" t="inlineStr">
+      <c r="AJ26" s="121" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="AK26" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL26" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW26" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX26" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY26" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ26" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>PIPPII</t>
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:CH27)</f>
+        <f>SUM(G27:CJ27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:CH27),1)</f>
-        <v/>
-      </c>
-      <c r="G27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I27" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M27" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="N27" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T27" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V27" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G27:CJ27),1)</f>
+        <v/>
+      </c>
+      <c r="Y27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z27" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AC27" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD27" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="AE27" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF27" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI27" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ27" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK27" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL27" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BM27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ27" t="n">
-        <v>2</v>
-      </c>
-      <c r="BR27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BS27" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BU27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BV27" t="n">
         <v>2</v>
       </c>
-      <c r="BW27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY27" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB27" t="n">
-        <v>2</v>
-      </c>
       <c r="CC27" t="n">
         <v>3</v>
       </c>
       <c r="CD27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF27" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>pigiamone99</t>
+          <t>revolver</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
+        <v>9</v>
+      </c>
+      <c r="C28" s="68" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="68" t="n">
-        <v>2</v>
-      </c>
       <c r="D28" s="79" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:CH28)</f>
+        <f>SUM(G28:CJ28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:CH28),1)</f>
-        <v/>
-      </c>
-      <c r="I28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P28" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q28" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R28" s="80" t="n">
-        <v>3</v>
+        <f>ROUND(AVERAGE(G28:CJ28),1)</f>
+        <v/>
+      </c>
+      <c r="S28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="T28" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U28" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="V28" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="W28" s="79" t="n">
         <v>3</v>
@@ -15944,8 +15965,14 @@
       <c r="Z28" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="AC28" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD28" s="80" t="n">
+        <v>3</v>
+      </c>
       <c r="AE28" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF28" s="80" t="n">
         <v>3</v>
@@ -15961,235 +15988,267 @@
         </is>
       </c>
       <c r="AK28" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL28" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB28" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="AL28" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD28" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BM28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP28" t="n">
+        <v>1</v>
       </c>
       <c r="BQ28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BR28" t="n">
         <v>3</v>
       </c>
-      <c r="BS28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BT28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW28" t="inlineStr">
+      <c r="BU28" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV28" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA28" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB28" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BX28" t="inlineStr">
+      <c r="CD28" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
-      </c>
-      <c r="BY28" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ28" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:CH29)</f>
+        <f>SUM(G29:CJ29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:CH29),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G29:CJ29),1)</f>
+        <v/>
+      </c>
+      <c r="I29" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J29" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="K29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="M29" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Q29" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R29" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X29" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="Y29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z29" s="80" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="Z29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB29" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC29" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE29" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF29" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM29" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN29" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ29" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AC29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE29" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF29" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV29" t="n">
-        <v>2</v>
-      </c>
-      <c r="CC29" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD29" t="n">
+      <c r="BV29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CA29" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB29" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:CH30)</f>
+        <f>SUM(G30:CJ30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:CH30),1)</f>
-        <v/>
-      </c>
-      <c r="S30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U30" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G30:CJ30),1)</f>
+        <v/>
+      </c>
+      <c r="G30" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O30" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P30" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q30" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R30" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU30" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV30" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="V30" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC30" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE30" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF30" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI30" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ30" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK30" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL30" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD30" t="n">
-        <v>2</v>
-      </c>
-      <c r="BI30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BJ30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BM30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU30" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV30" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA30" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB30" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD30" t="inlineStr">
+      <c r="BH30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16198,99 +16257,113 @@
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>Stentaaa</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C31" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:CH31)</f>
+        <f>SUM(G31:CJ31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:CH31),1)</f>
-        <v/>
-      </c>
-      <c r="I31" s="79" t="inlineStr">
+        <f>ROUND(AVERAGE(G31:CJ31),1)</f>
+        <v/>
+      </c>
+      <c r="G31" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="O31" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y31" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z31" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA31" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB31" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI31" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="J31" s="80" t="inlineStr">
+      <c r="AJ31" s="121" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="K31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L31" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M31" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Q31" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R31" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X31" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z31" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC31" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF31" s="80" t="n">
-        <v>2</v>
+      <c r="AK31" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL31" s="121" t="n">
+        <v>3</v>
       </c>
       <c r="AM31" s="120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN31" s="121" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AS31" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT31" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM31" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN31" t="n">
+        <v>1</v>
       </c>
       <c r="BO31" t="n">
         <v>1</v>
@@ -16298,126 +16371,70 @@
       <c r="BP31" t="n">
         <v>1</v>
       </c>
-      <c r="BQ31" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR31" t="n">
-        <v>1</v>
-      </c>
-      <c r="BU31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="BS31" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT31" t="n">
+        <v>2</v>
       </c>
       <c r="CA31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="CB31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:CH32)</f>
+        <f>SUM(G32:CJ32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:CH32),1)</f>
-        <v/>
-      </c>
-      <c r="G32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q32" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R32" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU32" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV32" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA32" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB32" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE32" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF32" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BH32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <f>ROUND(AVERAGE(G32:CJ32),1)</f>
+        <v/>
+      </c>
+      <c r="AS32" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT32" s="121" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C33" s="68" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:CH33)</f>
+        <f>SUM(G33:CJ33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:CH33),1)</f>
+        <f>ROUND(AVERAGE(G33:CJ33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16427,51 +16444,61 @@
         <v>3</v>
       </c>
       <c r="I33" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L33" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="M33" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N33" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K33" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L33" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="O33" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P33" s="80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q33" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R33" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="U33" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V33" s="80" t="n">
-        <v>2</v>
+      <c r="S33" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W33" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X33" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="Y33" s="79" t="n">
         <v>2</v>
       </c>
       <c r="Z33" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA33" s="79" t="n">
         <v>3</v>
       </c>
       <c r="AB33" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC33" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD33" s="80" t="n">
         <v>3</v>
       </c>
       <c r="AI33" s="120" t="inlineStr">
@@ -16502,394 +16529,318 @@
       <c r="AT33" s="121" t="n">
         <v>3</v>
       </c>
+      <c r="AU33" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV33" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL33" t="n">
+        <v>2</v>
+      </c>
       <c r="BM33" t="n">
         <v>3</v>
       </c>
       <c r="BN33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BO33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP33" t="n">
-        <v>1</v>
-      </c>
-      <c r="BS33" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT33" t="n">
-        <v>2</v>
-      </c>
-      <c r="CA33" t="n">
-        <v>1</v>
-      </c>
-      <c r="CB33" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="BQ33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BR33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BU33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV33" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>zordan</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C34" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D34" s="79" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:CH34)</f>
+        <f>SUM(G34:CJ34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:CH34),1)</f>
-        <v/>
-      </c>
-      <c r="AS34" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT34" s="121" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G34:CJ34),1)</f>
+        <v/>
+      </c>
+      <c r="U34" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V34" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W34" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X34" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="Y34" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z34" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA34" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB34" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC34" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD34" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE34" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF34" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI34" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ34" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK34" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL34" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AM34" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN34" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO34" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP34" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ34" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA34" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB34" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC34" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD34" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE34" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BQ34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BR34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>falcuns</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:CH35)</f>
+        <f>SUM(G35:CJ35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:CH35),1)</f>
-        <v/>
-      </c>
-      <c r="G35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K35" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L35" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O35" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P35" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q35" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T35" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W35" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA35" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB35" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD35" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI35" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ35" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK35" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL35" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM35" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN35" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS35" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT35" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU35" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV35" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA35" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG35" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL35" t="n">
-        <v>2</v>
-      </c>
-      <c r="BM35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP35" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BS35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BT35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BU35" t="n">
-        <v>2</v>
-      </c>
-      <c r="BV35" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
+        <f>ROUND(AVERAGE(G35:CJ35),1)</f>
+        <v/>
+      </c>
+      <c r="AI35" s="120" t="n"/>
+      <c r="AJ35" s="121" t="n"/>
+      <c r="AK35" s="120" t="n"/>
+      <c r="AL35" s="121" t="n"/>
+      <c r="AM35" s="120" t="n"/>
+      <c r="AN35" s="121" t="n"/>
+      <c r="AO35" s="120" t="n"/>
+      <c r="AP35" s="121" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C36" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:CH36)</f>
+        <f>SUM(G36:CJ36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:CH36),1)</f>
-        <v/>
-      </c>
-      <c r="U36" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V36" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W36" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X36" s="80" t="inlineStr">
+        <f>ROUND(AVERAGE(G36:CJ36),1)</f>
+        <v/>
+      </c>
+      <c r="AI36" s="120" t="n"/>
+      <c r="AJ36" s="121" t="n"/>
+      <c r="AK36" s="120" t="n"/>
+      <c r="AL36" s="121" t="n"/>
+      <c r="AM36" s="120" t="n"/>
+      <c r="AN36" s="121" t="n"/>
+      <c r="AO36" s="120" t="n"/>
+      <c r="AP36" s="121" t="n"/>
+      <c r="CE36" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="Y36" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z36" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA36" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB36" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC36" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD36" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE36" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF36" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI36" s="120" t="inlineStr">
+      <c r="CF36" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ36" s="121" t="inlineStr">
+      <c r="CI36" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AK36" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL36" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AM36" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN36" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO36" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP36" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY36" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ36" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA36" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB36" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC36" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD36" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE36" t="n">
-        <v>2</v>
-      </c>
-      <c r="BF36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BQ36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR36" t="inlineStr">
+      <c r="CJ36" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -16898,24 +16849,24 @@
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>falcuns</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C37" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:CH37)</f>
+        <f>SUM(G37:CJ37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:CH37),1)</f>
+        <f>ROUND(AVERAGE(G37:CJ37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16926,28 +16877,38 @@
       <c r="AN37" s="121" t="n"/>
       <c r="AO37" s="120" t="n"/>
       <c r="AP37" s="121" t="n"/>
+      <c r="CC37" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD37" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:CH38)</f>
+        <f>SUM(G38:CJ38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:CH38),1)</f>
+        <f>ROUND(AVERAGE(G38:CJ38),1)</f>
         <v/>
       </c>
       <c r="AI38" s="120" t="n"/>
@@ -16958,38 +16919,52 @@
       <c r="AN38" s="121" t="n"/>
       <c r="AO38" s="120" t="n"/>
       <c r="AP38" s="121" t="n"/>
-      <c r="CE38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="CA38" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB38" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC38" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD38" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE38" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF38" t="n">
+        <v>2</v>
+      </c>
+      <c r="CI38" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ38" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>matty</t>
+          <t>Ema alba003</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C39" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:CH39)</f>
+        <f>SUM(G39:CJ39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:CH39),1)</f>
+        <f>ROUND(AVERAGE(G39:CJ39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -17000,62 +16975,28 @@
       <c r="AN39" s="121" t="n"/>
       <c r="AO39" s="120" t="n"/>
       <c r="AP39" s="121" t="n"/>
-      <c r="BW39" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX39" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY39" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ39" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA39" t="n">
-        <v>1</v>
-      </c>
-      <c r="CB39" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC39" t="n">
-        <v>0</v>
-      </c>
-      <c r="CD39" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE39" t="n">
-        <v>2</v>
-      </c>
-      <c r="CF39" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:CH40)</f>
+        <f>SUM(G40:CJ40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:CH40),1)</f>
+        <f>ROUND(AVERAGE(G40:CJ40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -17066,21 +17007,11 @@
       <c r="AN40" s="121" t="n"/>
       <c r="AO40" s="120" t="n"/>
       <c r="AP40" s="121" t="n"/>
-      <c r="CC40" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD40" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>re deo</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
@@ -17090,14 +17021,14 @@
         <v>0</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:CH41)</f>
+        <f>SUM(G41:CJ41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:CH41),1)</f>
+        <f>ROUND(AVERAGE(G41:CJ41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -17108,29 +17039,11 @@
       <c r="AN41" s="121" t="n"/>
       <c r="AO41" s="120" t="n"/>
       <c r="AP41" s="121" t="n"/>
-      <c r="CA41" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB41" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC41" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD41" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE41" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF41" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>Ema alba003</t>
+          <t>Dade_Aca_03</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
@@ -17143,11 +17056,11 @@
         <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:CH42)</f>
+        <f>SUM(G42:CJ42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:CH42),1)</f>
+        <f>ROUND(AVERAGE(G42:CJ42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -17162,7 +17075,7 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>AnT0x</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -17175,11 +17088,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:CH43)</f>
+        <f>SUM(G43:CJ43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:CH43),1)</f>
+        <f>ROUND(AVERAGE(G43:CJ43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -17194,24 +17107,24 @@
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>re deo</t>
+          <t>ldl</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:CH44)</f>
+        <f>SUM(G44:CJ44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:CH44),1)</f>
+        <f>ROUND(AVERAGE(G44:CJ44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -17222,11 +17135,21 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
+      <c r="CI44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Dade_Aca_03</t>
+          <t>Tropical</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -17239,11 +17162,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:CH45)</f>
+        <f>SUM(G45:CJ45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:CH45),1)</f>
+        <f>ROUND(AVERAGE(G45:CJ45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -17258,7 +17181,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>AnT0x</t>
+          <t>-WOLF-</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -17271,11 +17194,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:CH46)</f>
+        <f>SUM(G46:CJ46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:CH46),1)</f>
+        <f>ROUND(AVERAGE(G46:CJ46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17290,24 +17213,24 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>ldl</t>
+          <t>-_HORROR_-</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:CH47)</f>
+        <f>SUM(G47:CJ47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:CH47),1)</f>
+        <f>ROUND(AVERAGE(G47:CJ47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17318,11 +17241,21 @@
       <c r="AN47" s="121" t="n"/>
       <c r="AO47" s="120" t="n"/>
       <c r="AP47" s="121" t="n"/>
+      <c r="CI47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ47" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>Tropical</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -17335,11 +17268,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:CH48)</f>
+        <f>SUM(G48:CJ48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:CH48),1)</f>
+        <f>ROUND(AVERAGE(G48:CJ48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17350,70 +17283,6 @@
       <c r="AN48" s="121" t="n"/>
       <c r="AO48" s="120" t="n"/>
       <c r="AP48" s="121" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="79" t="inlineStr">
-        <is>
-          <t>-WOLF-</t>
-        </is>
-      </c>
-      <c r="B49" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="68">
-        <f>SUM(G49:CH49)</f>
-        <v/>
-      </c>
-      <c r="F49" s="68">
-        <f>ROUND(AVERAGE(G49:CH49),1)</f>
-        <v/>
-      </c>
-      <c r="AI49" s="120" t="n"/>
-      <c r="AJ49" s="121" t="n"/>
-      <c r="AK49" s="120" t="n"/>
-      <c r="AL49" s="121" t="n"/>
-      <c r="AM49" s="120" t="n"/>
-      <c r="AN49" s="121" t="n"/>
-      <c r="AO49" s="120" t="n"/>
-      <c r="AP49" s="121" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>-_HORROR_-</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:CH50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:CH50),1)</f>
-        <v/>
-      </c>
-      <c r="AI50" s="120" t="n"/>
-      <c r="AJ50" s="121" t="n"/>
-      <c r="AK50" s="120" t="n"/>
-      <c r="AL50" s="121" t="n"/>
-      <c r="AM50" s="120" t="n"/>
-      <c r="AN50" s="121" t="n"/>
-      <c r="AO50" s="120" t="n"/>
-      <c r="AP50" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-02
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -12720,7 +12720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ48"/>
+  <dimension ref="A1:CJ51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -13236,11 +13236,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="68">
-        <f>SUM(G2:CJ2)</f>
+        <f>SUM(G2:H2)</f>
         <v/>
       </c>
       <c r="F2" s="68">
-        <f>ROUND(AVERAGE(G2:CJ2),1)</f>
+        <f>ROUND(AVERAGE(G2:H2),1)</f>
         <v/>
       </c>
     </row>
@@ -13260,11 +13260,11 @@
         <v>3</v>
       </c>
       <c r="E3" s="68">
-        <f>SUM(G3:CJ3)</f>
+        <f>SUM(G3:H3)</f>
         <v/>
       </c>
       <c r="F3" s="68">
-        <f>ROUND(AVERAGE(G3:CJ3),1)</f>
+        <f>ROUND(AVERAGE(G3:H3),1)</f>
         <v/>
       </c>
       <c r="AI3" s="68" t="n"/>
@@ -13313,15 +13313,21 @@
         <v>1</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="68">
-        <f>SUM(G4:CJ4)</f>
+        <f>SUM(G4:H4)</f>
         <v/>
       </c>
       <c r="F4" s="68">
-        <f>ROUND(AVERAGE(G4:CJ4),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G4:H4),1)</f>
+        <v/>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
       </c>
       <c r="AM4" t="n">
         <v>3</v>
@@ -13452,11 +13458,11 @@
         <v>9</v>
       </c>
       <c r="E5" s="68">
-        <f>SUM(G5:CJ5)</f>
+        <f>SUM(G5:H5)</f>
         <v/>
       </c>
       <c r="F5" s="68">
-        <f>ROUND(AVERAGE(G5:CJ5),1)</f>
+        <f>ROUND(AVERAGE(G5:H5),1)</f>
         <v/>
       </c>
       <c r="BI5" t="n">
@@ -13533,27 +13539,31 @@
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C6" s="68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E6" s="68">
-        <f>SUM(G6:CJ6)</f>
+        <f>SUM(G6:H6)</f>
         <v/>
       </c>
       <c r="F6" s="68">
-        <f>ROUND(AVERAGE(G6:CJ6),1)</f>
-        <v/>
-      </c>
-      <c r="G6" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" s="80" t="n">
-        <v>1</v>
+        <f>ROUND(AVERAGE(G6:H6),1)</f>
+        <v/>
+      </c>
+      <c r="G6" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H6" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I6" s="79" t="n">
         <v>0</v>
@@ -13768,11 +13778,11 @@
         <v>13</v>
       </c>
       <c r="E7" s="68">
-        <f>SUM(G7:CJ7)</f>
+        <f>SUM(G7:H7)</f>
         <v/>
       </c>
       <c r="F7" s="68">
-        <f>ROUND(AVERAGE(G7:CJ7),1)</f>
+        <f>ROUND(AVERAGE(G7:H7),1)</f>
         <v/>
       </c>
       <c r="K7" s="79" t="n">
@@ -13874,11 +13884,11 @@
         <v>1</v>
       </c>
       <c r="E8" s="68">
-        <f>SUM(G8:CJ8)</f>
+        <f>SUM(G8:H8)</f>
         <v/>
       </c>
       <c r="F8" s="68">
-        <f>ROUND(AVERAGE(G8:CJ8),1)</f>
+        <f>ROUND(AVERAGE(G8:H8),1)</f>
         <v/>
       </c>
       <c r="AS8" s="68" t="n"/>
@@ -13905,15 +13915,21 @@
         <v>1</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="68">
-        <f>SUM(G9:CJ9)</f>
+        <f>SUM(G9:H9)</f>
         <v/>
       </c>
       <c r="F9" s="68">
-        <f>ROUND(AVERAGE(G9:CJ9),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G9:H9),1)</f>
+        <v/>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
       </c>
       <c r="AM9" t="n">
         <v>1</v>
@@ -14029,14 +14045,14 @@
         <v>4</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="68">
-        <f>SUM(G10:CJ10)</f>
+        <f>SUM(G10:H10)</f>
         <v/>
       </c>
       <c r="F10" s="68">
-        <f>ROUND(AVERAGE(G10:CJ10),1)</f>
+        <f>ROUND(AVERAGE(G10:H10),1)</f>
         <v/>
       </c>
       <c r="G10" s="79" t="n">
@@ -14206,11 +14222,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="68">
-        <f>SUM(G11:CJ11)</f>
+        <f>SUM(G11:H11)</f>
         <v/>
       </c>
       <c r="F11" s="68">
-        <f>ROUND(AVERAGE(G11:CJ11),1)</f>
+        <f>ROUND(AVERAGE(G11:H11),1)</f>
         <v/>
       </c>
       <c r="AI11" s="68" t="n"/>
@@ -14241,15 +14257,21 @@
         <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E12" s="68">
-        <f>SUM(G12:CJ12)</f>
+        <f>SUM(G12:H12)</f>
         <v/>
       </c>
       <c r="F12" s="68">
-        <f>ROUND(AVERAGE(G12:CJ12),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G12:H12),1)</f>
+        <v/>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
       </c>
       <c r="BO12" t="n">
         <v>3</v>
@@ -14316,11 +14338,11 @@
         <v>0</v>
       </c>
       <c r="E13" s="68">
-        <f>SUM(G13:CJ13)</f>
+        <f>SUM(G13:H13)</f>
         <v/>
       </c>
       <c r="F13" s="68">
-        <f>ROUND(AVERAGE(G13:CJ13),1)</f>
+        <f>ROUND(AVERAGE(G13:H13),1)</f>
         <v/>
       </c>
     </row>
@@ -14337,15 +14359,21 @@
         <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E14" s="68">
-        <f>SUM(G14:CJ14)</f>
+        <f>SUM(G14:H14)</f>
         <v/>
       </c>
       <c r="F14" s="68">
-        <f>ROUND(AVERAGE(G14:CJ14),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G14:H14),1)</f>
+        <v/>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
       </c>
       <c r="Q14" s="79" t="n">
         <v>3</v>
@@ -14482,11 +14510,11 @@
         <v>1</v>
       </c>
       <c r="E15" s="68">
-        <f>SUM(G15:CJ15)</f>
+        <f>SUM(G15:H15)</f>
         <v/>
       </c>
       <c r="F15" s="68">
-        <f>ROUND(AVERAGE(G15:CJ15),1)</f>
+        <f>ROUND(AVERAGE(G15:H15),1)</f>
         <v/>
       </c>
       <c r="BA15" t="n">
@@ -14503,27 +14531,31 @@
         </is>
       </c>
       <c r="B16" s="79" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C16" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E16" s="68">
-        <f>SUM(G16:CJ16)</f>
+        <f>SUM(G16:H16)</f>
         <v/>
       </c>
       <c r="F16" s="68">
-        <f>ROUND(AVERAGE(G16:CJ16),1)</f>
-        <v/>
-      </c>
-      <c r="G16" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="80" t="n">
-        <v>2</v>
+        <f>ROUND(AVERAGE(G16:H16),1)</f>
+        <v/>
+      </c>
+      <c r="G16" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H16" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I16" s="79" t="n">
         <v>1</v>
@@ -14642,11 +14674,11 @@
         <v>23</v>
       </c>
       <c r="E17" s="68">
-        <f>SUM(G17:CJ17)</f>
+        <f>SUM(G17:H17)</f>
         <v/>
       </c>
       <c r="F17" s="68">
-        <f>ROUND(AVERAGE(G17:CJ17),1)</f>
+        <f>ROUND(AVERAGE(G17:H17),1)</f>
         <v/>
       </c>
       <c r="I17" s="79" t="n">
@@ -14818,11 +14850,11 @@
         <v>18</v>
       </c>
       <c r="E18" s="68">
-        <f>SUM(G18:CJ18)</f>
+        <f>SUM(G18:H18)</f>
         <v/>
       </c>
       <c r="F18" s="68">
-        <f>ROUND(AVERAGE(G18:CJ18),1)</f>
+        <f>ROUND(AVERAGE(G18:H18),1)</f>
         <v/>
       </c>
       <c r="S18" s="79" t="n">
@@ -14958,11 +14990,11 @@
         <v>6</v>
       </c>
       <c r="E19" s="68">
-        <f>SUM(G19:CJ19)</f>
+        <f>SUM(G19:H19)</f>
         <v/>
       </c>
       <c r="F19" s="68">
-        <f>ROUND(AVERAGE(G19:CJ19),1)</f>
+        <f>ROUND(AVERAGE(G19:H19),1)</f>
         <v/>
       </c>
       <c r="AI19" s="68" t="n"/>
@@ -15026,11 +15058,11 @@
         <v>5</v>
       </c>
       <c r="E20" s="68">
-        <f>SUM(G20:CJ20)</f>
+        <f>SUM(G20:H20)</f>
         <v/>
       </c>
       <c r="F20" s="68">
-        <f>ROUND(AVERAGE(G20:CJ20),1)</f>
+        <f>ROUND(AVERAGE(G20:H20),1)</f>
         <v/>
       </c>
       <c r="AE20" s="79" t="n">
@@ -15085,15 +15117,21 @@
         <v>1</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" s="68">
-        <f>SUM(G21:CJ21)</f>
+        <f>SUM(G21:H21)</f>
         <v/>
       </c>
       <c r="F21" s="68">
-        <f>ROUND(AVERAGE(G21:CJ21),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G21:H21),1)</f>
+        <v/>
+      </c>
+      <c r="G21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
       </c>
       <c r="AM21" s="68" t="n"/>
       <c r="AN21" s="68" t="n"/>
@@ -15189,15 +15227,21 @@
         <v>1</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E22" s="68">
-        <f>SUM(G22:CJ22)</f>
+        <f>SUM(G22:H22)</f>
         <v/>
       </c>
       <c r="F22" s="68">
-        <f>ROUND(AVERAGE(G22:CJ22),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G22:H22),1)</f>
+        <v/>
+      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3</v>
       </c>
       <c r="I22" s="79" t="n">
         <v>2</v>
@@ -15327,27 +15371,29 @@
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C23" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E23" s="68">
-        <f>SUM(G23:CJ23)</f>
+        <f>SUM(G23:H23)</f>
         <v/>
       </c>
       <c r="F23" s="68">
-        <f>ROUND(AVERAGE(G23:CJ23),1)</f>
+        <f>ROUND(AVERAGE(G23:H23),1)</f>
         <v/>
       </c>
       <c r="G23" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="H23" s="80" t="n">
-        <v>1</v>
+      <c r="H23" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I23" s="79" t="n">
         <v>3</v>
@@ -15536,11 +15582,11 @@
         <v>4</v>
       </c>
       <c r="E24" s="68">
-        <f>SUM(G24:CJ24)</f>
+        <f>SUM(G24:H24)</f>
         <v/>
       </c>
       <c r="F24" s="68">
-        <f>ROUND(AVERAGE(G24:CJ24),1)</f>
+        <f>ROUND(AVERAGE(G24:H24),1)</f>
         <v/>
       </c>
       <c r="AM24" s="120" t="n">
@@ -15585,14 +15631,14 @@
         <v>2</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="68">
-        <f>SUM(G25:CJ25)</f>
+        <f>SUM(G25:H25)</f>
         <v/>
       </c>
       <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:CJ25),1)</f>
+        <f>ROUND(AVERAGE(G25:H25),1)</f>
         <v/>
       </c>
       <c r="G25" s="79" t="n">
@@ -15755,15 +15801,21 @@
         <v>2</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E26" s="68">
-        <f>SUM(G26:CJ26)</f>
+        <f>SUM(G26:H26)</f>
         <v/>
       </c>
       <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:CJ26),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G26:H26),1)</f>
+        <v/>
+      </c>
+      <c r="G26" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
       </c>
       <c r="I26" s="79" t="n">
         <v>3</v>
@@ -15874,11 +15926,11 @@
         <v>5</v>
       </c>
       <c r="E27" s="68">
-        <f>SUM(G27:CJ27)</f>
+        <f>SUM(G27:H27)</f>
         <v/>
       </c>
       <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:CJ27),1)</f>
+        <f>ROUND(AVERAGE(G27:H27),1)</f>
         <v/>
       </c>
       <c r="Y27" s="79" t="n">
@@ -15930,11 +15982,11 @@
         <v>16</v>
       </c>
       <c r="E28" s="68">
-        <f>SUM(G28:CJ28)</f>
+        <f>SUM(G28:H28)</f>
         <v/>
       </c>
       <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:CJ28),1)</f>
+        <f>ROUND(AVERAGE(G28:H28),1)</f>
         <v/>
       </c>
       <c r="S28" s="79" t="n">
@@ -16065,15 +16117,21 @@
         <v>2</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E29" s="68">
-        <f>SUM(G29:CJ29)</f>
+        <f>SUM(G29:H29)</f>
         <v/>
       </c>
       <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:CJ29),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G29:H29),1)</f>
+        <v/>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
       </c>
       <c r="I29" s="79" t="inlineStr">
         <is>
@@ -16194,11 +16252,11 @@
         <v>8</v>
       </c>
       <c r="E30" s="68">
-        <f>SUM(G30:CJ30)</f>
+        <f>SUM(G30:H30)</f>
         <v/>
       </c>
       <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:CJ30),1)</f>
+        <f>ROUND(AVERAGE(G30:H30),1)</f>
         <v/>
       </c>
       <c r="G30" s="79" t="n">
@@ -16267,21 +16325,21 @@
         <v>1</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E31" s="68">
-        <f>SUM(G31:CJ31)</f>
+        <f>SUM(G31:H31)</f>
         <v/>
       </c>
       <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:CJ31),1)</f>
+        <f>ROUND(AVERAGE(G31:H31),1)</f>
         <v/>
       </c>
       <c r="G31" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H31" s="80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I31" s="79" t="n">
         <v>1</v>
@@ -16400,11 +16458,11 @@
         <v>1</v>
       </c>
       <c r="E32" s="68">
-        <f>SUM(G32:CJ32)</f>
+        <f>SUM(G32:H32)</f>
         <v/>
       </c>
       <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:CJ32),1)</f>
+        <f>ROUND(AVERAGE(G32:H32),1)</f>
         <v/>
       </c>
       <c r="AS32" s="120" t="n">
@@ -16430,11 +16488,11 @@
         <v>28</v>
       </c>
       <c r="E33" s="68">
-        <f>SUM(G33:CJ33)</f>
+        <f>SUM(G33:H33)</f>
         <v/>
       </c>
       <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:CJ33),1)</f>
+        <f>ROUND(AVERAGE(G33:H33),1)</f>
         <v/>
       </c>
       <c r="G33" s="79" t="n">
@@ -16650,11 +16708,11 @@
         <v>15</v>
       </c>
       <c r="E34" s="68">
-        <f>SUM(G34:CJ34)</f>
+        <f>SUM(G34:H34)</f>
         <v/>
       </c>
       <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:CJ34),1)</f>
+        <f>ROUND(AVERAGE(G34:H34),1)</f>
         <v/>
       </c>
       <c r="U34" s="79" t="n">
@@ -16778,11 +16836,11 @@
         <v>0</v>
       </c>
       <c r="E35" s="68">
-        <f>SUM(G35:CJ35)</f>
+        <f>SUM(G35:H35)</f>
         <v/>
       </c>
       <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:CJ35),1)</f>
+        <f>ROUND(AVERAGE(G35:H35),1)</f>
         <v/>
       </c>
       <c r="AI35" s="120" t="n"/>
@@ -16810,11 +16868,11 @@
         <v>2</v>
       </c>
       <c r="E36" s="68">
-        <f>SUM(G36:CJ36)</f>
+        <f>SUM(G36:H36)</f>
         <v/>
       </c>
       <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:CJ36),1)</f>
+        <f>ROUND(AVERAGE(G36:H36),1)</f>
         <v/>
       </c>
       <c r="AI36" s="120" t="n"/>
@@ -16862,11 +16920,11 @@
         <v>1</v>
       </c>
       <c r="E37" s="68">
-        <f>SUM(G37:CJ37)</f>
+        <f>SUM(G37:H37)</f>
         <v/>
       </c>
       <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:CJ37),1)</f>
+        <f>ROUND(AVERAGE(G37:H37),1)</f>
         <v/>
       </c>
       <c r="AI37" s="120" t="n"/>
@@ -16901,15 +16959,21 @@
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" s="68">
-        <f>SUM(G38:CJ38)</f>
+        <f>SUM(G38:H38)</f>
         <v/>
       </c>
       <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:CJ38),1)</f>
-        <v/>
+        <f>ROUND(AVERAGE(G38:H38),1)</f>
+        <v/>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -16960,11 +17024,11 @@
         <v>0</v>
       </c>
       <c r="E39" s="68">
-        <f>SUM(G39:CJ39)</f>
+        <f>SUM(G39:H39)</f>
         <v/>
       </c>
       <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:CJ39),1)</f>
+        <f>ROUND(AVERAGE(G39:H39),1)</f>
         <v/>
       </c>
       <c r="AI39" s="120" t="n"/>
@@ -16992,11 +17056,11 @@
         <v>0</v>
       </c>
       <c r="E40" s="68">
-        <f>SUM(G40:CJ40)</f>
+        <f>SUM(G40:H40)</f>
         <v/>
       </c>
       <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:CJ40),1)</f>
+        <f>ROUND(AVERAGE(G40:H40),1)</f>
         <v/>
       </c>
       <c r="AI40" s="120" t="n"/>
@@ -17024,11 +17088,11 @@
         <v>0</v>
       </c>
       <c r="E41" s="68">
-        <f>SUM(G41:CJ41)</f>
+        <f>SUM(G41:H41)</f>
         <v/>
       </c>
       <c r="F41" s="68">
-        <f>ROUND(AVERAGE(G41:CJ41),1)</f>
+        <f>ROUND(AVERAGE(G41:H41),1)</f>
         <v/>
       </c>
       <c r="AI41" s="120" t="n"/>
@@ -17056,11 +17120,11 @@
         <v>0</v>
       </c>
       <c r="E42" s="68">
-        <f>SUM(G42:CJ42)</f>
+        <f>SUM(G42:H42)</f>
         <v/>
       </c>
       <c r="F42" s="68">
-        <f>ROUND(AVERAGE(G42:CJ42),1)</f>
+        <f>ROUND(AVERAGE(G42:H42),1)</f>
         <v/>
       </c>
       <c r="AI42" s="120" t="n"/>
@@ -17088,11 +17152,11 @@
         <v>0</v>
       </c>
       <c r="E43" s="68">
-        <f>SUM(G43:CJ43)</f>
+        <f>SUM(G43:H43)</f>
         <v/>
       </c>
       <c r="F43" s="68">
-        <f>ROUND(AVERAGE(G43:CJ43),1)</f>
+        <f>ROUND(AVERAGE(G43:H43),1)</f>
         <v/>
       </c>
       <c r="AI43" s="120" t="n"/>
@@ -17120,11 +17184,11 @@
         <v>1</v>
       </c>
       <c r="E44" s="68">
-        <f>SUM(G44:CJ44)</f>
+        <f>SUM(G44:H44)</f>
         <v/>
       </c>
       <c r="F44" s="68">
-        <f>ROUND(AVERAGE(G44:CJ44),1)</f>
+        <f>ROUND(AVERAGE(G44:H44),1)</f>
         <v/>
       </c>
       <c r="AI44" s="120" t="n"/>
@@ -17162,11 +17226,11 @@
         <v>0</v>
       </c>
       <c r="E45" s="68">
-        <f>SUM(G45:CJ45)</f>
+        <f>SUM(G45:H45)</f>
         <v/>
       </c>
       <c r="F45" s="68">
-        <f>ROUND(AVERAGE(G45:CJ45),1)</f>
+        <f>ROUND(AVERAGE(G45:H45),1)</f>
         <v/>
       </c>
       <c r="AI45" s="120" t="n"/>
@@ -17194,11 +17258,11 @@
         <v>0</v>
       </c>
       <c r="E46" s="68">
-        <f>SUM(G46:CJ46)</f>
+        <f>SUM(G46:H46)</f>
         <v/>
       </c>
       <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:CJ46),1)</f>
+        <f>ROUND(AVERAGE(G46:H46),1)</f>
         <v/>
       </c>
       <c r="AI46" s="120" t="n"/>
@@ -17213,24 +17277,24 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>-_HORROR_-</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C47" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" s="68">
-        <f>SUM(G47:CJ47)</f>
+        <f>SUM(G47:H47)</f>
         <v/>
       </c>
       <c r="F47" s="68">
-        <f>ROUND(AVERAGE(G47:CJ47),1)</f>
+        <f>ROUND(AVERAGE(G47:H47),1)</f>
         <v/>
       </c>
       <c r="AI47" s="120" t="n"/>
@@ -17241,21 +17305,11 @@
       <c r="AN47" s="121" t="n"/>
       <c r="AO47" s="120" t="n"/>
       <c r="AP47" s="121" t="n"/>
-      <c r="CI47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CJ47" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -17268,11 +17322,11 @@
         <v>0</v>
       </c>
       <c r="E48" s="68">
-        <f>SUM(G48:CJ48)</f>
+        <f>SUM(G48:H48)</f>
         <v/>
       </c>
       <c r="F48" s="68">
-        <f>ROUND(AVERAGE(G48:CJ48),1)</f>
+        <f>ROUND(AVERAGE(G48:H48),1)</f>
         <v/>
       </c>
       <c r="AI48" s="120" t="n"/>
@@ -17283,6 +17337,102 @@
       <c r="AN48" s="121" t="n"/>
       <c r="AO48" s="120" t="n"/>
       <c r="AP48" s="121" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="79" t="inlineStr">
+        <is>
+          <t>⁰LÜKÄ⁰</t>
+        </is>
+      </c>
+      <c r="B49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="68">
+        <f>SUM(G49:H49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="68">
+        <f>ROUND(AVERAGE(G49:H49),1)</f>
+        <v/>
+      </c>
+      <c r="AI49" s="120" t="n"/>
+      <c r="AJ49" s="121" t="n"/>
+      <c r="AK49" s="120" t="n"/>
+      <c r="AL49" s="121" t="n"/>
+      <c r="AM49" s="120" t="n"/>
+      <c r="AN49" s="121" t="n"/>
+      <c r="AO49" s="120" t="n"/>
+      <c r="AP49" s="121" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>Francesco10</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:H50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:H50),1)</f>
+        <v/>
+      </c>
+      <c r="AI50" s="120" t="n"/>
+      <c r="AJ50" s="121" t="n"/>
+      <c r="AK50" s="120" t="n"/>
+      <c r="AL50" s="121" t="n"/>
+      <c r="AM50" s="120" t="n"/>
+      <c r="AN50" s="121" t="n"/>
+      <c r="AO50" s="120" t="n"/>
+      <c r="AP50" s="121" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>El sushino</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="68">
+        <f>SUM(G51:H51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="68">
+        <f>ROUND(AVERAGE(G51:H51),1)</f>
+        <v/>
+      </c>
+      <c r="AI51" s="120" t="n"/>
+      <c r="AJ51" s="121" t="n"/>
+      <c r="AK51" s="120" t="n"/>
+      <c r="AL51" s="121" t="n"/>
+      <c r="AM51" s="120" t="n"/>
+      <c r="AN51" s="121" t="n"/>
+      <c r="AO51" s="120" t="n"/>
+      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-15
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ42"/>
+  <dimension ref="A1:CJ46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18678,13 +18678,13 @@
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -18824,13 +18824,13 @@
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5" s="68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="68">
         <f>SUM(G5:H5)</f>
@@ -19324,13 +19324,13 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19340,11 +19340,15 @@
         <f>ROUND(AVERAGE(G9:H9),1)</f>
         <v/>
       </c>
-      <c r="G9" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="80" t="n">
-        <v>3</v>
+      <c r="G9" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H9" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I9" s="79" t="n">
         <v>3</v>
@@ -19604,13 +19608,13 @@
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19620,11 +19624,15 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="Q12" s="79" t="n">
         <v>3</v>
@@ -20198,13 +20206,13 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -20312,13 +20320,13 @@
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C18" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E18" s="68">
         <f>SUM(G18:H18)</f>
@@ -20328,11 +20336,15 @@
         <f>ROUND(AVERAGE(G18:H18),1)</f>
         <v/>
       </c>
-      <c r="G18" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" t="n">
-        <v>3</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I18" s="79" t="n">
         <v>2</v>
@@ -20462,13 +20474,13 @@
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C19" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -20478,8 +20490,10 @@
         <f>ROUND(AVERAGE(G19:H19),1)</f>
         <v/>
       </c>
-      <c r="G19" s="79" t="n">
-        <v>3</v>
+      <c r="G19" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="H19" s="80" t="inlineStr">
         <is>
@@ -20664,13 +20678,13 @@
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E20" s="68">
         <f>SUM(G20:H20)</f>
@@ -21526,13 +21540,13 @@
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E28" s="68">
         <f>SUM(G28:H28)</f>
@@ -21542,11 +21556,15 @@
         <f>ROUND(AVERAGE(G28:H28),1)</f>
         <v/>
       </c>
-      <c r="G28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="80" t="n">
-        <v>3</v>
+      <c r="G28" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H28" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I28" s="79" t="n">
         <v>2</v>
@@ -21968,13 +21986,13 @@
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -22108,13 +22126,13 @@
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -22150,13 +22168,13 @@
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C36" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="68">
         <f>SUM(G36:H36)</f>
@@ -22165,6 +22183,16 @@
       <c r="F36" s="68">
         <f>ROUND(AVERAGE(G36:H36),1)</f>
         <v/>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI36" s="120" t="n"/>
       <c r="AJ36" s="121" t="n"/>
@@ -22278,13 +22306,13 @@
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22293,6 +22321,16 @@
       <c r="F40" s="68">
         <f>ROUND(AVERAGE(G40:H40),1)</f>
         <v/>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI40" s="120" t="n"/>
       <c r="AJ40" s="121" t="n"/>
@@ -22342,13 +22380,13 @@
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22376,6 +22414,144 @@
       <c r="AN42" s="121" t="n"/>
       <c r="AO42" s="120" t="n"/>
       <c r="AP42" s="121" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="79" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="B43" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="68">
+        <f>SUM(G43:H43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="68">
+        <f>ROUND(AVERAGE(G43:H43),1)</f>
+        <v/>
+      </c>
+      <c r="AI43" s="120" t="n"/>
+      <c r="AJ43" s="121" t="n"/>
+      <c r="AK43" s="120" t="n"/>
+      <c r="AL43" s="121" t="n"/>
+      <c r="AM43" s="120" t="n"/>
+      <c r="AN43" s="121" t="n"/>
+      <c r="AO43" s="120" t="n"/>
+      <c r="AP43" s="121" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="79" t="inlineStr">
+        <is>
+          <t>Space_GG</t>
+        </is>
+      </c>
+      <c r="B44" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="68">
+        <f>SUM(G44:H44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="68">
+        <f>ROUND(AVERAGE(G44:H44),1)</f>
+        <v/>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI44" s="120" t="n"/>
+      <c r="AJ44" s="121" t="n"/>
+      <c r="AK44" s="120" t="n"/>
+      <c r="AL44" s="121" t="n"/>
+      <c r="AM44" s="120" t="n"/>
+      <c r="AN44" s="121" t="n"/>
+      <c r="AO44" s="120" t="n"/>
+      <c r="AP44" s="121" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="79" t="inlineStr">
+        <is>
+          <t>jehoshua</t>
+        </is>
+      </c>
+      <c r="B45" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="68">
+        <f>SUM(G45:H45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="68">
+        <f>ROUND(AVERAGE(G45:H45),1)</f>
+        <v/>
+      </c>
+      <c r="AI45" s="120" t="n"/>
+      <c r="AJ45" s="121" t="n"/>
+      <c r="AK45" s="120" t="n"/>
+      <c r="AL45" s="121" t="n"/>
+      <c r="AM45" s="120" t="n"/>
+      <c r="AN45" s="121" t="n"/>
+      <c r="AO45" s="120" t="n"/>
+      <c r="AP45" s="121" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="79" t="inlineStr">
+        <is>
+          <t>Matrox☆ita</t>
+        </is>
+      </c>
+      <c r="B46" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="68">
+        <f>SUM(G46:H46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="68">
+        <f>ROUND(AVERAGE(G46:H46),1)</f>
+        <v/>
+      </c>
+      <c r="AI46" s="120" t="n"/>
+      <c r="AJ46" s="121" t="n"/>
+      <c r="AK46" s="120" t="n"/>
+      <c r="AL46" s="121" t="n"/>
+      <c r="AM46" s="120" t="n"/>
+      <c r="AN46" s="121" t="n"/>
+      <c r="AO46" s="120" t="n"/>
+      <c r="AP46" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-17
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ46"/>
+  <dimension ref="A1:CJ45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18678,13 +18678,13 @@
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -19502,13 +19502,13 @@
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E10" s="68">
         <f>SUM(G10:H10)</f>
@@ -19760,13 +19760,13 @@
         </is>
       </c>
       <c r="B13" s="79" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C13" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="68">
         <f>SUM(G13:H13)</f>
@@ -19775,6 +19775,16 @@
       <c r="F13" s="68">
         <f>ROUND(AVERAGE(G13:H13),1)</f>
         <v/>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I13" s="79" t="n">
         <v>3</v>
@@ -21540,13 +21550,13 @@
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E28" s="68">
         <f>SUM(G28:H28)</f>
@@ -21760,17 +21770,17 @@
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>zordan</t>
+          <t>Juri</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C29" s="68" t="n">
         <v>2</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E29" s="68">
         <f>SUM(G29:H29)</f>
@@ -21780,106 +21790,30 @@
         <f>ROUND(AVERAGE(G29:H29),1)</f>
         <v/>
       </c>
-      <c r="U29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X29" s="80" t="inlineStr">
+      <c r="AI29" s="120" t="n"/>
+      <c r="AJ29" s="121" t="n"/>
+      <c r="AK29" s="120" t="n"/>
+      <c r="AL29" s="121" t="n"/>
+      <c r="AM29" s="120" t="n"/>
+      <c r="AN29" s="121" t="n"/>
+      <c r="AO29" s="120" t="n"/>
+      <c r="AP29" s="121" t="n"/>
+      <c r="CE29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="Y29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB29" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE29" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF29" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI29" s="120" t="inlineStr">
+      <c r="CF29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ29" s="121" t="inlineStr">
+      <c r="CI29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AK29" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL29" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AM29" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN29" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO29" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP29" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY29" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ29" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA29" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD29" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE29" t="n">
-        <v>2</v>
-      </c>
-      <c r="BF29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BQ29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR29" t="inlineStr">
+      <c r="CJ29" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -21888,17 +21822,17 @@
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>Juri</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -21916,22 +21850,12 @@
       <c r="AN30" s="121" t="n"/>
       <c r="AO30" s="120" t="n"/>
       <c r="AP30" s="121" t="n"/>
-      <c r="CE30" t="inlineStr">
+      <c r="CC30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CF30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CJ30" t="inlineStr">
+      <c r="CD30" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -21940,17 +21864,17 @@
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C31" s="68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E31" s="68">
         <f>SUM(G31:H31)</f>
@@ -21959,6 +21883,16 @@
       <c r="F31" s="68">
         <f>ROUND(AVERAGE(G31:H31),1)</f>
         <v/>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI31" s="120" t="n"/>
       <c r="AJ31" s="121" t="n"/>
@@ -21968,31 +21902,45 @@
       <c r="AN31" s="121" t="n"/>
       <c r="AO31" s="120" t="n"/>
       <c r="AP31" s="121" t="n"/>
-      <c r="CC31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD31" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="CA31" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB31" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE31" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF31" t="n">
+        <v>2</v>
+      </c>
+      <c r="CI31" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -22020,45 +21968,21 @@
       <c r="AN32" s="121" t="n"/>
       <c r="AO32" s="120" t="n"/>
       <c r="AP32" s="121" t="n"/>
-      <c r="CA32" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB32" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC32" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD32" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE32" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF32" t="n">
-        <v>2</v>
-      </c>
-      <c r="CI32" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ32" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C33" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="68">
         <f>SUM(G33:H33)</f>
@@ -22067,16 +21991,6 @@
       <c r="F33" s="68">
         <f>ROUND(AVERAGE(G33:H33),1)</f>
         <v/>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI33" s="120" t="n"/>
       <c r="AJ33" s="121" t="n"/>
@@ -22090,17 +22004,17 @@
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C34" s="68" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D34" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E34" s="68">
         <f>SUM(G34:H34)</f>
@@ -22109,6 +22023,16 @@
       <c r="F34" s="68">
         <f>ROUND(AVERAGE(G34:H34),1)</f>
         <v/>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI34" s="120" t="n"/>
       <c r="AJ34" s="121" t="n"/>
@@ -22122,7 +22046,7 @@
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
@@ -22164,17 +22088,17 @@
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>El sushino</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C36" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E36" s="68">
         <f>SUM(G36:H36)</f>
@@ -22183,16 +22107,6 @@
       <c r="F36" s="68">
         <f>ROUND(AVERAGE(G36:H36),1)</f>
         <v/>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI36" s="120" t="n"/>
       <c r="AJ36" s="121" t="n"/>
@@ -22206,7 +22120,7 @@
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>El sushino</t>
+          <t>i love nutella</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
@@ -22238,17 +22152,17 @@
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>DJ Tony</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -22257,6 +22171,16 @@
       <c r="F38" s="68">
         <f>ROUND(AVERAGE(G38:H38),1)</f>
         <v/>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -22270,7 +22194,7 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
@@ -22302,17 +22226,17 @@
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22344,17 +22268,17 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>Space_GG</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="68">
         <f>SUM(G41:H41)</f>
@@ -22363,6 +22287,16 @@
       <c r="F41" s="68">
         <f>ROUND(AVERAGE(G41:H41),1)</f>
         <v/>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI41" s="120" t="n"/>
       <c r="AJ41" s="121" t="n"/>
@@ -22376,17 +22310,17 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22395,16 +22329,6 @@
       <c r="F42" s="68">
         <f>ROUND(AVERAGE(G42:H42),1)</f>
         <v/>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI42" s="120" t="n"/>
       <c r="AJ42" s="121" t="n"/>
@@ -22418,17 +22342,17 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>Bruno</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C43" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="68">
         <f>SUM(G43:H43)</f>
@@ -22437,6 +22361,16 @@
       <c r="F43" s="68">
         <f>ROUND(AVERAGE(G43:H43),1)</f>
         <v/>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI43" s="120" t="n"/>
       <c r="AJ43" s="121" t="n"/>
@@ -22450,7 +22384,7 @@
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -22492,17 +22426,17 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C45" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="68">
         <f>SUM(G45:H45)</f>
@@ -22511,6 +22445,16 @@
       <c r="F45" s="68">
         <f>ROUND(AVERAGE(G45:H45),1)</f>
         <v/>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI45" s="120" t="n"/>
       <c r="AJ45" s="121" t="n"/>
@@ -22520,38 +22464,6 @@
       <c r="AN45" s="121" t="n"/>
       <c r="AO45" s="120" t="n"/>
       <c r="AP45" s="121" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="79" t="inlineStr">
-        <is>
-          <t>Matrox☆ita</t>
-        </is>
-      </c>
-      <c r="B46" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="68">
-        <f>SUM(G46:H46)</f>
-        <v/>
-      </c>
-      <c r="F46" s="68">
-        <f>ROUND(AVERAGE(G46:H46),1)</f>
-        <v/>
-      </c>
-      <c r="AI46" s="120" t="n"/>
-      <c r="AJ46" s="121" t="n"/>
-      <c r="AK46" s="120" t="n"/>
-      <c r="AL46" s="121" t="n"/>
-      <c r="AM46" s="120" t="n"/>
-      <c r="AN46" s="121" t="n"/>
-      <c r="AO46" s="120" t="n"/>
-      <c r="AP46" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-22
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ44"/>
+  <dimension ref="A1:CJ49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18622,13 +18622,13 @@
         </is>
       </c>
       <c r="B3" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -18638,11 +18638,15 @@
         <f>ROUND(AVERAGE(G3:H3),1)</f>
         <v/>
       </c>
-      <c r="G3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H3" t="n">
-        <v>3</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -19264,13 +19268,13 @@
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C8" s="68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -19442,13 +19446,13 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19458,11 +19462,15 @@
         <f>ROUND(AVERAGE(G9:H9),1)</f>
         <v/>
       </c>
-      <c r="G9" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" t="n">
-        <v>3</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -19544,13 +19552,13 @@
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C11" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E11" s="68">
         <f>SUM(G11:H11)</f>
@@ -19696,13 +19704,13 @@
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19712,11 +19720,15 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>3</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I12" s="79" t="n">
         <v>3</v>
@@ -20148,13 +20160,13 @@
         </is>
       </c>
       <c r="B16" s="79" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C16" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E16" s="68">
         <f>SUM(G16:H16)</f>
@@ -20262,13 +20274,13 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -20620,13 +20632,13 @@
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C19" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -20794,13 +20806,13 @@
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="68">
         <f>SUM(G20:H20)</f>
@@ -20810,11 +20822,15 @@
         <f>ROUND(AVERAGE(G20:H20),1)</f>
         <v/>
       </c>
-      <c r="G20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" t="n">
-        <v>3</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I20" s="79" t="n">
         <v>3</v>
@@ -21744,13 +21760,13 @@
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C29" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E29" s="68">
         <f>SUM(G29:H29)</f>
@@ -21760,11 +21776,15 @@
         <f>ROUND(AVERAGE(G29:H29),1)</f>
         <v/>
       </c>
-      <c r="G29" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" t="n">
-        <v>3</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI29" s="120" t="n"/>
       <c r="AJ29" s="121" t="n"/>
@@ -21806,13 +21826,13 @@
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -21880,13 +21900,13 @@
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -21896,11 +21916,15 @@
         <f>ROUND(AVERAGE(G32:H32),1)</f>
         <v/>
       </c>
-      <c r="G32" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" t="n">
-        <v>3</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI32" s="120" t="n"/>
       <c r="AJ32" s="121" t="n"/>
@@ -22094,13 +22118,13 @@
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -22250,13 +22274,13 @@
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22266,11 +22290,15 @@
         <f>ROUND(AVERAGE(G42:H42),1)</f>
         <v/>
       </c>
-      <c r="G42" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" t="n">
-        <v>1</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI42" s="120" t="n"/>
       <c r="AJ42" s="121" t="n"/>
@@ -22326,13 +22354,13 @@
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="68">
         <f>SUM(G44:H44)</f>
@@ -22341,6 +22369,16 @@
       <c r="F44" s="68">
         <f>ROUND(AVERAGE(G44:H44),1)</f>
         <v/>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI44" s="120" t="n"/>
       <c r="AJ44" s="121" t="n"/>
@@ -22350,6 +22388,166 @@
       <c r="AN44" s="121" t="n"/>
       <c r="AO44" s="120" t="n"/>
       <c r="AP44" s="121" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="79" t="inlineStr">
+        <is>
+          <t>Breso</t>
+        </is>
+      </c>
+      <c r="B45" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="68">
+        <f>SUM(G45:H45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="68">
+        <f>ROUND(AVERAGE(G45:H45),1)</f>
+        <v/>
+      </c>
+      <c r="AI45" s="120" t="n"/>
+      <c r="AJ45" s="121" t="n"/>
+      <c r="AK45" s="120" t="n"/>
+      <c r="AL45" s="121" t="n"/>
+      <c r="AM45" s="120" t="n"/>
+      <c r="AN45" s="121" t="n"/>
+      <c r="AO45" s="120" t="n"/>
+      <c r="AP45" s="121" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="79" t="inlineStr">
+        <is>
+          <t>escanor</t>
+        </is>
+      </c>
+      <c r="B46" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="68">
+        <f>SUM(G46:H46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="68">
+        <f>ROUND(AVERAGE(G46:H46),1)</f>
+        <v/>
+      </c>
+      <c r="AI46" s="120" t="n"/>
+      <c r="AJ46" s="121" t="n"/>
+      <c r="AK46" s="120" t="n"/>
+      <c r="AL46" s="121" t="n"/>
+      <c r="AM46" s="120" t="n"/>
+      <c r="AN46" s="121" t="n"/>
+      <c r="AO46" s="120" t="n"/>
+      <c r="AP46" s="121" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="79" t="inlineStr">
+        <is>
+          <t>zpercu</t>
+        </is>
+      </c>
+      <c r="B47" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="68">
+        <f>SUM(G47:H47)</f>
+        <v/>
+      </c>
+      <c r="F47" s="68">
+        <f>ROUND(AVERAGE(G47:H47),1)</f>
+        <v/>
+      </c>
+      <c r="AI47" s="120" t="n"/>
+      <c r="AJ47" s="121" t="n"/>
+      <c r="AK47" s="120" t="n"/>
+      <c r="AL47" s="121" t="n"/>
+      <c r="AM47" s="120" t="n"/>
+      <c r="AN47" s="121" t="n"/>
+      <c r="AO47" s="120" t="n"/>
+      <c r="AP47" s="121" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="79" t="inlineStr">
+        <is>
+          <t>Z☆PAINKILLER☆Z</t>
+        </is>
+      </c>
+      <c r="B48" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="68">
+        <f>SUM(G48:H48)</f>
+        <v/>
+      </c>
+      <c r="F48" s="68">
+        <f>ROUND(AVERAGE(G48:H48),1)</f>
+        <v/>
+      </c>
+      <c r="AI48" s="120" t="n"/>
+      <c r="AJ48" s="121" t="n"/>
+      <c r="AK48" s="120" t="n"/>
+      <c r="AL48" s="121" t="n"/>
+      <c r="AM48" s="120" t="n"/>
+      <c r="AN48" s="121" t="n"/>
+      <c r="AO48" s="120" t="n"/>
+      <c r="AP48" s="121" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="79" t="inlineStr">
+        <is>
+          <t>ARES</t>
+        </is>
+      </c>
+      <c r="B49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="68">
+        <f>SUM(G49:H49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="68">
+        <f>ROUND(AVERAGE(G49:H49),1)</f>
+        <v/>
+      </c>
+      <c r="AI49" s="120" t="n"/>
+      <c r="AJ49" s="121" t="n"/>
+      <c r="AK49" s="120" t="n"/>
+      <c r="AL49" s="121" t="n"/>
+      <c r="AM49" s="120" t="n"/>
+      <c r="AN49" s="121" t="n"/>
+      <c r="AO49" s="120" t="n"/>
+      <c r="AP49" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-24
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ49"/>
+  <dimension ref="A1:CJ51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18628,7 +18628,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -18638,15 +18638,11 @@
         <f>ROUND(AVERAGE(G3:H3),1)</f>
         <v/>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -19274,7 +19270,7 @@
         <v>6</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -19284,15 +19280,11 @@
         <f>ROUND(AVERAGE(G8:H8),1)</f>
         <v/>
       </c>
-      <c r="G8" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H8" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I8" s="79" t="n">
         <v>3</v>
@@ -19452,7 +19444,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19462,15 +19454,11 @@
         <f>ROUND(AVERAGE(G9:H9),1)</f>
         <v/>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -19552,13 +19540,13 @@
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="68" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E11" s="68">
         <f>SUM(G11:H11)</f>
@@ -19568,10 +19556,8 @@
         <f>ROUND(AVERAGE(G11:H11),1)</f>
         <v/>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G11" t="n">
+        <v>3</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -19710,7 +19696,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19720,15 +19706,11 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
       </c>
       <c r="I12" s="79" t="n">
         <v>3</v>
@@ -20166,7 +20148,7 @@
         <v>4</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E16" s="68">
         <f>SUM(G16:H16)</f>
@@ -20176,15 +20158,11 @@
         <f>ROUND(AVERAGE(G16:H16),1)</f>
         <v/>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
       </c>
       <c r="AM16" s="68" t="n"/>
       <c r="AN16" s="68" t="n"/>
@@ -20274,13 +20252,13 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -20638,7 +20616,7 @@
         <v>5</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -20648,15 +20626,11 @@
         <f>ROUND(AVERAGE(G19:H19),1)</f>
         <v/>
       </c>
-      <c r="G19" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H19" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I19" s="79" t="n">
         <v>2</v>
@@ -20812,7 +20786,7 @@
         <v>3</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E20" s="68">
         <f>SUM(G20:H20)</f>
@@ -20822,15 +20796,11 @@
         <f>ROUND(AVERAGE(G20:H20),1)</f>
         <v/>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3</v>
       </c>
       <c r="I20" s="79" t="n">
         <v>3</v>
@@ -21766,7 +21736,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E29" s="68">
         <f>SUM(G29:H29)</f>
@@ -21776,15 +21746,11 @@
         <f>ROUND(AVERAGE(G29:H29),1)</f>
         <v/>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2</v>
       </c>
       <c r="AI29" s="120" t="n"/>
       <c r="AJ29" s="121" t="n"/>
@@ -21826,13 +21792,13 @@
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -21906,7 +21872,7 @@
         <v>4</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -21916,15 +21882,11 @@
         <f>ROUND(AVERAGE(G32:H32),1)</f>
         <v/>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3</v>
       </c>
       <c r="AI32" s="120" t="n"/>
       <c r="AJ32" s="121" t="n"/>
@@ -22008,17 +21970,17 @@
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>i love nutella</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -22027,6 +21989,16 @@
       <c r="F35" s="68">
         <f>ROUND(AVERAGE(G35:H35),1)</f>
         <v/>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI35" s="120" t="n"/>
       <c r="AJ35" s="121" t="n"/>
@@ -22040,17 +22012,17 @@
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>cesadjsocc</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C36" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E36" s="68">
         <f>SUM(G36:H36)</f>
@@ -22059,16 +22031,6 @@
       <c r="F36" s="68">
         <f>ROUND(AVERAGE(G36:H36),1)</f>
         <v/>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI36" s="120" t="n"/>
       <c r="AJ36" s="121" t="n"/>
@@ -22082,17 +22044,17 @@
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>cesadjsocc</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C37" s="68" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E37" s="68">
         <f>SUM(G37:H37)</f>
@@ -22101,6 +22063,14 @@
       <c r="F37" s="68">
         <f>ROUND(AVERAGE(G37:H37),1)</f>
         <v/>
+      </c>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI37" s="120" t="n"/>
       <c r="AJ37" s="121" t="n"/>
@@ -22114,17 +22084,17 @@
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>jehoshua</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -22133,16 +22103,6 @@
       <c r="F38" s="68">
         <f>ROUND(AVERAGE(G38:H38),1)</f>
         <v/>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -22156,17 +22116,17 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>Space_GG</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C39" s="68" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" s="68">
         <f>SUM(G39:H39)</f>
@@ -22176,10 +22136,8 @@
         <f>ROUND(AVERAGE(G39:H39),1)</f>
         <v/>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G39" t="n">
+        <v>2</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -22198,17 +22156,17 @@
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22217,6 +22175,14 @@
       <c r="F40" s="68">
         <f>ROUND(AVERAGE(G40:H40),1)</f>
         <v/>
+      </c>
+      <c r="G40" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI40" s="120" t="n"/>
       <c r="AJ40" s="121" t="n"/>
@@ -22230,11 +22196,11 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C41" s="68" t="n">
         <v>1</v>
@@ -22251,12 +22217,10 @@
         <v/>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2</v>
       </c>
       <c r="AI41" s="120" t="n"/>
       <c r="AJ41" s="121" t="n"/>
@@ -22270,7 +22234,7 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>Frost Walker</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
@@ -22280,7 +22244,7 @@
         <v>2</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22312,17 +22276,17 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>Breso</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C43" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E43" s="68">
         <f>SUM(G43:H43)</f>
@@ -22331,12 +22295,6 @@
       <c r="F43" s="68">
         <f>ROUND(AVERAGE(G43:H43),1)</f>
         <v/>
-      </c>
-      <c r="G43" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" t="n">
-        <v>2</v>
       </c>
       <c r="AI43" s="120" t="n"/>
       <c r="AJ43" s="121" t="n"/>
@@ -22350,17 +22308,17 @@
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>escanor</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C44" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E44" s="68">
         <f>SUM(G44:H44)</f>
@@ -22369,16 +22327,6 @@
       <c r="F44" s="68">
         <f>ROUND(AVERAGE(G44:H44),1)</f>
         <v/>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI44" s="120" t="n"/>
       <c r="AJ44" s="121" t="n"/>
@@ -22392,7 +22340,7 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>Breso</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -22424,7 +22372,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>Z☆PAINKILLER☆Z</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -22456,7 +22404,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -22488,7 +22436,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>Z☆PAINKILLER☆Z</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -22520,7 +22468,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>Mini Golem</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -22548,6 +22496,70 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>KingAleGolem03</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:H50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:H50),1)</f>
+        <v/>
+      </c>
+      <c r="AI50" s="120" t="n"/>
+      <c r="AJ50" s="121" t="n"/>
+      <c r="AK50" s="120" t="n"/>
+      <c r="AL50" s="121" t="n"/>
+      <c r="AM50" s="120" t="n"/>
+      <c r="AN50" s="121" t="n"/>
+      <c r="AO50" s="120" t="n"/>
+      <c r="AP50" s="121" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>cioli03</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="68">
+        <f>SUM(G51:H51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="68">
+        <f>ROUND(AVERAGE(G51:H51),1)</f>
+        <v/>
+      </c>
+      <c r="AI51" s="120" t="n"/>
+      <c r="AJ51" s="121" t="n"/>
+      <c r="AK51" s="120" t="n"/>
+      <c r="AL51" s="121" t="n"/>
+      <c r="AM51" s="120" t="n"/>
+      <c r="AN51" s="121" t="n"/>
+      <c r="AO51" s="120" t="n"/>
+      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-26
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ51"/>
+  <dimension ref="A1:CJ49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18622,13 +18622,13 @@
         </is>
       </c>
       <c r="B3" s="79" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" s="68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -18638,11 +18638,15 @@
         <f>ROUND(AVERAGE(G3:H3),1)</f>
         <v/>
       </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="n">
-        <v>3</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -18764,13 +18768,13 @@
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -19264,13 +19268,13 @@
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C8" s="68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -19280,11 +19284,15 @@
         <f>ROUND(AVERAGE(G8:H8),1)</f>
         <v/>
       </c>
-      <c r="G8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="80" t="n">
-        <v>3</v>
+      <c r="G8" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H8" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I8" s="79" t="n">
         <v>3</v>
@@ -19438,13 +19446,13 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19454,11 +19462,15 @@
         <f>ROUND(AVERAGE(G9:H9),1)</f>
         <v/>
       </c>
-      <c r="G9" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" t="n">
-        <v>3</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -19690,13 +19702,13 @@
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19706,11 +19718,15 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>3</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I12" s="79" t="n">
         <v>3</v>
@@ -20252,13 +20268,13 @@
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -21468,13 +21484,13 @@
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E27" s="68">
         <f>SUM(G27:H27)</f>
@@ -21484,11 +21500,15 @@
         <f>ROUND(AVERAGE(G27:H27),1)</f>
         <v/>
       </c>
-      <c r="G27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="80" t="n">
-        <v>3</v>
+      <c r="G27" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H27" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I27" s="79" t="n">
         <v>2</v>
@@ -21792,13 +21812,13 @@
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C30" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -21866,13 +21886,13 @@
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -21882,11 +21902,15 @@
         <f>ROUND(AVERAGE(G32:H32),1)</f>
         <v/>
       </c>
-      <c r="G32" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" t="n">
-        <v>3</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI32" s="120" t="n"/>
       <c r="AJ32" s="121" t="n"/>
@@ -21904,13 +21928,13 @@
         </is>
       </c>
       <c r="B33" s="79" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="79" t="n">
         <v>4</v>
-      </c>
-      <c r="C33" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" s="79" t="n">
-        <v>3</v>
       </c>
       <c r="E33" s="68">
         <f>SUM(G33:H33)</f>
@@ -21920,11 +21944,15 @@
         <f>ROUND(AVERAGE(G33:H33),1)</f>
         <v/>
       </c>
-      <c r="G33" t="n">
-        <v>3</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI33" s="120" t="n"/>
       <c r="AJ33" s="121" t="n"/>
@@ -21974,13 +22002,13 @@
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -22048,13 +22076,13 @@
         </is>
       </c>
       <c r="B37" s="79" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C37" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E37" s="68">
         <f>SUM(G37:H37)</f>
@@ -22064,8 +22092,10 @@
         <f>ROUND(AVERAGE(G37:H37),1)</f>
         <v/>
       </c>
-      <c r="G37" t="n">
-        <v>3</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -22160,13 +22190,13 @@
         </is>
       </c>
       <c r="B40" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="79" t="n">
         <v>5</v>
-      </c>
-      <c r="C40" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="79" t="n">
-        <v>4</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22176,8 +22206,10 @@
         <f>ROUND(AVERAGE(G40:H40),1)</f>
         <v/>
       </c>
-      <c r="G40" t="n">
-        <v>3</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -22200,13 +22232,13 @@
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="68">
         <f>SUM(G41:H41)</f>
@@ -22216,11 +22248,15 @@
         <f>ROUND(AVERAGE(G41:H41),1)</f>
         <v/>
       </c>
-      <c r="G41" t="n">
-        <v>1</v>
-      </c>
-      <c r="H41" t="n">
-        <v>2</v>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI41" s="120" t="n"/>
       <c r="AJ41" s="121" t="n"/>
@@ -22238,13 +22274,13 @@
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22372,7 +22408,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>Z☆PAINKILLER☆Z</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -22404,7 +22440,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>Mini Golem</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -22436,7 +22472,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>KingAleGolem03</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -22468,7 +22504,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>Mini Golem</t>
+          <t>cioli03</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -22496,70 +22532,6 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="79" t="inlineStr">
-        <is>
-          <t>KingAleGolem03</t>
-        </is>
-      </c>
-      <c r="B50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="68">
-        <f>SUM(G50:H50)</f>
-        <v/>
-      </c>
-      <c r="F50" s="68">
-        <f>ROUND(AVERAGE(G50:H50),1)</f>
-        <v/>
-      </c>
-      <c r="AI50" s="120" t="n"/>
-      <c r="AJ50" s="121" t="n"/>
-      <c r="AK50" s="120" t="n"/>
-      <c r="AL50" s="121" t="n"/>
-      <c r="AM50" s="120" t="n"/>
-      <c r="AN50" s="121" t="n"/>
-      <c r="AO50" s="120" t="n"/>
-      <c r="AP50" s="121" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="79" t="inlineStr">
-        <is>
-          <t>cioli03</t>
-        </is>
-      </c>
-      <c r="B51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="68">
-        <f>SUM(G51:H51)</f>
-        <v/>
-      </c>
-      <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:H51),1)</f>
-        <v/>
-      </c>
-      <c r="AI51" s="120" t="n"/>
-      <c r="AJ51" s="121" t="n"/>
-      <c r="AK51" s="120" t="n"/>
-      <c r="AL51" s="121" t="n"/>
-      <c r="AM51" s="120" t="n"/>
-      <c r="AN51" s="121" t="n"/>
-      <c r="AO51" s="120" t="n"/>
-      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-28
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ49"/>
+  <dimension ref="A1:CJ51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18628,7 +18628,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -18638,15 +18638,11 @@
         <f>ROUND(AVERAGE(G3:H3),1)</f>
         <v/>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -18774,7 +18770,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -18784,15 +18780,11 @@
         <f>ROUND(AVERAGE(G4:H4),1)</f>
         <v/>
       </c>
-      <c r="G4" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H4" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G4" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I4" s="79" t="n">
         <v>0</v>
@@ -19274,7 +19266,7 @@
         <v>7</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -19284,15 +19276,11 @@
         <f>ROUND(AVERAGE(G8:H8),1)</f>
         <v/>
       </c>
-      <c r="G8" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H8" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G8" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="80" t="n">
+        <v>2</v>
       </c>
       <c r="I8" s="79" t="n">
         <v>3</v>
@@ -19452,7 +19440,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19462,15 +19450,11 @@
         <f>ROUND(AVERAGE(G9:H9),1)</f>
         <v/>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -19708,7 +19692,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19718,15 +19702,11 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
       </c>
       <c r="I12" s="79" t="n">
         <v>3</v>
@@ -20274,7 +20254,7 @@
         <v>5</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -20284,15 +20264,11 @@
         <f>ROUND(AVERAGE(G17:H17),1)</f>
         <v/>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
       </c>
       <c r="I17" s="79" t="n">
         <v>2</v>
@@ -21490,7 +21466,7 @@
         <v>10</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E27" s="68">
         <f>SUM(G27:H27)</f>
@@ -21500,15 +21476,11 @@
         <f>ROUND(AVERAGE(G27:H27),1)</f>
         <v/>
       </c>
-      <c r="G27" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H27" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G27" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="I27" s="79" t="n">
         <v>2</v>
@@ -21818,7 +21790,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -21828,15 +21800,11 @@
         <f>ROUND(AVERAGE(G30:H30),1)</f>
         <v/>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G30" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
       </c>
       <c r="AI30" s="120" t="n"/>
       <c r="AJ30" s="121" t="n"/>
@@ -21892,7 +21860,7 @@
         <v>5</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -21902,15 +21870,11 @@
         <f>ROUND(AVERAGE(G32:H32),1)</f>
         <v/>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3</v>
       </c>
       <c r="AI32" s="120" t="n"/>
       <c r="AJ32" s="121" t="n"/>
@@ -21934,7 +21898,7 @@
         <v>3</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" s="68">
         <f>SUM(G33:H33)</f>
@@ -21944,15 +21908,11 @@
         <f>ROUND(AVERAGE(G33:H33),1)</f>
         <v/>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
       </c>
       <c r="AI33" s="120" t="n"/>
       <c r="AJ33" s="121" t="n"/>
@@ -22002,13 +21962,13 @@
         </is>
       </c>
       <c r="B35" s="79" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C35" s="68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -22082,7 +22042,7 @@
         <v>4</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" s="68">
         <f>SUM(G37:H37)</f>
@@ -22092,15 +22052,11 @@
         <f>ROUND(AVERAGE(G37:H37),1)</f>
         <v/>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3</v>
       </c>
       <c r="AI37" s="120" t="n"/>
       <c r="AJ37" s="121" t="n"/>
@@ -22114,17 +22070,17 @@
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>jehoshua</t>
+          <t>Matrox☆ita</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C38" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -22133,6 +22089,14 @@
       <c r="F38" s="68">
         <f>ROUND(AVERAGE(G38:H38),1)</f>
         <v/>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -22146,17 +22110,17 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>Matrox☆ita</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C39" s="68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E39" s="68">
         <f>SUM(G39:H39)</f>
@@ -22186,17 +22150,17 @@
     <row r="40">
       <c r="A40" s="79" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>fre 2000</t>
         </is>
       </c>
       <c r="B40" s="79" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C40" s="68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22206,15 +22170,11 @@
         <f>ROUND(AVERAGE(G40:H40),1)</f>
         <v/>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2</v>
       </c>
       <c r="AI40" s="120" t="n"/>
       <c r="AJ40" s="121" t="n"/>
@@ -22228,17 +22188,17 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>fre 2000</t>
+          <t>Frost Walker</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" s="68" t="n">
         <v>4</v>
       </c>
-      <c r="C41" s="68" t="n">
-        <v>2</v>
-      </c>
       <c r="D41" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E41" s="68">
         <f>SUM(G41:H41)</f>
@@ -22270,17 +22230,17 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>escanor</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C42" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D42" s="79" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E42" s="68">
         <f>SUM(G42:H42)</f>
@@ -22289,16 +22249,6 @@
       <c r="F42" s="68">
         <f>ROUND(AVERAGE(G42:H42),1)</f>
         <v/>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI42" s="120" t="n"/>
       <c r="AJ42" s="121" t="n"/>
@@ -22312,7 +22262,7 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>Breso</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -22344,7 +22294,7 @@
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -22376,7 +22326,7 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>KingAleGolem03</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -22408,7 +22358,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>ale mugna</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -22440,7 +22390,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>Mini Golem</t>
+          <t>ale 12</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -22472,7 +22422,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>KingAleGolem03</t>
+          <t>marcobeltra._</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -22504,7 +22454,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>cioli03</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -22532,6 +22482,70 @@
       <c r="AN49" s="121" t="n"/>
       <c r="AO49" s="120" t="n"/>
       <c r="AP49" s="121" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>vito</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="68">
+        <f>SUM(G50:H50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="68">
+        <f>ROUND(AVERAGE(G50:H50),1)</f>
+        <v/>
+      </c>
+      <c r="AI50" s="120" t="n"/>
+      <c r="AJ50" s="121" t="n"/>
+      <c r="AK50" s="120" t="n"/>
+      <c r="AL50" s="121" t="n"/>
+      <c r="AM50" s="120" t="n"/>
+      <c r="AN50" s="121" t="n"/>
+      <c r="AO50" s="120" t="n"/>
+      <c r="AP50" s="121" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>rasim01</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="68">
+        <f>SUM(G51:H51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="68">
+        <f>ROUND(AVERAGE(G51:H51),1)</f>
+        <v/>
+      </c>
+      <c r="AI51" s="120" t="n"/>
+      <c r="AJ51" s="121" t="n"/>
+      <c r="AK51" s="120" t="n"/>
+      <c r="AL51" s="121" t="n"/>
+      <c r="AM51" s="120" t="n"/>
+      <c r="AN51" s="121" t="n"/>
+      <c r="AO51" s="120" t="n"/>
+      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-05-31
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -18091,7 +18091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ51"/>
+  <dimension ref="A1:CJ50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -18628,7 +18628,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -18642,7 +18642,7 @@
         <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -18770,7 +18770,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -18784,7 +18784,7 @@
         <v>2</v>
       </c>
       <c r="H4" s="80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I4" s="79" t="n">
         <v>0</v>
@@ -18996,7 +18996,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="68">
         <f>SUM(G5:H5)</f>
@@ -19005,6 +19005,12 @@
       <c r="F5" s="68">
         <f>ROUND(AVERAGE(G5:H5),1)</f>
         <v/>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
       </c>
       <c r="K5" s="79" t="n">
         <v>3</v>
@@ -19130,13 +19136,13 @@
         </is>
       </c>
       <c r="B7" s="79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C7" s="68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="68">
         <f>SUM(G7:H7)</f>
@@ -19146,11 +19152,15 @@
         <f>ROUND(AVERAGE(G7:H7),1)</f>
         <v/>
       </c>
-      <c r="G7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" t="n">
-        <v>2</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AM7" t="n">
         <v>1</v>
@@ -19260,13 +19270,13 @@
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" s="68" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -19279,8 +19289,10 @@
       <c r="G8" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="80" t="n">
-        <v>2</v>
+      <c r="H8" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I8" s="79" t="n">
         <v>3</v>
@@ -19440,7 +19452,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -19451,10 +19463,10 @@
         <v/>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -19692,7 +19704,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -19874,7 +19886,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E13" s="68">
         <f>SUM(G13:H13)</f>
@@ -19883,6 +19895,12 @@
       <c r="F13" s="68">
         <f>ROUND(AVERAGE(G13:H13),1)</f>
         <v/>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
       </c>
       <c r="S13" s="79" t="n">
         <v>2</v>
@@ -20144,7 +20162,7 @@
         <v>4</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E16" s="68">
         <f>SUM(G16:H16)</f>
@@ -20158,7 +20176,7 @@
         <v>2</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM16" s="68" t="n"/>
       <c r="AN16" s="68" t="n"/>
@@ -20254,7 +20272,7 @@
         <v>5</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -20265,10 +20283,10 @@
         <v/>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I17" s="79" t="n">
         <v>2</v>
@@ -20398,13 +20416,13 @@
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="68" t="n">
         <v>3</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E18" s="68">
         <f>SUM(G18:H18)</f>
@@ -20414,10 +20432,8 @@
         <f>ROUND(AVERAGE(G18:H18),1)</f>
         <v/>
       </c>
-      <c r="G18" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G18" s="79" t="n">
+        <v>3</v>
       </c>
       <c r="H18" s="80" t="inlineStr">
         <is>
@@ -20608,7 +20624,7 @@
         <v>5</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -21460,13 +21476,13 @@
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" s="68" t="n">
         <v>10</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E27" s="68">
         <f>SUM(G27:H27)</f>
@@ -21477,10 +21493,12 @@
         <v/>
       </c>
       <c r="G27" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="H27" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I27" s="79" t="n">
         <v>2</v>
@@ -21728,7 +21746,7 @@
         <v>4</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E29" s="68">
         <f>SUM(G29:H29)</f>
@@ -21739,7 +21757,7 @@
         <v/>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
@@ -21860,7 +21878,7 @@
         <v>5</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -21968,7 +21986,7 @@
         <v>3</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -21978,15 +21996,11 @@
         <f>ROUND(AVERAGE(G35:H35),1)</f>
         <v/>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="G35" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2</v>
       </c>
       <c r="AI35" s="120" t="n"/>
       <c r="AJ35" s="121" t="n"/>
@@ -22080,7 +22094,7 @@
         <v>1</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -22093,10 +22107,8 @@
       <c r="G38" t="n">
         <v>2</v>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="H38" t="n">
+        <v>2</v>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -22114,13 +22126,13 @@
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C39" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E39" s="68">
         <f>SUM(G39:H39)</f>
@@ -22130,8 +22142,10 @@
         <f>ROUND(AVERAGE(G39:H39),1)</f>
         <v/>
       </c>
-      <c r="G39" t="n">
-        <v>2</v>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -22160,7 +22174,7 @@
         <v>2</v>
       </c>
       <c r="D40" s="79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" s="68">
         <f>SUM(G40:H40)</f>
@@ -22188,17 +22202,17 @@
     <row r="41">
       <c r="A41" s="79" t="inlineStr">
         <is>
-          <t>Frost Walker</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B41" s="79" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C41" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D41" s="79" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E41" s="68">
         <f>SUM(G41:H41)</f>
@@ -22207,16 +22221,6 @@
       <c r="F41" s="68">
         <f>ROUND(AVERAGE(G41:H41),1)</f>
         <v/>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI41" s="120" t="n"/>
       <c r="AJ41" s="121" t="n"/>
@@ -22230,7 +22234,7 @@
     <row r="42">
       <c r="A42" s="79" t="inlineStr">
         <is>
-          <t>escanor</t>
+          <t>SgherroMutante</t>
         </is>
       </c>
       <c r="B42" s="79" t="n">
@@ -22262,7 +22266,7 @@
     <row r="43">
       <c r="A43" s="79" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>KingAleGolem03</t>
         </is>
       </c>
       <c r="B43" s="79" t="n">
@@ -22294,7 +22298,7 @@
     <row r="44">
       <c r="A44" s="79" t="inlineStr">
         <is>
-          <t>SgherroMutante</t>
+          <t>ale mugna</t>
         </is>
       </c>
       <c r="B44" s="79" t="n">
@@ -22326,7 +22330,7 @@
     <row r="45">
       <c r="A45" s="79" t="inlineStr">
         <is>
-          <t>KingAleGolem03</t>
+          <t>ale 12</t>
         </is>
       </c>
       <c r="B45" s="79" t="n">
@@ -22358,7 +22362,7 @@
     <row r="46">
       <c r="A46" s="79" t="inlineStr">
         <is>
-          <t>ale mugna</t>
+          <t>marcobeltra._</t>
         </is>
       </c>
       <c r="B46" s="79" t="n">
@@ -22390,7 +22394,7 @@
     <row r="47">
       <c r="A47" s="79" t="inlineStr">
         <is>
-          <t>ale 12</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B47" s="79" t="n">
@@ -22400,7 +22404,7 @@
         <v>0</v>
       </c>
       <c r="D47" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="68">
         <f>SUM(G47:H47)</f>
@@ -22409,6 +22413,12 @@
       <c r="F47" s="68">
         <f>ROUND(AVERAGE(G47:H47),1)</f>
         <v/>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2</v>
       </c>
       <c r="AI47" s="120" t="n"/>
       <c r="AJ47" s="121" t="n"/>
@@ -22422,7 +22432,7 @@
     <row r="48">
       <c r="A48" s="79" t="inlineStr">
         <is>
-          <t>marcobeltra._</t>
+          <t>vito</t>
         </is>
       </c>
       <c r="B48" s="79" t="n">
@@ -22454,7 +22464,7 @@
     <row r="49">
       <c r="A49" s="79" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B49" s="79" t="n">
@@ -22486,7 +22496,7 @@
     <row r="50">
       <c r="A50" s="79" t="inlineStr">
         <is>
-          <t>vito</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B50" s="79" t="n">
@@ -22514,38 +22524,6 @@
       <c r="AN50" s="121" t="n"/>
       <c r="AO50" s="120" t="n"/>
       <c r="AP50" s="121" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="79" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="68">
-        <f>SUM(G51:H51)</f>
-        <v/>
-      </c>
-      <c r="F51" s="68">
-        <f>ROUND(AVERAGE(G51:H51),1)</f>
-        <v/>
-      </c>
-      <c r="AI51" s="120" t="n"/>
-      <c r="AJ51" s="121" t="n"/>
-      <c r="AK51" s="120" t="n"/>
-      <c r="AL51" s="121" t="n"/>
-      <c r="AM51" s="120" t="n"/>
-      <c r="AN51" s="121" t="n"/>
-      <c r="AO51" s="120" t="n"/>
-      <c r="AP51" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-06-17
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -3388,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ40"/>
+  <dimension ref="A1:CJ39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -3925,7 +3925,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -3936,7 +3936,7 @@
         <v/>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>3</v>
@@ -4293,7 +4293,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="68">
         <f>SUM(G5:H5)</f>
@@ -4307,7 +4307,7 @@
         <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" s="79" t="n">
         <v>3</v>
@@ -4743,13 +4743,13 @@
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="68" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -4760,10 +4760,12 @@
         <v/>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BO9" t="n">
         <v>3</v>
@@ -5001,7 +5003,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -5012,7 +5014,7 @@
         <v/>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
         <v>3</v>
@@ -6425,17 +6427,17 @@
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>Stentaaa</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E23" s="68">
         <f>SUM(G23:H23)</f>
@@ -6445,127 +6447,27 @@
         <f>ROUND(AVERAGE(G23:H23),1)</f>
         <v/>
       </c>
-      <c r="G23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="M23" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O23" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="R23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y23" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z23" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA23" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB23" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI23" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ23" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK23" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL23" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM23" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN23" s="121" t="n">
-        <v>3</v>
-      </c>
       <c r="AS23" s="120" t="n">
         <v>3</v>
       </c>
       <c r="AT23" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BM23" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BO23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BS23" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT23" t="n">
-        <v>2</v>
-      </c>
-      <c r="CA23" t="n">
-        <v>1</v>
-      </c>
-      <c r="CB23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="C24" s="68" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" s="68">
         <f>SUM(G24:H24)</f>
@@ -6575,27 +6477,221 @@
         <f>ROUND(AVERAGE(G24:H24),1)</f>
         <v/>
       </c>
+      <c r="G24" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H24" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="I24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L24" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="O24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA24" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB24" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC24" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD24" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI24" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ24" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK24" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL24" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM24" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN24" s="121" t="n">
+        <v>3</v>
+      </c>
       <c r="AS24" s="120" t="n">
         <v>3</v>
       </c>
       <c r="AT24" s="121" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AU24" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV24" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BR24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BU24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV24" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ24" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E25" s="68">
         <f>SUM(G25:H25)</f>
@@ -6605,200 +6701,20 @@
         <f>ROUND(AVERAGE(G25:H25),1)</f>
         <v/>
       </c>
-      <c r="G25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" s="80" t="inlineStr">
+      <c r="AI25" s="120" t="n"/>
+      <c r="AJ25" s="121" t="n"/>
+      <c r="AK25" s="120" t="n"/>
+      <c r="AL25" s="121" t="n"/>
+      <c r="AM25" s="120" t="n"/>
+      <c r="AN25" s="121" t="n"/>
+      <c r="AO25" s="120" t="n"/>
+      <c r="AP25" s="121" t="n"/>
+      <c r="CC25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="I25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K25" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L25" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P25" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T25" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA25" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB25" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC25" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD25" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI25" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ25" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK25" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL25" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM25" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN25" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS25" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT25" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU25" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV25" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BM25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP25" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BS25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BT25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BU25" t="n">
-        <v>2</v>
-      </c>
-      <c r="BV25" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="CD25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CJ25" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -6807,17 +6723,17 @@
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>Anto</t>
         </is>
       </c>
       <c r="B26" s="79" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C26" s="68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E26" s="68">
         <f>SUM(G26:H26)</f>
@@ -6826,6 +6742,14 @@
       <c r="F26" s="68">
         <f>ROUND(AVERAGE(G26:H26),1)</f>
         <v/>
+      </c>
+      <c r="G26" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI26" s="120" t="n"/>
       <c r="AJ26" s="121" t="n"/>
@@ -6835,31 +6759,45 @@
       <c r="AN26" s="121" t="n"/>
       <c r="AO26" s="120" t="n"/>
       <c r="AP26" s="121" t="n"/>
-      <c r="CC26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="CA26" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB26" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD26" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE26" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF26" t="n">
+        <v>2</v>
+      </c>
+      <c r="CI26" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" s="68" t="n">
         <v>4</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E27" s="68">
         <f>SUM(G27:H27)</f>
@@ -6872,10 +6810,8 @@
       <c r="G27" t="n">
         <v>3</v>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="H27" t="n">
+        <v>2</v>
       </c>
       <c r="AI27" s="120" t="n"/>
       <c r="AJ27" s="121" t="n"/>
@@ -6885,45 +6821,21 @@
       <c r="AN27" s="121" t="n"/>
       <c r="AO27" s="120" t="n"/>
       <c r="AP27" s="121" t="n"/>
-      <c r="CA27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC27" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD27" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF27" t="n">
-        <v>2</v>
-      </c>
-      <c r="CI27" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ27" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C28" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E28" s="68">
         <f>SUM(G28:H28)</f>
@@ -6937,7 +6849,7 @@
         <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI28" s="120" t="n"/>
       <c r="AJ28" s="121" t="n"/>
@@ -6951,17 +6863,17 @@
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B29" s="79" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C29" s="68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29" s="79" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E29" s="68">
         <f>SUM(G29:H29)</f>
@@ -6970,6 +6882,12 @@
       <c r="F29" s="68">
         <f>ROUND(AVERAGE(G29:H29),1)</f>
         <v/>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3</v>
       </c>
       <c r="AI29" s="120" t="n"/>
       <c r="AJ29" s="121" t="n"/>
@@ -6983,17 +6901,17 @@
     <row r="30">
       <c r="A30" s="79" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Francesco10</t>
         </is>
       </c>
       <c r="B30" s="79" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C30" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="79" t="n">
         <v>5</v>
-      </c>
-      <c r="D30" s="79" t="n">
-        <v>10</v>
       </c>
       <c r="E30" s="68">
         <f>SUM(G30:H30)</f>
@@ -7004,10 +6922,10 @@
         <v/>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI30" s="120" t="n"/>
       <c r="AJ30" s="121" t="n"/>
@@ -7021,7 +6939,7 @@
     <row r="31">
       <c r="A31" s="79" t="inlineStr">
         <is>
-          <t>Francesco10</t>
+          <t>roberto</t>
         </is>
       </c>
       <c r="B31" s="79" t="n">
@@ -7031,7 +6949,7 @@
         <v>3</v>
       </c>
       <c r="D31" s="79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="68">
         <f>SUM(G31:H31)</f>
@@ -7042,10 +6960,10 @@
         <v/>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI31" s="120" t="n"/>
       <c r="AJ31" s="121" t="n"/>
@@ -7059,17 +6977,17 @@
     <row r="32">
       <c r="A32" s="79" t="inlineStr">
         <is>
-          <t>roberto</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B32" s="79" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C32" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" s="79" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E32" s="68">
         <f>SUM(G32:H32)</f>
@@ -7080,10 +6998,10 @@
         <v/>
       </c>
       <c r="G32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI32" s="120" t="n"/>
       <c r="AJ32" s="121" t="n"/>
@@ -7097,17 +7015,17 @@
     <row r="33">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>KAIZERS</t>
         </is>
       </c>
       <c r="B33" s="79" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C33" s="68" t="n">
         <v>4</v>
       </c>
       <c r="D33" s="79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E33" s="68">
         <f>SUM(G33:H33)</f>
@@ -7117,11 +7035,15 @@
         <f>ROUND(AVERAGE(G33:H33),1)</f>
         <v/>
       </c>
-      <c r="G33" t="n">
-        <v>3</v>
-      </c>
-      <c r="H33" t="n">
-        <v>3</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI33" s="120" t="n"/>
       <c r="AJ33" s="121" t="n"/>
@@ -7135,17 +7057,17 @@
     <row r="34">
       <c r="A34" s="79" t="inlineStr">
         <is>
-          <t>KAIZERS</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B34" s="79" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C34" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D34" s="79" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E34" s="68">
         <f>SUM(G34:H34)</f>
@@ -7154,16 +7076,6 @@
       <c r="F34" s="68">
         <f>ROUND(AVERAGE(G34:H34),1)</f>
         <v/>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI34" s="120" t="n"/>
       <c r="AJ34" s="121" t="n"/>
@@ -7177,7 +7089,7 @@
     <row r="35">
       <c r="A35" s="79" t="inlineStr">
         <is>
-          <t>zpercu</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B35" s="79" t="n">
@@ -7187,7 +7099,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" s="68">
         <f>SUM(G35:H35)</f>
@@ -7196,6 +7108,12 @@
       <c r="F35" s="68">
         <f>ROUND(AVERAGE(G35:H35),1)</f>
         <v/>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2</v>
       </c>
       <c r="AI35" s="120" t="n"/>
       <c r="AJ35" s="121" t="n"/>
@@ -7209,14 +7127,14 @@
     <row r="36">
       <c r="A36" s="79" t="inlineStr">
         <is>
-          <t>maragno</t>
+          <t>rasim01</t>
         </is>
       </c>
       <c r="B36" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C36" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" s="79" t="n">
         <v>1</v>
@@ -7229,11 +7147,15 @@
         <f>ROUND(AVERAGE(G36:H36),1)</f>
         <v/>
       </c>
-      <c r="G36" t="n">
-        <v>2</v>
-      </c>
-      <c r="H36" t="n">
-        <v>2</v>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI36" s="120" t="n"/>
       <c r="AJ36" s="121" t="n"/>
@@ -7247,17 +7169,17 @@
     <row r="37">
       <c r="A37" s="79" t="inlineStr">
         <is>
-          <t>rasim01</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B37" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C37" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" s="68">
         <f>SUM(G37:H37)</f>
@@ -7266,16 +7188,6 @@
       <c r="F37" s="68">
         <f>ROUND(AVERAGE(G37:H37),1)</f>
         <v/>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI37" s="120" t="n"/>
       <c r="AJ37" s="121" t="n"/>
@@ -7289,17 +7201,17 @@
     <row r="38">
       <c r="A38" s="79" t="inlineStr">
         <is>
-          <t>Akemi</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B38" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E38" s="68">
         <f>SUM(G38:H38)</f>
@@ -7308,6 +7220,12 @@
       <c r="F38" s="68">
         <f>ROUND(AVERAGE(G38:H38),1)</f>
         <v/>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
       </c>
       <c r="AI38" s="120" t="n"/>
       <c r="AJ38" s="121" t="n"/>
@@ -7321,17 +7239,17 @@
     <row r="39">
       <c r="A39" s="79" t="inlineStr">
         <is>
-          <t>Elatanvsb108</t>
+          <t>vTrxzys</t>
         </is>
       </c>
       <c r="B39" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C39" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="68">
         <f>SUM(G39:H39)</f>
@@ -7340,14 +7258,6 @@
       <c r="F39" s="68">
         <f>ROUND(AVERAGE(G39:H39),1)</f>
         <v/>
-      </c>
-      <c r="G39" t="n">
-        <v>3</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
       </c>
       <c r="AI39" s="120" t="n"/>
       <c r="AJ39" s="121" t="n"/>
@@ -7357,38 +7267,6 @@
       <c r="AN39" s="121" t="n"/>
       <c r="AO39" s="120" t="n"/>
       <c r="AP39" s="121" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="79" t="inlineStr">
-        <is>
-          <t>vTrxzys</t>
-        </is>
-      </c>
-      <c r="B40" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="68">
-        <f>SUM(G40:H40)</f>
-        <v/>
-      </c>
-      <c r="F40" s="68">
-        <f>ROUND(AVERAGE(G40:H40),1)</f>
-        <v/>
-      </c>
-      <c r="AI40" s="120" t="n"/>
-      <c r="AJ40" s="121" t="n"/>
-      <c r="AK40" s="120" t="n"/>
-      <c r="AL40" s="121" t="n"/>
-      <c r="AM40" s="120" t="n"/>
-      <c r="AN40" s="121" t="n"/>
-      <c r="AO40" s="120" t="n"/>
-      <c r="AP40" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">
@@ -22222,9 +22100,9 @@
     <col hidden="1" width="9.140625" customWidth="1" min="34" max="34"/>
     <col hidden="1" width="12.85546875" customWidth="1" min="36" max="36"/>
     <col hidden="1" width="9.140625" customWidth="1" style="157" min="37" max="37"/>
-    <col hidden="1" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" min="38" max="38"/>
     <col hidden="1" width="9.140625" customWidth="1" style="157" min="39" max="39"/>
-    <col hidden="1" min="40" max="40"/>
+    <col hidden="1" width="13" customWidth="1" min="40" max="40"/>
     <col width="14.85546875" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Update WAR data - 2026-07-15
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -3388,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ39"/>
+  <dimension ref="A1:CJ28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -3925,7 +3925,7 @@
         <v>6</v>
       </c>
       <c r="D3" s="79" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="68">
         <f>SUM(G3:H3)</f>
@@ -3936,10 +3936,10 @@
         <v/>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM3" t="n">
         <v>3</v>
@@ -4057,17 +4057,17 @@
     <row r="4">
       <c r="A4" s="79" t="inlineStr">
         <is>
-          <t>BigMc23</t>
+          <t>buff x-bow</t>
         </is>
       </c>
       <c r="B4" s="79" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="C4" s="68" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D4" s="79" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E4" s="68">
         <f>SUM(G4:H4)</f>
@@ -4077,223 +4077,109 @@
         <f>ROUND(AVERAGE(G4:H4),1)</f>
         <v/>
       </c>
-      <c r="G4" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="80" t="n">
-        <v>0</v>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
       </c>
       <c r="K4" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L4" s="80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M4" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N4" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="R4" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W4" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="X4" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Y4" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z4" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA4" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB4" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC4" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AD4" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI4" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ4" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK4" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL4" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AM4" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN4" s="121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO4" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP4" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AU4" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AV4" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AY4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AZ4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BA4" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="Q4" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC4" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD4" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI4" s="68" t="n"/>
+      <c r="AJ4" s="68" t="n"/>
+      <c r="AK4" s="68" t="n"/>
+      <c r="AL4" s="68" t="n"/>
+      <c r="AM4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU4" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV4" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>3</v>
       </c>
       <c r="BE4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF4" t="n">
         <v>3</v>
       </c>
-      <c r="BI4" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>2</v>
-      </c>
-      <c r="BO4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP4" t="n">
-        <v>2</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="BG4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>2</v>
       </c>
       <c r="BU4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BV4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY4" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>3</v>
       </c>
       <c r="CC4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CD4" t="n">
         <v>3</v>
       </c>
       <c r="CE4" t="n">
-        <v>1</v>
-      </c>
-      <c r="CF4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="CF4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="79" t="inlineStr">
         <is>
-          <t>buff x-bow</t>
+          <t>Chabby</t>
         </is>
       </c>
       <c r="B5" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="79" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E5" s="68">
         <f>SUM(G5:H5)</f>
@@ -4303,109 +4189,31 @@
         <f>ROUND(AVERAGE(G5:H5),1)</f>
         <v/>
       </c>
-      <c r="G5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L5" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q5" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R5" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC5" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD5" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI5" s="68" t="n"/>
-      <c r="AJ5" s="68" t="n"/>
-      <c r="AK5" s="68" t="n"/>
-      <c r="AL5" s="68" t="n"/>
-      <c r="AM5" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU5" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV5" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH5" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE5" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF5" t="n">
-        <v>3</v>
+      <c r="AS5" s="68" t="n"/>
+      <c r="AT5" s="68" t="n"/>
+      <c r="BA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="79" t="inlineStr">
         <is>
-          <t>Chabby</t>
+          <t>cucco</t>
         </is>
       </c>
       <c r="B6" s="79" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C6" s="68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" s="79" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E6" s="68">
         <f>SUM(G6:H6)</f>
@@ -4415,31 +4223,129 @@
         <f>ROUND(AVERAGE(G6:H6),1)</f>
         <v/>
       </c>
-      <c r="AS6" s="68" t="n"/>
-      <c r="AT6" s="68" t="n"/>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>2</v>
+      </c>
       <c r="BA6" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB6" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW6" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
+      </c>
+      <c r="BX6" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="79" t="inlineStr">
         <is>
-          <t>cucco</t>
+          <t>Edoardo9</t>
         </is>
       </c>
       <c r="B7" s="79" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" s="68" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="68" t="n">
-        <v>2</v>
-      </c>
       <c r="D7" s="79" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" s="68">
         <f>SUM(G7:H7)</f>
@@ -4449,104 +4355,50 @@
         <f>ROUND(AVERAGE(G7:H7),1)</f>
         <v/>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="BO7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AM7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>2</v>
-      </c>
-      <c r="BC7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BD7" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK7" t="n">
-        <v>2</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ7" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR7" t="n">
-        <v>2</v>
-      </c>
       <c r="BS7" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT7" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BU7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BV7" t="n">
         <v>3</v>
       </c>
-      <c r="BW7" t="inlineStr">
+      <c r="CA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB7" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BX7" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY7" t="n">
-        <v>2</v>
-      </c>
-      <c r="BZ7" t="n">
-        <v>2</v>
-      </c>
       <c r="CC7" t="n">
         <v>3</v>
       </c>
@@ -4554,26 +4406,26 @@
         <v>3</v>
       </c>
       <c r="CI7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CJ7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="79" t="inlineStr">
         <is>
-          <t>dado</t>
+          <t>EdoDodo</t>
         </is>
       </c>
       <c r="B8" s="79" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C8" s="68" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D8" s="79" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E8" s="68">
         <f>SUM(G8:H8)</f>
@@ -4583,173 +4435,21 @@
         <f>ROUND(AVERAGE(G8:H8),1)</f>
         <v/>
       </c>
-      <c r="G8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="S8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="U8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W8" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y8" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB8" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC8" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD8" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI8" s="68" t="n"/>
-      <c r="AJ8" s="68" t="n"/>
-      <c r="AK8" s="68" t="n"/>
-      <c r="AL8" s="68" t="n"/>
-      <c r="AM8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO8" s="68" t="n"/>
-      <c r="AP8" s="68" t="n"/>
-      <c r="AS8" s="68" t="n"/>
-      <c r="AT8" s="68" t="n"/>
-      <c r="AU8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BH8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BM8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BN8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BQ8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR8" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU8" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV8" t="n">
-        <v>2</v>
-      </c>
-      <c r="CE8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF8" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI8" t="n">
-        <v>2</v>
-      </c>
-      <c r="CJ8" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="79" t="inlineStr">
         <is>
-          <t>Edoardo9</t>
+          <t>Floky23</t>
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C9" s="68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -4767,69 +4467,139 @@
           <t>SKIP</t>
         </is>
       </c>
+      <c r="Q9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R9" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="U9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V9" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z9" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AE9" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF9" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" s="68" t="n"/>
+      <c r="AJ9" s="68" t="n"/>
+      <c r="AK9" s="68" t="n"/>
+      <c r="AL9" s="68" t="n"/>
+      <c r="AS9" s="120" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT9" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BL9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="BO9" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP9" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BQ9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR9" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BS9" t="n">
-        <v>3</v>
-      </c>
-      <c r="BT9" t="inlineStr">
+      <c r="BX9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BU9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BV9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB9" t="inlineStr">
+      <c r="BY9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CC9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD9" t="n">
-        <v>3</v>
-      </c>
       <c r="CI9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CJ9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="79" t="inlineStr">
         <is>
-          <t>EdoDodo</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E10" s="68">
         <f>SUM(G10:H10)</f>
@@ -4839,21 +4609,179 @@
         <f>ROUND(AVERAGE(G10:H10),1)</f>
         <v/>
       </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="U10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="V10" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD10" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF10" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI10" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ10" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK10" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL10" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO10" s="120" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP10" s="121" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS10" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT10" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU10" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV10" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BC10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BX10" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BY10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C11" s="68" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" s="68">
         <f>SUM(G11:H11)</f>
@@ -4866,108 +4794,112 @@
       <c r="G11" t="n">
         <v>3</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="S11" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W11" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X11" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC11" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD11" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI11" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="Q11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R11" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="U11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V11" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z11" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB11" s="80" t="inlineStr">
+      <c r="AJ11" s="121" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AE11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF11" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI11" s="68" t="n"/>
-      <c r="AJ11" s="68" t="n"/>
-      <c r="AK11" s="68" t="n"/>
-      <c r="AL11" s="68" t="n"/>
-      <c r="AS11" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT11" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AY11" t="inlineStr">
+      <c r="AK11" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL11" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM11" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN11" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AZ11" t="inlineStr">
+      <c r="BX11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BK11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BL11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BO11" t="n">
-        <v>2</v>
-      </c>
-      <c r="BP11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BQ11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR11" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BW11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="BY11" t="n">
         <v>3</v>
       </c>
       <c r="BZ11" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>3</v>
       </c>
       <c r="CC11" t="n">
         <v>2</v>
@@ -4978,32 +4910,24 @@
       <c r="CE11" t="n">
         <v>3</v>
       </c>
-      <c r="CF11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ11" t="n">
-        <v>3</v>
+      <c r="CF11" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="79" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -5013,179 +4937,65 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="G12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J12" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P12" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R12" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V12" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB12" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC12" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD12" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE12" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF12" s="80" t="inlineStr">
+      <c r="AI12" s="68" t="n"/>
+      <c r="AJ12" s="68" t="n"/>
+      <c r="AK12" s="68" t="n"/>
+      <c r="AL12" s="68" t="n"/>
+      <c r="AM12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO12" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP12" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU12" s="68" t="n"/>
+      <c r="AV12" s="68" t="n"/>
+      <c r="AY12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF12" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AI12" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ12" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK12" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL12" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO12" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP12" s="121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS12" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT12" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU12" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV12" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BI12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BO12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP12" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX12" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ12" t="n">
-        <v>1</v>
+      <c r="BS12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="79" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="B13" s="79" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="68" t="n">
         <v>4</v>
       </c>
-      <c r="C13" s="68" t="n">
-        <v>2</v>
-      </c>
       <c r="D13" s="79" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13" s="68">
         <f>SUM(G13:H13)</f>
@@ -5199,100 +5009,70 @@
         <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
-      </c>
-      <c r="S13" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W13" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X13" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC13" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD13" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI13" s="120" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="AM13" s="68" t="n"/>
+      <c r="AN13" s="68" t="n"/>
+      <c r="AO13" s="68" t="n"/>
+      <c r="AP13" s="68" t="n"/>
+      <c r="AS13" s="68" t="n"/>
+      <c r="AT13" s="68" t="n"/>
+      <c r="AU13" s="68" t="n"/>
+      <c r="AV13" s="68" t="n"/>
+      <c r="BC13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ13" s="121" t="inlineStr">
+      <c r="BG13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AK13" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL13" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM13" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN13" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BS13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BT13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW13" t="inlineStr">
+      <c r="BX13" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BX13" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="BY13" t="n">
         <v>3</v>
       </c>
@@ -5300,38 +5080,32 @@
         <v>3</v>
       </c>
       <c r="CA13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CB13" t="n">
         <v>3</v>
       </c>
-      <c r="CC13" t="n">
-        <v>2</v>
-      </c>
-      <c r="CD13" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE13" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF13" t="n">
-        <v>2</v>
+      <c r="CI13" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C14" s="68" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="E14" s="68">
         <f>SUM(G14:H14)</f>
@@ -5341,65 +5115,151 @@
         <f>ROUND(AVERAGE(G14:H14),1)</f>
         <v/>
       </c>
-      <c r="AI14" s="68" t="n"/>
-      <c r="AJ14" s="68" t="n"/>
-      <c r="AK14" s="68" t="n"/>
-      <c r="AL14" s="68" t="n"/>
-      <c r="AM14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO14" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP14" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU14" s="68" t="n"/>
-      <c r="AV14" s="68" t="n"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="I14" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="M14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W14" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X14" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB14" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC14" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM14" s="68" t="n"/>
+      <c r="AN14" s="68" t="n"/>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS14" s="68" t="n"/>
+      <c r="AT14" s="68" t="n"/>
+      <c r="AU14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>1</v>
+      </c>
       <c r="AY14" t="n">
         <v>3</v>
       </c>
       <c r="AZ14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF14" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BS14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT14" t="n">
+      <c r="CF14" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ14" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B15" s="79" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C15" s="68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E15" s="68">
         <f>SUM(G15:H15)</f>
@@ -5409,28 +5269,98 @@
         <f>ROUND(AVERAGE(G15:H15),1)</f>
         <v/>
       </c>
-      <c r="G15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" t="n">
+      <c r="G15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P15" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S15" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T15" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X15" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB15" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AE15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF15" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI15" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ15" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK15" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL15" s="121" t="n">
         <v>3</v>
       </c>
       <c r="AM15" s="68" t="n"/>
       <c r="AN15" s="68" t="n"/>
-      <c r="AO15" s="68" t="n"/>
-      <c r="AP15" s="68" t="n"/>
-      <c r="AS15" s="68" t="n"/>
-      <c r="AT15" s="68" t="n"/>
-      <c r="AU15" s="68" t="n"/>
-      <c r="AV15" s="68" t="n"/>
-      <c r="BC15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD15" t="n">
-        <v>3</v>
+      <c r="AO15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AS15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BE15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF15" t="inlineStr">
         <is>
@@ -5438,34 +5368,32 @@
         </is>
       </c>
       <c r="BG15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BH15" t="n">
-        <v>2</v>
-      </c>
-      <c r="BI15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BK15" t="n">
         <v>3</v>
       </c>
-      <c r="BL15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR15" t="n">
-        <v>2</v>
+      <c r="BL15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>3</v>
       </c>
       <c r="BU15" t="n">
         <v>3</v>
       </c>
-      <c r="BV15" t="n">
-        <v>3</v>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BW15" t="inlineStr">
         <is>
@@ -5480,36 +5408,58 @@
       <c r="BY15" t="n">
         <v>3</v>
       </c>
-      <c r="BZ15" t="n">
-        <v>3</v>
+      <c r="BZ15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="CA15" t="n">
         <v>2</v>
       </c>
-      <c r="CB15" t="n">
-        <v>3</v>
+      <c r="CB15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CC15" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE15" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="CI15" t="n">
         <v>3</v>
       </c>
-      <c r="CJ15" t="n">
-        <v>3</v>
+      <c r="CJ15" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="79" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B16" s="79" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C16" s="68" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E16" s="68">
         <f>SUM(G16:H16)</f>
@@ -5523,27 +5473,37 @@
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="I16" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="J16" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
+      <c r="K16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" s="80" t="n">
+        <v>3</v>
+      </c>
       <c r="M16" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="80" t="n">
         <v>1</v>
       </c>
       <c r="O16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P16" s="80" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="P16" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="Q16" s="79" t="n">
         <v>2</v>
@@ -5554,112 +5514,84 @@
         </is>
       </c>
       <c r="W16" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z16" s="80" t="n">
         <v>2</v>
       </c>
       <c r="AA16" s="79" t="n">
         <v>3</v>
       </c>
       <c r="AB16" s="80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC16" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD16" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM16" s="68" t="n"/>
-      <c r="AN16" s="68" t="n"/>
-      <c r="AO16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS16" s="68" t="n"/>
-      <c r="AT16" s="68" t="n"/>
-      <c r="AU16" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY16" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA16" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB16" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG16" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE16" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF16" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM16" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN16" s="121" t="n">
         <v>2</v>
       </c>
       <c r="BO16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BP16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BS16" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT16" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC16" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD16" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE16" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CF16" t="inlineStr">
+      <c r="BV16" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CI16" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ16" t="n">
-        <v>3</v>
+      <c r="CA16" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -5672,177 +5604,51 @@
       <c r="G17" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="80" t="inlineStr">
+      <c r="H17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU17" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV17" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="I17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J17" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P17" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="S17" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T17" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X17" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB17" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF17" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI17" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ17" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK17" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL17" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM17" s="68" t="n"/>
-      <c r="AN17" s="68" t="n"/>
-      <c r="AO17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AS17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BE17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BG17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BO17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY17" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CA17" t="n">
-        <v>2</v>
-      </c>
-      <c r="CB17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CC17" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE17" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF17" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI17" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ17" t="inlineStr">
+      <c r="BH17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -5851,17 +5657,17 @@
     <row r="18">
       <c r="A18" s="79" t="inlineStr">
         <is>
-          <t>piegian99</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C18" s="68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E18" s="68">
         <f>SUM(G18:H18)</f>
@@ -5871,167 +5677,27 @@
         <f>ROUND(AVERAGE(G18:H18),1)</f>
         <v/>
       </c>
-      <c r="G18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I18" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M18" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="N18" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="O18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V18" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE18" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF18" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI18" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ18" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK18" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL18" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BM18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ18" t="n">
-        <v>2</v>
-      </c>
-      <c r="BR18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BS18" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT18" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU18" t="n">
-        <v>2</v>
-      </c>
-      <c r="BV18" t="n">
-        <v>2</v>
-      </c>
-      <c r="BW18" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX18" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY18" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB18" t="n">
-        <v>2</v>
-      </c>
-      <c r="CC18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF18" t="n">
-        <v>2</v>
-      </c>
-      <c r="CI18" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ18" t="n">
-        <v>3</v>
+      <c r="AS18" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT18" s="121" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>PIPPII</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C19" s="68" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -6041,53 +5707,221 @@
         <f>ROUND(AVERAGE(G19:H19),1)</f>
         <v/>
       </c>
+      <c r="G19" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="I19" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L19" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="O19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P19" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="S19" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T19" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X19" s="80" t="n">
+        <v>3</v>
+      </c>
       <c r="Y19" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="Z19" s="80" t="inlineStr">
+      <c r="Z19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB19" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC19" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD19" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI19" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AC19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE19" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF19" s="80" t="n">
-        <v>3</v>
+      <c r="AJ19" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK19" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL19" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM19" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN19" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS19" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT19" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU19" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV19" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BR19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BU19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BV19" t="n">
-        <v>2</v>
-      </c>
-      <c r="CC19" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD19" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="CC19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ19" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>revolver</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E20" s="68">
         <f>SUM(G20:H20)</f>
@@ -6097,110 +5931,14 @@
         <f>ROUND(AVERAGE(G20:H20),1)</f>
         <v/>
       </c>
-      <c r="S20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="T20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U20" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="V20" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC20" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE20" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF20" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI20" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ20" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK20" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL20" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BC20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD20" t="n">
-        <v>2</v>
-      </c>
-      <c r="BI20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BJ20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BM20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU20" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV20" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA20" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB20" t="n">
-        <v>3</v>
-      </c>
+      <c r="AI20" s="120" t="n"/>
+      <c r="AJ20" s="121" t="n"/>
+      <c r="AK20" s="120" t="n"/>
+      <c r="AL20" s="121" t="n"/>
+      <c r="AM20" s="120" t="n"/>
+      <c r="AN20" s="121" t="n"/>
+      <c r="AO20" s="120" t="n"/>
+      <c r="AP20" s="121" t="n"/>
       <c r="CC20" t="inlineStr">
         <is>
           <t>SKIP</t>
@@ -6215,17 +5953,17 @@
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C21" s="68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E21" s="68">
         <f>SUM(G21:H21)</f>
@@ -6235,133 +5973,35 @@
         <f>ROUND(AVERAGE(G21:H21),1)</f>
         <v/>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I21" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J21" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="K21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M21" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N21" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Q21" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R21" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X21" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z21" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB21" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC21" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD21" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE21" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF21" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM21" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN21" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="BO21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ21" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BU21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV21" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CA21" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB21" t="n">
-        <v>2</v>
-      </c>
+      <c r="G21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI21" s="120" t="n"/>
+      <c r="AJ21" s="121" t="n"/>
+      <c r="AK21" s="120" t="n"/>
+      <c r="AL21" s="121" t="n"/>
+      <c r="AM21" s="120" t="n"/>
+      <c r="AN21" s="121" t="n"/>
+      <c r="AO21" s="120" t="n"/>
+      <c r="AP21" s="121" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>TinoGiusa</t>
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C22" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E22" s="68">
         <f>SUM(G22:H22)</f>
@@ -6371,73 +6011,35 @@
         <f>ROUND(AVERAGE(G22:H22),1)</f>
         <v/>
       </c>
-      <c r="G22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="I22" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J22" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P22" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q22" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R22" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU22" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV22" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE22" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF22" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BH22" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI22" s="120" t="n"/>
+      <c r="AJ22" s="121" t="n"/>
+      <c r="AK22" s="120" t="n"/>
+      <c r="AL22" s="121" t="n"/>
+      <c r="AM22" s="120" t="n"/>
+      <c r="AN22" s="121" t="n"/>
+      <c r="AO22" s="120" t="n"/>
+      <c r="AP22" s="121" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E23" s="68">
         <f>SUM(G23:H23)</f>
@@ -6447,27 +6049,35 @@
         <f>ROUND(AVERAGE(G23:H23),1)</f>
         <v/>
       </c>
-      <c r="AS23" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT23" s="121" t="n">
-        <v>2</v>
-      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI23" s="120" t="n"/>
+      <c r="AJ23" s="121" t="n"/>
+      <c r="AK23" s="120" t="n"/>
+      <c r="AL23" s="121" t="n"/>
+      <c r="AM23" s="120" t="n"/>
+      <c r="AN23" s="121" t="n"/>
+      <c r="AO23" s="120" t="n"/>
+      <c r="AP23" s="121" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C24" s="68" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E24" s="68">
         <f>SUM(G24:H24)</f>
@@ -6477,221 +6087,35 @@
         <f>ROUND(AVERAGE(G24:H24),1)</f>
         <v/>
       </c>
-      <c r="G24" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K24" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L24" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P24" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T24" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA24" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB24" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC24" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD24" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI24" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ24" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK24" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL24" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM24" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN24" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS24" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT24" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU24" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV24" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG24" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL24" t="n">
-        <v>2</v>
-      </c>
-      <c r="BM24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP24" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BS24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BT24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BU24" t="n">
-        <v>2</v>
-      </c>
-      <c r="BV24" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CJ24" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
+      <c r="G24" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI24" s="120" t="n"/>
+      <c r="AJ24" s="121" t="n"/>
+      <c r="AK24" s="120" t="n"/>
+      <c r="AL24" s="121" t="n"/>
+      <c r="AM24" s="120" t="n"/>
+      <c r="AN24" s="121" t="n"/>
+      <c r="AO24" s="120" t="n"/>
+      <c r="AP24" s="121" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>zpercu</t>
         </is>
       </c>
       <c r="B25" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C25" s="68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" s="79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="68">
         <f>SUM(G25:H25)</f>
@@ -6709,31 +6133,21 @@
       <c r="AN25" s="121" t="n"/>
       <c r="AO25" s="120" t="n"/>
       <c r="AP25" s="121" t="n"/>
-      <c r="CC25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD25" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="79" t="inlineStr">
         <is>
-          <t>Anto</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B26" s="79" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C26" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D26" s="79" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E26" s="68">
         <f>SUM(G26:H26)</f>
@@ -6744,7 +6158,7 @@
         <v/>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -6759,45 +6173,21 @@
       <c r="AN26" s="121" t="n"/>
       <c r="AO26" s="120" t="n"/>
       <c r="AP26" s="121" t="n"/>
-      <c r="CA26" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB26" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC26" t="n">
-        <v>1</v>
-      </c>
-      <c r="CD26" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE26" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF26" t="n">
-        <v>2</v>
-      </c>
-      <c r="CI26" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ26" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B27" s="79" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C27" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D27" s="79" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E27" s="68">
         <f>SUM(G27:H27)</f>
@@ -6806,12 +6196,6 @@
       <c r="F27" s="68">
         <f>ROUND(AVERAGE(G27:H27),1)</f>
         <v/>
-      </c>
-      <c r="G27" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" t="n">
-        <v>2</v>
       </c>
       <c r="AI27" s="120" t="n"/>
       <c r="AJ27" s="121" t="n"/>
@@ -6825,17 +6209,17 @@
     <row r="28">
       <c r="A28" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B28" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="68">
         <f>SUM(G28:H28)</f>
@@ -6846,10 +6230,10 @@
         <v/>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI28" s="120" t="n"/>
       <c r="AJ28" s="121" t="n"/>
@@ -6859,414 +6243,6 @@
       <c r="AN28" s="121" t="n"/>
       <c r="AO28" s="120" t="n"/>
       <c r="AP28" s="121" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="79" t="inlineStr">
-        <is>
-          <t>xNullx</t>
-        </is>
-      </c>
-      <c r="B29" s="79" t="n">
-        <v>10</v>
-      </c>
-      <c r="C29" s="68" t="n">
-        <v>5</v>
-      </c>
-      <c r="D29" s="79" t="n">
-        <v>11</v>
-      </c>
-      <c r="E29" s="68">
-        <f>SUM(G29:H29)</f>
-        <v/>
-      </c>
-      <c r="F29" s="68">
-        <f>ROUND(AVERAGE(G29:H29),1)</f>
-        <v/>
-      </c>
-      <c r="G29" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI29" s="120" t="n"/>
-      <c r="AJ29" s="121" t="n"/>
-      <c r="AK29" s="120" t="n"/>
-      <c r="AL29" s="121" t="n"/>
-      <c r="AM29" s="120" t="n"/>
-      <c r="AN29" s="121" t="n"/>
-      <c r="AO29" s="120" t="n"/>
-      <c r="AP29" s="121" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="79" t="inlineStr">
-        <is>
-          <t>Francesco10</t>
-        </is>
-      </c>
-      <c r="B30" s="79" t="n">
-        <v>6</v>
-      </c>
-      <c r="C30" s="68" t="n">
-        <v>3</v>
-      </c>
-      <c r="D30" s="79" t="n">
-        <v>5</v>
-      </c>
-      <c r="E30" s="68">
-        <f>SUM(G30:H30)</f>
-        <v/>
-      </c>
-      <c r="F30" s="68">
-        <f>ROUND(AVERAGE(G30:H30),1)</f>
-        <v/>
-      </c>
-      <c r="G30" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI30" s="120" t="n"/>
-      <c r="AJ30" s="121" t="n"/>
-      <c r="AK30" s="120" t="n"/>
-      <c r="AL30" s="121" t="n"/>
-      <c r="AM30" s="120" t="n"/>
-      <c r="AN30" s="121" t="n"/>
-      <c r="AO30" s="120" t="n"/>
-      <c r="AP30" s="121" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="79" t="inlineStr">
-        <is>
-          <t>roberto</t>
-        </is>
-      </c>
-      <c r="B31" s="79" t="n">
-        <v>6</v>
-      </c>
-      <c r="C31" s="68" t="n">
-        <v>3</v>
-      </c>
-      <c r="D31" s="79" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" s="68">
-        <f>SUM(G31:H31)</f>
-        <v/>
-      </c>
-      <c r="F31" s="68">
-        <f>ROUND(AVERAGE(G31:H31),1)</f>
-        <v/>
-      </c>
-      <c r="G31" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI31" s="120" t="n"/>
-      <c r="AJ31" s="121" t="n"/>
-      <c r="AK31" s="120" t="n"/>
-      <c r="AL31" s="121" t="n"/>
-      <c r="AM31" s="120" t="n"/>
-      <c r="AN31" s="121" t="n"/>
-      <c r="AO31" s="120" t="n"/>
-      <c r="AP31" s="121" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="79" t="inlineStr">
-        <is>
-          <t>fhhgggf</t>
-        </is>
-      </c>
-      <c r="B32" s="79" t="n">
-        <v>9</v>
-      </c>
-      <c r="C32" s="68" t="n">
-        <v>4</v>
-      </c>
-      <c r="D32" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="E32" s="68">
-        <f>SUM(G32:H32)</f>
-        <v/>
-      </c>
-      <c r="F32" s="68">
-        <f>ROUND(AVERAGE(G32:H32),1)</f>
-        <v/>
-      </c>
-      <c r="G32" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI32" s="120" t="n"/>
-      <c r="AJ32" s="121" t="n"/>
-      <c r="AK32" s="120" t="n"/>
-      <c r="AL32" s="121" t="n"/>
-      <c r="AM32" s="120" t="n"/>
-      <c r="AN32" s="121" t="n"/>
-      <c r="AO32" s="120" t="n"/>
-      <c r="AP32" s="121" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="79" t="inlineStr">
-        <is>
-          <t>KAIZERS</t>
-        </is>
-      </c>
-      <c r="B33" s="79" t="n">
-        <v>10</v>
-      </c>
-      <c r="C33" s="68" t="n">
-        <v>4</v>
-      </c>
-      <c r="D33" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="E33" s="68">
-        <f>SUM(G33:H33)</f>
-        <v/>
-      </c>
-      <c r="F33" s="68">
-        <f>ROUND(AVERAGE(G33:H33),1)</f>
-        <v/>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI33" s="120" t="n"/>
-      <c r="AJ33" s="121" t="n"/>
-      <c r="AK33" s="120" t="n"/>
-      <c r="AL33" s="121" t="n"/>
-      <c r="AM33" s="120" t="n"/>
-      <c r="AN33" s="121" t="n"/>
-      <c r="AO33" s="120" t="n"/>
-      <c r="AP33" s="121" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="79" t="inlineStr">
-        <is>
-          <t>zpercu</t>
-        </is>
-      </c>
-      <c r="B34" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="68">
-        <f>SUM(G34:H34)</f>
-        <v/>
-      </c>
-      <c r="F34" s="68">
-        <f>ROUND(AVERAGE(G34:H34),1)</f>
-        <v/>
-      </c>
-      <c r="AI34" s="120" t="n"/>
-      <c r="AJ34" s="121" t="n"/>
-      <c r="AK34" s="120" t="n"/>
-      <c r="AL34" s="121" t="n"/>
-      <c r="AM34" s="120" t="n"/>
-      <c r="AN34" s="121" t="n"/>
-      <c r="AO34" s="120" t="n"/>
-      <c r="AP34" s="121" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="79" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B35" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" s="68">
-        <f>SUM(G35:H35)</f>
-        <v/>
-      </c>
-      <c r="F35" s="68">
-        <f>ROUND(AVERAGE(G35:H35),1)</f>
-        <v/>
-      </c>
-      <c r="G35" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI35" s="120" t="n"/>
-      <c r="AJ35" s="121" t="n"/>
-      <c r="AK35" s="120" t="n"/>
-      <c r="AL35" s="121" t="n"/>
-      <c r="AM35" s="120" t="n"/>
-      <c r="AN35" s="121" t="n"/>
-      <c r="AO35" s="120" t="n"/>
-      <c r="AP35" s="121" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="79" t="inlineStr">
-        <is>
-          <t>rasim01</t>
-        </is>
-      </c>
-      <c r="B36" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="68">
-        <f>SUM(G36:H36)</f>
-        <v/>
-      </c>
-      <c r="F36" s="68">
-        <f>ROUND(AVERAGE(G36:H36),1)</f>
-        <v/>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI36" s="120" t="n"/>
-      <c r="AJ36" s="121" t="n"/>
-      <c r="AK36" s="120" t="n"/>
-      <c r="AL36" s="121" t="n"/>
-      <c r="AM36" s="120" t="n"/>
-      <c r="AN36" s="121" t="n"/>
-      <c r="AO36" s="120" t="n"/>
-      <c r="AP36" s="121" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="79" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B37" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C37" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="68">
-        <f>SUM(G37:H37)</f>
-        <v/>
-      </c>
-      <c r="F37" s="68">
-        <f>ROUND(AVERAGE(G37:H37),1)</f>
-        <v/>
-      </c>
-      <c r="AI37" s="120" t="n"/>
-      <c r="AJ37" s="121" t="n"/>
-      <c r="AK37" s="120" t="n"/>
-      <c r="AL37" s="121" t="n"/>
-      <c r="AM37" s="120" t="n"/>
-      <c r="AN37" s="121" t="n"/>
-      <c r="AO37" s="120" t="n"/>
-      <c r="AP37" s="121" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="79" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B38" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" s="68">
-        <f>SUM(G38:H38)</f>
-        <v/>
-      </c>
-      <c r="F38" s="68">
-        <f>ROUND(AVERAGE(G38:H38),1)</f>
-        <v/>
-      </c>
-      <c r="G38" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI38" s="120" t="n"/>
-      <c r="AJ38" s="121" t="n"/>
-      <c r="AK38" s="120" t="n"/>
-      <c r="AL38" s="121" t="n"/>
-      <c r="AM38" s="120" t="n"/>
-      <c r="AN38" s="121" t="n"/>
-      <c r="AO38" s="120" t="n"/>
-      <c r="AP38" s="121" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="79" t="inlineStr">
-        <is>
-          <t>vTrxzys</t>
-        </is>
-      </c>
-      <c r="B39" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="68">
-        <f>SUM(G39:H39)</f>
-        <v/>
-      </c>
-      <c r="F39" s="68">
-        <f>ROUND(AVERAGE(G39:H39),1)</f>
-        <v/>
-      </c>
-      <c r="AI39" s="120" t="n"/>
-      <c r="AJ39" s="121" t="n"/>
-      <c r="AK39" s="120" t="n"/>
-      <c r="AL39" s="121" t="n"/>
-      <c r="AM39" s="120" t="n"/>
-      <c r="AN39" s="121" t="n"/>
-      <c r="AO39" s="120" t="n"/>
-      <c r="AP39" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>

<commit_message>
Update WAR data - 2026-08-15
</commit_message>
<xml_diff>
--- a/rewards.xlsx
+++ b/rewards.xlsx
@@ -3388,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ28"/>
+  <dimension ref="A1:CJ24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16.42578125" customWidth="1" style="78" min="1" max="1"/>
@@ -4439,17 +4439,17 @@
     <row r="9">
       <c r="A9" s="79" t="inlineStr">
         <is>
-          <t>Floky23</t>
+          <t>GiornoBrando</t>
         </is>
       </c>
       <c r="B9" s="79" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="68" t="n">
         <v>5</v>
       </c>
       <c r="D9" s="79" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="E9" s="68">
         <f>SUM(G9:H9)</f>
@@ -4460,18 +4460,34 @@
         <v/>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P9" s="80" t="n">
+        <v>1</v>
       </c>
       <c r="Q9" s="79" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="79" t="n">
         <v>3</v>
@@ -4479,75 +4495,111 @@
       <c r="V9" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="Y9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z9" s="80" t="n">
-        <v>2</v>
-      </c>
       <c r="AA9" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="AB9" s="80" t="inlineStr">
+      <c r="AB9" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC9" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD9" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE9" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF9" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AE9" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF9" s="80" t="n">
+      <c r="AI9" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ9" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK9" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL9" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO9" s="120" t="n">
         <v>1</v>
       </c>
-      <c r="AI9" s="68" t="n"/>
-      <c r="AJ9" s="68" t="n"/>
-      <c r="AK9" s="68" t="n"/>
-      <c r="AL9" s="68" t="n"/>
+      <c r="AP9" s="121" t="n">
+        <v>1</v>
+      </c>
       <c r="AS9" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT9" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU9" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV9" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA9" t="n">
         <v>1</v>
       </c>
-      <c r="AT9" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AY9" t="inlineStr">
+      <c r="BB9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AZ9" t="inlineStr">
+      <c r="BC9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL9" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BK9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BL9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="BO9" t="n">
-        <v>2</v>
-      </c>
-      <c r="BP9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BQ9" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP9" t="n">
         <v>2</v>
       </c>
       <c r="BU9" t="n">
         <v>3</v>
       </c>
       <c r="BV9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BW9" t="inlineStr">
         <is>
@@ -4565,41 +4617,21 @@
       <c r="BZ9" t="n">
         <v>1</v>
       </c>
-      <c r="CC9" t="n">
-        <v>2</v>
-      </c>
-      <c r="CD9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF9" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI9" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ9" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="79" t="inlineStr">
         <is>
-          <t>GiornoBrando</t>
+          <t>haha</t>
         </is>
       </c>
       <c r="B10" s="79" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C10" s="68" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D10" s="79" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E10" s="68">
         <f>SUM(G10:H10)</f>
@@ -4610,40 +4642,28 @@
         <v/>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
         <v>3</v>
       </c>
-      <c r="I10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="O10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="V10" s="80" t="n">
-        <v>1</v>
+      <c r="S10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T10" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="W10" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X10" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y10" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z10" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="AA10" s="79" t="n">
         <v>3</v>
@@ -4652,136 +4672,112 @@
         <v>3</v>
       </c>
       <c r="AC10" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD10" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE10" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF10" s="80" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AI10" s="120" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AI10" s="120" t="inlineStr">
+      <c r="AJ10" s="121" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ10" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="AK10" s="120" t="n">
         <v>3</v>
       </c>
       <c r="AL10" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO10" s="120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP10" s="121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS10" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT10" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU10" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV10" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM10" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN10" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV10" t="n">
         <v>3</v>
       </c>
       <c r="BA10" t="n">
         <v>1</v>
       </c>
-      <c r="BB10" t="inlineStr">
+      <c r="BB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BC10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BI10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL10" t="inlineStr">
+      <c r="BX10" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BO10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP10" t="n">
-        <v>2</v>
-      </c>
-      <c r="BU10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV10" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX10" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
       <c r="BY10" t="n">
         <v>3</v>
       </c>
       <c r="BZ10" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="79" t="inlineStr">
         <is>
-          <t>haha</t>
+          <t>Kle</t>
         </is>
       </c>
       <c r="B11" s="79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C11" s="68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" s="79" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E11" s="68">
         <f>SUM(G11:H11)</f>
@@ -4791,143 +4787,65 @@
         <f>ROUND(AVERAGE(G11:H11),1)</f>
         <v/>
       </c>
-      <c r="G11" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" t="n">
-        <v>3</v>
-      </c>
-      <c r="S11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T11" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="W11" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="X11" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z11" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB11" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC11" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD11" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI11" s="120" t="inlineStr">
+      <c r="AI11" s="68" t="n"/>
+      <c r="AJ11" s="68" t="n"/>
+      <c r="AK11" s="68" t="n"/>
+      <c r="AL11" s="68" t="n"/>
+      <c r="AM11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO11" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP11" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU11" s="68" t="n"/>
+      <c r="AV11" s="68" t="n"/>
+      <c r="AY11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF11" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="AJ11" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK11" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL11" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM11" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN11" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BB11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR11" t="n">
-        <v>3</v>
-      </c>
       <c r="BS11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BT11" t="n">
         <v>3</v>
-      </c>
-      <c r="BU11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BW11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX11" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY11" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CA11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC11" t="n">
-        <v>2</v>
-      </c>
-      <c r="CD11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE11" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF11" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="79" t="inlineStr">
         <is>
-          <t>Kle</t>
+          <t>Luigi</t>
         </is>
       </c>
       <c r="B12" s="79" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C12" s="68" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D12" s="79" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="E12" s="68">
         <f>SUM(G12:H12)</f>
@@ -4937,65 +4855,151 @@
         <f>ROUND(AVERAGE(G12:H12),1)</f>
         <v/>
       </c>
-      <c r="AI12" s="68" t="n"/>
-      <c r="AJ12" s="68" t="n"/>
-      <c r="AK12" s="68" t="n"/>
-      <c r="AL12" s="68" t="n"/>
-      <c r="AM12" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO12" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP12" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS12" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT12" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU12" s="68" t="n"/>
-      <c r="AV12" s="68" t="n"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="I12" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="M12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="R12" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W12" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="X12" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC12" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD12" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM12" s="68" t="n"/>
+      <c r="AN12" s="68" t="n"/>
+      <c r="AO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS12" s="68" t="n"/>
+      <c r="AT12" s="68" t="n"/>
+      <c r="AU12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>1</v>
+      </c>
       <c r="AY12" t="n">
         <v>3</v>
       </c>
       <c r="AZ12" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE12" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF12" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CE12" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BS12" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT12" t="n">
+      <c r="CF12" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ12" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="79" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>maikol_lix</t>
         </is>
       </c>
       <c r="B13" s="79" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C13" s="68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="79" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E13" s="68">
         <f>SUM(G13:H13)</f>
@@ -5005,28 +5009,98 @@
         <f>ROUND(AVERAGE(G13:H13),1)</f>
         <v/>
       </c>
-      <c r="G13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H13" t="n">
-        <v>2</v>
+      <c r="G13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="S13" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T13" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="W13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X13" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB13" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AE13" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF13" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AI13" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ13" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK13" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL13" s="121" t="n">
+        <v>3</v>
       </c>
       <c r="AM13" s="68" t="n"/>
       <c r="AN13" s="68" t="n"/>
-      <c r="AO13" s="68" t="n"/>
-      <c r="AP13" s="68" t="n"/>
-      <c r="AS13" s="68" t="n"/>
-      <c r="AT13" s="68" t="n"/>
-      <c r="AU13" s="68" t="n"/>
-      <c r="AV13" s="68" t="n"/>
-      <c r="BC13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>3</v>
+      <c r="AO13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AS13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BE13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF13" t="inlineStr">
         <is>
@@ -5034,34 +5108,32 @@
         </is>
       </c>
       <c r="BG13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BH13" t="n">
-        <v>2</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BK13" t="n">
         <v>3</v>
       </c>
-      <c r="BL13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR13" t="n">
-        <v>2</v>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BO13" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>3</v>
       </c>
       <c r="BU13" t="n">
         <v>3</v>
       </c>
-      <c r="BV13" t="n">
-        <v>3</v>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="BW13" t="inlineStr">
         <is>
@@ -5076,36 +5148,58 @@
       <c r="BY13" t="n">
         <v>3</v>
       </c>
-      <c r="BZ13" t="n">
-        <v>3</v>
+      <c r="BZ13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="CA13" t="n">
         <v>2</v>
       </c>
-      <c r="CB13" t="n">
-        <v>3</v>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CC13" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE13" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="CI13" t="n">
         <v>3</v>
       </c>
-      <c r="CJ13" t="n">
-        <v>3</v>
+      <c r="CJ13" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="79" t="inlineStr">
         <is>
-          <t>Luigi</t>
+          <t>RobbyCV</t>
         </is>
       </c>
       <c r="B14" s="79" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C14" s="68" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E14" s="68">
         <f>SUM(G14:H14)</f>
@@ -5115,35 +5209,41 @@
         <f>ROUND(AVERAGE(G14:H14),1)</f>
         <v/>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="79" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="J14" s="80" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="I14" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
+      <c r="K14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="80" t="n">
+        <v>3</v>
       </c>
       <c r="M14" s="79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="80" t="n">
         <v>1</v>
       </c>
       <c r="O14" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P14" s="80" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="P14" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="Q14" s="79" t="n">
         <v>2</v>
@@ -5154,112 +5254,84 @@
         </is>
       </c>
       <c r="W14" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X14" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z14" s="80" t="n">
         <v>2</v>
       </c>
       <c r="AA14" s="79" t="n">
         <v>3</v>
       </c>
       <c r="AB14" s="80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC14" s="79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD14" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM14" s="68" t="n"/>
-      <c r="AN14" s="68" t="n"/>
-      <c r="AO14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP14" t="n">
         <v>1</v>
       </c>
-      <c r="AS14" s="68" t="n"/>
-      <c r="AT14" s="68" t="n"/>
-      <c r="AU14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV14" t="n">
+      <c r="AE14" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF14" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM14" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN14" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO14" t="n">
         <v>1</v>
       </c>
-      <c r="AY14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AZ14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BO14" t="n">
-        <v>2</v>
-      </c>
       <c r="BP14" t="n">
-        <v>3</v>
-      </c>
-      <c r="BS14" t="n">
-        <v>2</v>
-      </c>
-      <c r="BT14" t="n">
-        <v>3</v>
-      </c>
-      <c r="CC14" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD14" t="n">
-        <v>3</v>
-      </c>
-      <c r="CE14" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CF14" t="inlineStr">
+      <c r="BV14" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="CI14" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ14" t="n">
-        <v>3</v>
+      <c r="CA14" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="79" t="inlineStr">
         <is>
-          <t>maikol_lix</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="B15" s="79" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C15" s="68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="E15" s="68">
         <f>SUM(G15:H15)</f>
@@ -5273,10 +5345,10 @@
         <v>3</v>
       </c>
       <c r="H15" s="80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J15" s="80" t="n">
         <v>3</v>
@@ -5284,163 +5356,39 @@
       <c r="O15" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="P15" s="80" t="inlineStr">
+      <c r="P15" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU15" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV15" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="S15" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T15" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X15" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB15" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AE15" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF15" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI15" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ15" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK15" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL15" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM15" s="68" t="n"/>
-      <c r="AN15" s="68" t="n"/>
-      <c r="AO15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AS15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BB15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BE15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BG15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BH15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BO15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BU15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BV15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BW15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BX15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BY15" t="n">
-        <v>3</v>
-      </c>
-      <c r="BZ15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CA15" t="n">
-        <v>2</v>
-      </c>
-      <c r="CB15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CC15" t="n">
-        <v>3</v>
-      </c>
-      <c r="CD15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE15" t="n">
-        <v>3</v>
-      </c>
-      <c r="CF15" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI15" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ15" t="inlineStr">
+      <c r="BH15" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -5449,17 +5397,17 @@
     <row r="16">
       <c r="A16" s="79" t="inlineStr">
         <is>
-          <t>RobbyCV</t>
+          <t>SubOhm</t>
         </is>
       </c>
       <c r="B16" s="79" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C16" s="68" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E16" s="68">
         <f>SUM(G16:H16)</f>
@@ -5469,129 +5417,27 @@
         <f>ROUND(AVERAGE(G16:H16),1)</f>
         <v/>
       </c>
-      <c r="G16" t="n">
-        <v>3</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J16" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="K16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="M16" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="Q16" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="R16" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="W16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X16" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z16" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB16" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC16" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD16" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE16" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF16" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM16" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN16" s="121" t="n">
-        <v>2</v>
-      </c>
-      <c r="BO16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ16" t="n">
-        <v>3</v>
-      </c>
-      <c r="BR16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BU16" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BV16" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CA16" t="n">
-        <v>3</v>
-      </c>
-      <c r="CB16" t="n">
+      <c r="AS16" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT16" s="121" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>xbladze</t>
         </is>
       </c>
       <c r="B17" s="79" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C17" s="68" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E17" s="68">
         <f>SUM(G17:H17)</f>
@@ -5601,11 +5447,15 @@
         <f>ROUND(AVERAGE(G17:H17),1)</f>
         <v/>
       </c>
-      <c r="G17" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H17" s="80" t="n">
-        <v>3</v>
+      <c r="G17" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="H17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="I17" s="79" t="n">
         <v>2</v>
@@ -5613,11 +5463,21 @@
       <c r="J17" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="K17" s="79" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="L17" s="80" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
       <c r="O17" s="79" t="n">
         <v>3</v>
       </c>
       <c r="P17" s="80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="79" t="n">
         <v>3</v>
@@ -5625,6 +5485,64 @@
       <c r="R17" s="80" t="n">
         <v>3</v>
       </c>
+      <c r="S17" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="T17" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="W17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="X17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y17" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA17" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC17" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD17" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI17" s="120" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AJ17" s="121" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="AK17" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL17" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM17" s="120" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN17" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS17" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT17" s="121" t="n">
+        <v>3</v>
+      </c>
       <c r="AU17" s="120" t="n">
         <v>3</v>
       </c>
@@ -5632,23 +5550,99 @@
         <v>3</v>
       </c>
       <c r="BA17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BB17" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>3</v>
       </c>
       <c r="BE17" t="n">
         <v>3</v>
       </c>
       <c r="BF17" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG17" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="BH17" t="inlineStr">
+      <c r="BR17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BS17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BT17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="BU17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CE17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CF17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CI17" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CJ17" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
@@ -5657,14 +5651,14 @@
     <row r="18">
       <c r="A18" s="79" t="inlineStr">
         <is>
-          <t>SubOhm</t>
+          <t>Anonymous</t>
         </is>
       </c>
       <c r="B18" s="79" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C18" s="68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="79" t="n">
         <v>1</v>
@@ -5677,27 +5671,39 @@
         <f>ROUND(AVERAGE(G18:H18),1)</f>
         <v/>
       </c>
-      <c r="AS18" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT18" s="121" t="n">
-        <v>2</v>
+      <c r="AI18" s="120" t="n"/>
+      <c r="AJ18" s="121" t="n"/>
+      <c r="AK18" s="120" t="n"/>
+      <c r="AL18" s="121" t="n"/>
+      <c r="AM18" s="120" t="n"/>
+      <c r="AN18" s="121" t="n"/>
+      <c r="AO18" s="120" t="n"/>
+      <c r="AP18" s="121" t="n"/>
+      <c r="CC18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="CD18" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>xbladze</t>
+          <t>ajaz064</t>
         </is>
       </c>
       <c r="B19" s="79" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C19" s="68" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D19" s="79" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E19" s="68">
         <f>SUM(G19:H19)</f>
@@ -5707,221 +5713,35 @@
         <f>ROUND(AVERAGE(G19:H19),1)</f>
         <v/>
       </c>
-      <c r="G19" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="H19" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="J19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="79" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="L19" s="80" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="O19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="P19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="R19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="S19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="T19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="W19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="X19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA19" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB19" s="80" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC19" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI19" s="120" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AJ19" s="121" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AK19" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL19" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM19" s="120" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN19" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS19" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT19" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="AU19" s="120" t="n">
-        <v>3</v>
-      </c>
-      <c r="AV19" s="121" t="n">
-        <v>3</v>
-      </c>
-      <c r="BA19" t="n">
-        <v>2</v>
-      </c>
-      <c r="BB19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BC19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BD19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BE19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BF19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BG19" t="n">
-        <v>2</v>
-      </c>
-      <c r="BH19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BK19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BL19" t="n">
-        <v>2</v>
-      </c>
-      <c r="BM19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BN19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BO19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BP19" t="n">
-        <v>3</v>
-      </c>
-      <c r="BQ19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BR19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BS19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BT19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="BU19" t="n">
-        <v>2</v>
-      </c>
-      <c r="BV19" t="n">
-        <v>1</v>
-      </c>
-      <c r="CC19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CE19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CF19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CI19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CJ19" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI19" s="120" t="n"/>
+      <c r="AJ19" s="121" t="n"/>
+      <c r="AK19" s="120" t="n"/>
+      <c r="AL19" s="121" t="n"/>
+      <c r="AM19" s="120" t="n"/>
+      <c r="AN19" s="121" t="n"/>
+      <c r="AO19" s="120" t="n"/>
+      <c r="AP19" s="121" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="79" t="inlineStr">
         <is>
-          <t>Anonymous</t>
+          <t>xNullx</t>
         </is>
       </c>
       <c r="B20" s="79" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C20" s="68" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D20" s="79" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E20" s="68">
         <f>SUM(G20:H20)</f>
@@ -5930,6 +5750,12 @@
       <c r="F20" s="68">
         <f>ROUND(AVERAGE(G20:H20),1)</f>
         <v/>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3</v>
       </c>
       <c r="AI20" s="120" t="n"/>
       <c r="AJ20" s="121" t="n"/>
@@ -5939,31 +5765,21 @@
       <c r="AN20" s="121" t="n"/>
       <c r="AO20" s="120" t="n"/>
       <c r="AP20" s="121" t="n"/>
-      <c r="CC20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="CD20" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>ajaz064</t>
+          <t>fhhgggf</t>
         </is>
       </c>
       <c r="B21" s="79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21" s="68" t="n">
         <v>4</v>
       </c>
       <c r="D21" s="79" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E21" s="68">
         <f>SUM(G21:H21)</f>
@@ -5977,7 +5793,7 @@
         <v>3</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI21" s="120" t="n"/>
       <c r="AJ21" s="121" t="n"/>
@@ -5991,17 +5807,17 @@
     <row r="22">
       <c r="A22" s="79" t="inlineStr">
         <is>
-          <t>TinoGiusa</t>
+          <t>maragno</t>
         </is>
       </c>
       <c r="B22" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" s="68" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E22" s="68">
         <f>SUM(G22:H22)</f>
@@ -6012,10 +5828,12 @@
         <v/>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
       <c r="AI22" s="120" t="n"/>
       <c r="AJ22" s="121" t="n"/>
@@ -6029,17 +5847,17 @@
     <row r="23">
       <c r="A23" s="79" t="inlineStr">
         <is>
-          <t>xNullx</t>
+          <t>Akemi</t>
         </is>
       </c>
       <c r="B23" s="79" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C23" s="68" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E23" s="68">
         <f>SUM(G23:H23)</f>
@@ -6048,12 +5866,6 @@
       <c r="F23" s="68">
         <f>ROUND(AVERAGE(G23:H23),1)</f>
         <v/>
-      </c>
-      <c r="G23" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" t="n">
-        <v>3</v>
       </c>
       <c r="AI23" s="120" t="n"/>
       <c r="AJ23" s="121" t="n"/>
@@ -6067,17 +5879,17 @@
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>fhhgggf</t>
+          <t>Elatanvsb108</t>
         </is>
       </c>
       <c r="B24" s="79" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C24" s="68" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E24" s="68">
         <f>SUM(G24:H24)</f>
@@ -6088,10 +5900,10 @@
         <v/>
       </c>
       <c r="G24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI24" s="120" t="n"/>
       <c r="AJ24" s="121" t="n"/>
@@ -6101,148 +5913,6 @@
       <c r="AN24" s="121" t="n"/>
       <c r="AO24" s="120" t="n"/>
       <c r="AP24" s="121" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="79" t="inlineStr">
-        <is>
-          <t>zpercu</t>
-        </is>
-      </c>
-      <c r="B25" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="68">
-        <f>SUM(G25:H25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="68">
-        <f>ROUND(AVERAGE(G25:H25),1)</f>
-        <v/>
-      </c>
-      <c r="AI25" s="120" t="n"/>
-      <c r="AJ25" s="121" t="n"/>
-      <c r="AK25" s="120" t="n"/>
-      <c r="AL25" s="121" t="n"/>
-      <c r="AM25" s="120" t="n"/>
-      <c r="AN25" s="121" t="n"/>
-      <c r="AO25" s="120" t="n"/>
-      <c r="AP25" s="121" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="79" t="inlineStr">
-        <is>
-          <t>maragno</t>
-        </is>
-      </c>
-      <c r="B26" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="E26" s="68">
-        <f>SUM(G26:H26)</f>
-        <v/>
-      </c>
-      <c r="F26" s="68">
-        <f>ROUND(AVERAGE(G26:H26),1)</f>
-        <v/>
-      </c>
-      <c r="G26" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="AI26" s="120" t="n"/>
-      <c r="AJ26" s="121" t="n"/>
-      <c r="AK26" s="120" t="n"/>
-      <c r="AL26" s="121" t="n"/>
-      <c r="AM26" s="120" t="n"/>
-      <c r="AN26" s="121" t="n"/>
-      <c r="AO26" s="120" t="n"/>
-      <c r="AP26" s="121" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="79" t="inlineStr">
-        <is>
-          <t>Akemi</t>
-        </is>
-      </c>
-      <c r="B27" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="68">
-        <f>SUM(G27:H27)</f>
-        <v/>
-      </c>
-      <c r="F27" s="68">
-        <f>ROUND(AVERAGE(G27:H27),1)</f>
-        <v/>
-      </c>
-      <c r="AI27" s="120" t="n"/>
-      <c r="AJ27" s="121" t="n"/>
-      <c r="AK27" s="120" t="n"/>
-      <c r="AL27" s="121" t="n"/>
-      <c r="AM27" s="120" t="n"/>
-      <c r="AN27" s="121" t="n"/>
-      <c r="AO27" s="120" t="n"/>
-      <c r="AP27" s="121" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="79" t="inlineStr">
-        <is>
-          <t>Elatanvsb108</t>
-        </is>
-      </c>
-      <c r="B28" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="68">
-        <f>SUM(G28:H28)</f>
-        <v/>
-      </c>
-      <c r="F28" s="68">
-        <f>ROUND(AVERAGE(G28:H28),1)</f>
-        <v/>
-      </c>
-      <c r="G28" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI28" s="120" t="n"/>
-      <c r="AJ28" s="121" t="n"/>
-      <c r="AK28" s="120" t="n"/>
-      <c r="AL28" s="121" t="n"/>
-      <c r="AM28" s="120" t="n"/>
-      <c r="AN28" s="121" t="n"/>
-      <c r="AO28" s="120" t="n"/>
-      <c r="AP28" s="121" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:CL1">

</xml_diff>